<commit_message>
Marca lacunas inclusas por IA e separa o que não se sustenta.
A coluna Indicação fica vazia nas atividades da equipe que permanecem no caminho. O que não tinha card e a arquitetura mostrou como falta leva a marca de gap. BigQuery no lugar do Databricks, DasaLogs e dois frontends cancelados que a documentação ainda cita vão para a aba de discussão.

Co-authored-by: waneron <waneron@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/BM-GCP-Atividades-DP-ordem-temporal.xlsx
+++ b/BM-GCP-Atividades-DP-ordem-temporal.xlsx
@@ -8,15 +8,18 @@
   </bookViews>
   <sheets>
     <sheet name="BM - GCP Atividades - DP" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Regra de ordem" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Dúvidas" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Discutir com a equipe" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Regra de ordem" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Dúvidas" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'BM - GCP Atividades - DP'!$A$1:$N$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'BM - GCP Atividades - DP'!$A$1:$O$45</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'BM - GCP Atividades - DP'!$1:$1</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Regra de ordem'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Dúvidas'!$A$1:$C$13</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="2">'Dúvidas'!$1:$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Discutir com a equipe'!$A$1:$K$5</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Discutir com a equipe'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="2">'Regra de ordem'!$1:$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Dúvidas'!$A$1:$C$13</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="3">'Dúvidas'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -25,7 +28,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -58,6 +61,12 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
+      <color rgb="00843C0C"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
       <color rgb="001F4E79"/>
       <sz val="14"/>
     </font>
@@ -66,7 +75,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="14">
+  <fills count="15">
     <fill>
       <patternFill/>
     </fill>
@@ -115,17 +124,22 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00E2D5F1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00F4B183"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E2D5F1"/>
+        <fgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F2F2F2"/>
+        <fgColor rgb="00F8D7DA"/>
       </patternFill>
     </fill>
     <fill>
@@ -160,7 +174,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -198,6 +212,9 @@
     <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -213,13 +230,19 @@
     <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -228,20 +251,23 @@
     <xf numFmtId="0" fontId="3" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -609,23 +635,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N51"/>
+  <dimension ref="A1:O45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="46" customWidth="1" min="2" max="2"/>
     <col width="38" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="62" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="46" customWidth="1" min="7" max="7"/>
-    <col width="28" customWidth="1" min="8" max="8"/>
-    <col width="26" customWidth="1" min="9" max="9"/>
-    <col width="36" customWidth="1" min="10" max="10"/>
-    <col width="55" customWidth="1" min="11" max="11"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="62" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="46" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="10" max="10"/>
+    <col width="36" customWidth="1" min="11" max="11"/>
     <col width="55" customWidth="1" min="12" max="12"/>
-    <col width="40" customWidth="1" min="13" max="13"/>
-    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="55" customWidth="1" min="13" max="13"/>
+    <col width="40" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -641,60 +668,65 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Indicação</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Origem</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Card ID</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Descrição</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Complexidade</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Depêndencia</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Cronograma original (não usado na ordem)</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Recurso Responsável</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Observações</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Base na planilha ou na documentação</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Por que nesta posição</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Card URL</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Linha na planilha original</t>
         </is>
@@ -709,46 +741,47 @@
           <t>1. HML — base já concluída</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>Card da planilha</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>424950</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>[DP] Provisionar ambiente GKE HML</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>Concluído</t>
         </is>
       </c>
-      <c r="G2" s="2" t="n"/>
       <c r="H2" s="2" t="n"/>
       <c r="I2" s="2" t="n"/>
       <c r="J2" s="2" t="n"/>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="n"/>
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>Status Concluído. Único card de ambiente, nome HML. A documentação cita o cluster Azure de homologação azr-hml02, namespaces busca, dataprovider-data e portal-cadastro.</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>Ponto de partida. O pedido é sair da homologação.</t>
         </is>
       </c>
-      <c r="M2" s="3" t="inlineStr">
+      <c r="N2" s="3" t="inlineStr">
         <is>
           <t>https://dasa.businessmap.io/ctrl_board/96/cards/424950/details</t>
         </is>
       </c>
-      <c r="N2" s="2" t="n">
+      <c r="O2" s="2" t="n">
         <v>40</v>
       </c>
     </row>
@@ -761,46 +794,47 @@
           <t>1. HML — base já concluída</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" s="2" t="n"/>
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>Card da planilha</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>451661</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>[DP] Migração GCP | Criar banco de dados</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>Concluído</t>
         </is>
       </c>
-      <c r="G3" s="2" t="n"/>
       <c r="H3" s="2" t="n"/>
       <c r="I3" s="2" t="n"/>
       <c r="J3" s="2" t="n"/>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="K3" s="2" t="n"/>
+      <c r="L3" s="2" t="inlineStr">
         <is>
           <t>Status Concluído. O card de migrar o SQL Server está abortado. A documentação descreve o Corporate (HML, master, réplica e staging) como o banco que serve as APIs.</t>
         </is>
       </c>
-      <c r="L3" s="2" t="inlineStr">
+      <c r="M3" s="2" t="inlineStr">
         <is>
           <t>O banco existe. A carga desse banco não tem card e entra mais adiante, antes do teste funcional.</t>
         </is>
       </c>
-      <c r="M3" s="3" t="inlineStr">
+      <c r="N3" s="3" t="inlineStr">
         <is>
           <t>https://dasa.businessmap.io/ctrl_board/96/cards/451661/details</t>
         </is>
       </c>
-      <c r="N3" s="2" t="n">
+      <c r="O3" s="2" t="n">
         <v>39</v>
       </c>
     </row>
@@ -813,54 +847,55 @@
           <t>1. HML — base já concluída</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" s="2" t="n"/>
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>Card da planilha</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>451684</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>[DP] Migração GCP | Redis</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>Concluído</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>Os pods precisam estar de pé para testar</t>
         </is>
       </c>
-      <c r="H4" s="2" t="n"/>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="I4" s="2" t="n"/>
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>Back End</t>
         </is>
       </c>
-      <c r="J4" s="2" t="n"/>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="K4" s="2" t="n"/>
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>Status Concluído. No diagrama, busca-cache fica entre o Corporate e as APIs. A documentação lista dois Redis de 6 GB: DP Cache PRD e Busca. A planilha não separa HML e PRD.</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr">
+      <c r="M4" s="2" t="inlineStr">
         <is>
           <t>Concluído. O teste que a dependência pede espera os pods das APIs.</t>
         </is>
       </c>
-      <c r="M4" s="3" t="inlineStr">
+      <c r="N4" s="3" t="inlineStr">
         <is>
           <t>https://dasa.businessmap.io/ctrl_board/96/cards/451684/details</t>
         </is>
       </c>
-      <c r="N4" s="2" t="n">
+      <c r="O4" s="2" t="n">
         <v>35</v>
       </c>
     </row>
@@ -873,46 +908,47 @@
           <t>1. HML — base já concluída</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" s="2" t="n"/>
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>Card da planilha</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>476416</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>Continuação - Criação de Workloads do projeto BUSCA -&gt; datp-searcher-api-commons</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>Concluído</t>
         </is>
       </c>
-      <c r="G5" s="2" t="n"/>
       <c r="H5" s="2" t="n"/>
       <c r="I5" s="2" t="n"/>
       <c r="J5" s="2" t="n"/>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="K5" s="2" t="n"/>
+      <c r="L5" s="2" t="inlineStr">
         <is>
           <t>Status Concluído. O card 470112, da criação do mesmo workload, segue com observação 'atuando'.</t>
         </is>
       </c>
-      <c r="L5" s="2" t="inlineStr">
+      <c r="M5" s="2" t="inlineStr">
         <is>
           <t>Concluído. O 470112 permanece na fila das APIs.</t>
         </is>
       </c>
-      <c r="M5" s="3" t="inlineStr">
+      <c r="N5" s="3" t="inlineStr">
         <is>
           <t>https://dasa.businessmap.io/ctrl_board/96/cards/476416/details</t>
         </is>
       </c>
-      <c r="N5" s="2" t="n">
+      <c r="O5" s="2" t="n">
         <v>30</v>
       </c>
     </row>
@@ -925,42 +961,43 @@
           <t>2. HML — antes de subir workload</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" s="4" t="n"/>
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>Card da planilha</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="E6" s="4" t="inlineStr">
         <is>
           <t>424949</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="F6" s="4" t="inlineStr">
         <is>
           <t>[DP] Definir conectividade</t>
         </is>
       </c>
-      <c r="F6" s="4" t="n"/>
       <c r="G6" s="4" t="n"/>
       <c r="H6" s="4" t="n"/>
       <c r="I6" s="4" t="n"/>
       <c r="J6" s="4" t="n"/>
-      <c r="K6" s="4" t="inlineStr">
+      <c r="K6" s="4" t="n"/>
+      <c r="L6" s="4" t="inlineStr">
         <is>
           <t>Único card de conectividade. Os workloads de busca registram que a conectividade por IP está errada. A seção de rede do documento (VNet, subnet, VPN, DNS, firewall) está vazia. O diagrama mostra as fontes K2/Gliese, base federada, MDM, GSC, hospitais e MV.</t>
         </is>
       </c>
-      <c r="L6" s="4" t="inlineStr">
+      <c r="M6" s="4" t="inlineStr">
         <is>
           <t>Antes dos workloads. Sem isso a aplicação sobe apontando para IP, que a própria planilha registra como errado.</t>
         </is>
       </c>
-      <c r="M6" s="5" t="inlineStr">
+      <c r="N6" s="5" t="inlineStr">
         <is>
           <t>https://dasa.businessmap.io/ctrl_board/96/cards/424949/details</t>
         </is>
       </c>
-      <c r="N6" s="4" t="n">
+      <c r="O6" s="4" t="n">
         <v>43</v>
       </c>
     </row>
@@ -973,58 +1010,59 @@
           <t>2. HML — antes de subir workload</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" s="4" t="n"/>
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>Card da planilha</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>424942</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="F7" s="4" t="inlineStr">
         <is>
           <t>[DP] Adequação de pipelines CI/CD</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="G7" s="4" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="G7" s="4" t="inlineStr">
+      <c r="H7" s="4" t="inlineStr">
         <is>
           <t>Infra, JulianoTelli</t>
         </is>
       </c>
-      <c r="H7" s="4" t="n"/>
-      <c r="I7" s="4" t="inlineStr">
+      <c r="I7" s="4" t="n"/>
+      <c r="J7" s="4" t="inlineStr">
         <is>
           <t>Infra</t>
         </is>
       </c>
-      <c r="J7" s="4" t="inlineStr">
+      <c r="K7" s="4" t="inlineStr">
         <is>
           <t>telli</t>
         </is>
       </c>
-      <c r="K7" s="4" t="inlineStr">
+      <c r="L7" s="4" t="inlineStr">
         <is>
           <t>Card de esteira, sem data. Nenhum workload cita este número como dependência.</t>
         </is>
       </c>
-      <c r="L7" s="4" t="inlineStr">
+      <c r="M7" s="4" t="inlineStr">
         <is>
           <t>Em paralelo com a conectividade. A planilha não diz que este card bloqueia a criação do workload.</t>
         </is>
       </c>
-      <c r="M7" s="5" t="inlineStr">
+      <c r="N7" s="5" t="inlineStr">
         <is>
           <t>https://dasa.businessmap.io/ctrl_board/96/cards/424942/details</t>
         </is>
       </c>
-      <c r="N7" s="4" t="n">
+      <c r="O7" s="4" t="n">
         <v>31</v>
       </c>
     </row>
@@ -1037,58 +1075,59 @@
           <t>3. HML — APIs e gateway, em paralelo com o Airflow</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C8" s="6" t="n"/>
+      <c r="D8" s="6" t="inlineStr">
         <is>
           <t>Card da planilha</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="E8" s="6" t="inlineStr">
         <is>
           <t>470110</t>
         </is>
       </c>
-      <c r="E8" s="6" t="inlineStr">
+      <c r="F8" s="6" t="inlineStr">
         <is>
           <t>Criação de Workloads do projeto BUSCA -&gt; datp-searcher-api-brand</t>
         </is>
       </c>
-      <c r="F8" s="6" t="inlineStr">
+      <c r="G8" s="6" t="inlineStr">
         <is>
           <t>Baixa</t>
         </is>
       </c>
-      <c r="G8" s="6" t="inlineStr">
+      <c r="H8" s="6" t="inlineStr">
         <is>
           <t>Backend Hj a conectividade está por IP, isso é errado</t>
         </is>
       </c>
-      <c r="H8" s="6" t="inlineStr">
+      <c r="I8" s="6" t="inlineStr">
         <is>
           <t>20/10/26</t>
         </is>
       </c>
-      <c r="I8" s="6" t="inlineStr">
+      <c r="J8" s="6" t="inlineStr">
         <is>
           <t>Back End</t>
         </is>
       </c>
-      <c r="J8" s="6" t="n"/>
-      <c r="K8" s="6" t="inlineStr">
+      <c r="K8" s="6" t="n"/>
+      <c r="L8" s="6" t="inlineStr">
         <is>
           <t>Uma das seis APIs do documento: exam, healthinsurance, commons, agendamento, local e brand. Este card não cita Airflow nem Cognitive Search.</t>
         </is>
       </c>
-      <c r="L8" s="6" t="inlineStr">
+      <c r="M8" s="6" t="inlineStr">
         <is>
           <t>Depois da conectividade. Não espera o Airflow. A data 20/10/26 foi ignorada na ordenação.</t>
         </is>
       </c>
-      <c r="M8" s="7" t="inlineStr">
+      <c r="N8" s="7" t="inlineStr">
         <is>
           <t>https://dasa.businessmap.io/ctrl_board/96/cards/470110/details</t>
         </is>
       </c>
-      <c r="N8" s="6" t="n">
+      <c r="O8" s="6" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1101,58 +1140,59 @@
           <t>3. HML — APIs e gateway, em paralelo com o Airflow</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="C9" s="6" t="n"/>
+      <c r="D9" s="6" t="inlineStr">
         <is>
           <t>Card da planilha</t>
         </is>
       </c>
-      <c r="D9" s="6" t="inlineStr">
+      <c r="E9" s="6" t="inlineStr">
         <is>
           <t>470109</t>
         </is>
       </c>
-      <c r="E9" s="6" t="inlineStr">
+      <c r="F9" s="6" t="inlineStr">
         <is>
           <t>Criação de Workloads do projeto BUSCA -&gt; datp-infra-gateway -&gt; (ZUUL)</t>
         </is>
       </c>
-      <c r="F9" s="6" t="inlineStr">
+      <c r="G9" s="6" t="inlineStr">
         <is>
           <t>Média</t>
         </is>
       </c>
-      <c r="G9" s="6" t="inlineStr">
+      <c r="H9" s="6" t="inlineStr">
         <is>
           <t>Backend Hj a conectividade está por IP, isso é errado</t>
         </is>
       </c>
-      <c r="H9" s="6" t="inlineStr">
+      <c r="I9" s="6" t="inlineStr">
         <is>
           <t>27/10/26</t>
         </is>
       </c>
-      <c r="I9" s="6" t="inlineStr">
+      <c r="J9" s="6" t="inlineStr">
         <is>
           <t>Back End</t>
         </is>
       </c>
-      <c r="J9" s="6" t="n"/>
-      <c r="K9" s="6" t="inlineStr">
+      <c r="K9" s="6" t="n"/>
+      <c r="L9" s="6" t="inlineStr">
         <is>
           <t>No diagrama o gateway aparece como dp-zuul-proxy, ao lado de autorização, rate limit e WAF. Não há card separado para WAF, rate limit ou API key.</t>
         </is>
       </c>
-      <c r="L9" s="6" t="inlineStr">
+      <c r="M9" s="6" t="inlineStr">
         <is>
           <t>Junto das APIs, depois da conectividade. A documentação não separa o gateway da entrada das APIs.</t>
         </is>
       </c>
-      <c r="M9" s="7" t="inlineStr">
+      <c r="N9" s="7" t="inlineStr">
         <is>
           <t>https://dasa.businessmap.io/ctrl_board/96/cards/470109/details</t>
         </is>
       </c>
-      <c r="N9" s="6" t="n">
+      <c r="O9" s="6" t="n">
         <v>4</v>
       </c>
     </row>
@@ -1165,58 +1205,59 @@
           <t>3. HML — APIs e gateway, em paralelo com o Airflow</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="C10" s="6" t="n"/>
+      <c r="D10" s="6" t="inlineStr">
         <is>
           <t>Card da planilha</t>
         </is>
       </c>
-      <c r="D10" s="6" t="inlineStr">
+      <c r="E10" s="6" t="inlineStr">
         <is>
           <t>470118</t>
         </is>
       </c>
-      <c r="E10" s="6" t="inlineStr">
+      <c r="F10" s="6" t="inlineStr">
         <is>
           <t>Criação de Workloads do projeto BUSCA -&gt; datp-searcher-api-local</t>
         </is>
       </c>
-      <c r="F10" s="6" t="inlineStr">
+      <c r="G10" s="6" t="inlineStr">
         <is>
           <t>Média</t>
         </is>
       </c>
-      <c r="G10" s="6" t="inlineStr">
+      <c r="H10" s="6" t="inlineStr">
         <is>
           <t>Backend Hj a conectividade está por IP, isso é errado</t>
         </is>
       </c>
-      <c r="H10" s="6" t="inlineStr">
+      <c r="I10" s="6" t="inlineStr">
         <is>
           <t>07/11/26</t>
         </is>
       </c>
-      <c r="I10" s="6" t="inlineStr">
+      <c r="J10" s="6" t="inlineStr">
         <is>
           <t>Back End</t>
         </is>
       </c>
-      <c r="J10" s="6" t="n"/>
-      <c r="K10" s="6" t="inlineStr">
+      <c r="K10" s="6" t="n"/>
+      <c r="L10" s="6" t="inlineStr">
         <is>
           <t>API local do documento. Não cita Airflow nem Cognitive Search.</t>
         </is>
       </c>
-      <c r="L10" s="6" t="inlineStr">
+      <c r="M10" s="6" t="inlineStr">
         <is>
           <t>Depois da conectividade. Data da planilha ignorada na ordenação.</t>
         </is>
       </c>
-      <c r="M10" s="7" t="inlineStr">
+      <c r="N10" s="7" t="inlineStr">
         <is>
           <t>https://dasa.businessmap.io/ctrl_board/96/cards/470118/details</t>
         </is>
       </c>
-      <c r="N10" s="6" t="n">
+      <c r="O10" s="6" t="n">
         <v>5</v>
       </c>
     </row>
@@ -1229,58 +1270,59 @@
           <t>3. HML — APIs e gateway, em paralelo com o Airflow</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C11" s="6" t="n"/>
+      <c r="D11" s="6" t="inlineStr">
         <is>
           <t>Card da planilha</t>
         </is>
       </c>
-      <c r="D11" s="6" t="inlineStr">
+      <c r="E11" s="6" t="inlineStr">
         <is>
           <t>470115</t>
         </is>
       </c>
-      <c r="E11" s="6" t="inlineStr">
+      <c r="F11" s="6" t="inlineStr">
         <is>
           <t>Criação de Workloads do projeto BUSCA -&gt; datp-searcher-api-healthinsurance</t>
         </is>
       </c>
-      <c r="F11" s="6" t="inlineStr">
+      <c r="G11" s="6" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="G11" s="6" t="inlineStr">
+      <c r="H11" s="6" t="inlineStr">
         <is>
           <t>Backend Hj a conectividade está por IP, isso é errado</t>
         </is>
       </c>
-      <c r="H11" s="6" t="inlineStr">
+      <c r="I11" s="6" t="inlineStr">
         <is>
           <t>20/11/26</t>
         </is>
       </c>
-      <c r="I11" s="6" t="inlineStr">
+      <c r="J11" s="6" t="inlineStr">
         <is>
           <t>Back End</t>
         </is>
       </c>
-      <c r="J11" s="6" t="n"/>
-      <c r="K11" s="6" t="inlineStr">
+      <c r="K11" s="6" t="n"/>
+      <c r="L11" s="6" t="inlineStr">
         <is>
           <t>API de convênio do documento. Não cita Airflow nem Cognitive Search.</t>
         </is>
       </c>
-      <c r="L11" s="6" t="inlineStr">
+      <c r="M11" s="6" t="inlineStr">
         <is>
           <t>Depois da conectividade. Data da planilha ignorada na ordenação.</t>
         </is>
       </c>
-      <c r="M11" s="7" t="inlineStr">
+      <c r="N11" s="7" t="inlineStr">
         <is>
           <t>https://dasa.businessmap.io/ctrl_board/96/cards/470115/details</t>
         </is>
       </c>
-      <c r="N11" s="6" t="n">
+      <c r="O11" s="6" t="n">
         <v>6</v>
       </c>
     </row>
@@ -1293,58 +1335,59 @@
           <t>3. HML — APIs e gateway, em paralelo com o Airflow</t>
         </is>
       </c>
-      <c r="C12" s="6" t="inlineStr">
+      <c r="C12" s="6" t="n"/>
+      <c r="D12" s="6" t="inlineStr">
         <is>
           <t>Card da planilha</t>
         </is>
       </c>
-      <c r="D12" s="6" t="inlineStr">
+      <c r="E12" s="6" t="inlineStr">
         <is>
           <t>470113</t>
         </is>
       </c>
-      <c r="E12" s="6" t="inlineStr">
+      <c r="F12" s="6" t="inlineStr">
         <is>
           <t>Criação de Workloads do projeto BUSCA -&gt; datp-searcher-api-elegibility</t>
         </is>
       </c>
-      <c r="F12" s="6" t="inlineStr">
+      <c r="G12" s="6" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="G12" s="6" t="inlineStr">
+      <c r="H12" s="6" t="inlineStr">
         <is>
           <t>Backend Hj a conectividade está por IP, isso é errado</t>
         </is>
       </c>
-      <c r="H12" s="6" t="inlineStr">
+      <c r="I12" s="6" t="inlineStr">
         <is>
           <t>29/11/26</t>
         </is>
       </c>
-      <c r="I12" s="6" t="inlineStr">
+      <c r="J12" s="6" t="inlineStr">
         <is>
           <t>Back End</t>
         </is>
       </c>
-      <c r="J12" s="6" t="n"/>
-      <c r="K12" s="6" t="inlineStr">
+      <c r="K12" s="6" t="n"/>
+      <c r="L12" s="6" t="inlineStr">
         <is>
           <t>O documento e o diagrama nomeiam busca-agendamento. A planilha nomeia elegibility. Não há outro card com o nome agendamento.</t>
         </is>
       </c>
-      <c r="L12" s="6" t="inlineStr">
+      <c r="M12" s="6" t="inlineStr">
         <is>
           <t>Permanece nesta fila porque o card não cita Airflow nem Cognitive Search. Não foi tratado como a API de agendamento.</t>
         </is>
       </c>
-      <c r="M12" s="7" t="inlineStr">
+      <c r="N12" s="7" t="inlineStr">
         <is>
           <t>https://dasa.businessmap.io/ctrl_board/96/cards/470113/details</t>
         </is>
       </c>
-      <c r="N12" s="6" t="n">
+      <c r="O12" s="6" t="n">
         <v>7</v>
       </c>
     </row>
@@ -1357,58 +1400,59 @@
           <t>3. HML — APIs e gateway, em paralelo com o Airflow</t>
         </is>
       </c>
-      <c r="C13" s="6" t="inlineStr">
+      <c r="C13" s="6" t="n"/>
+      <c r="D13" s="6" t="inlineStr">
         <is>
           <t>Card da planilha</t>
         </is>
       </c>
-      <c r="D13" s="6" t="inlineStr">
+      <c r="E13" s="6" t="inlineStr">
         <is>
           <t>470112</t>
         </is>
       </c>
-      <c r="E13" s="6" t="inlineStr">
+      <c r="F13" s="6" t="inlineStr">
         <is>
           <t>Criação de Workloads do projeto BUSCA -&gt; datp-searcher-api-commons</t>
         </is>
       </c>
-      <c r="F13" s="6" t="inlineStr">
+      <c r="G13" s="6" t="inlineStr">
         <is>
           <t>Baixa</t>
         </is>
       </c>
-      <c r="G13" s="6" t="inlineStr">
+      <c r="H13" s="6" t="inlineStr">
         <is>
           <t>Backend Hj a conectividade está por IP, isso é errado</t>
         </is>
       </c>
-      <c r="H13" s="6" t="n"/>
-      <c r="I13" s="6" t="inlineStr">
+      <c r="I13" s="6" t="n"/>
+      <c r="J13" s="6" t="inlineStr">
         <is>
           <t>Back End</t>
         </is>
       </c>
-      <c r="J13" s="6" t="inlineStr">
+      <c r="K13" s="6" t="inlineStr">
         <is>
           <t>atuando</t>
         </is>
       </c>
-      <c r="K13" s="6" t="inlineStr">
+      <c r="L13" s="6" t="inlineStr">
         <is>
           <t>API commons do documento. A continuação 476416 está concluída. Este card segue 'atuando'.</t>
         </is>
       </c>
-      <c r="L13" s="6" t="inlineStr">
+      <c r="M13" s="6" t="inlineStr">
         <is>
           <t>Na mesma fila das outras APIs de busca que não citam índice.</t>
         </is>
       </c>
-      <c r="M13" s="7" t="inlineStr">
+      <c r="N13" s="7" t="inlineStr">
         <is>
           <t>https://dasa.businessmap.io/ctrl_board/96/cards/470112/details</t>
         </is>
       </c>
-      <c r="N13" s="6" t="n">
+      <c r="O13" s="6" t="n">
         <v>17</v>
       </c>
     </row>
@@ -1421,58 +1465,59 @@
           <t>3. HML — APIs e gateway, em paralelo com o Airflow</t>
         </is>
       </c>
-      <c r="C14" s="6" t="inlineStr">
+      <c r="C14" s="6" t="n"/>
+      <c r="D14" s="6" t="inlineStr">
         <is>
           <t>Card da planilha</t>
         </is>
       </c>
-      <c r="D14" s="6" t="inlineStr">
+      <c r="E14" s="6" t="inlineStr">
         <is>
           <t>424944</t>
         </is>
       </c>
-      <c r="E14" s="6" t="inlineStr">
+      <c r="F14" s="6" t="inlineStr">
         <is>
           <t>[DP] Migração de aplicações, APIs</t>
         </is>
       </c>
-      <c r="F14" s="6" t="inlineStr">
+      <c r="G14" s="6" t="inlineStr">
         <is>
           <t>Baixa</t>
         </is>
       </c>
-      <c r="G14" s="6" t="inlineStr">
+      <c r="H14" s="6" t="inlineStr">
         <is>
           <t>testar conectividade</t>
         </is>
       </c>
-      <c r="H14" s="6" t="inlineStr">
+      <c r="I14" s="6" t="inlineStr">
         <is>
           <t>15/12/26</t>
         </is>
       </c>
-      <c r="I14" s="6" t="inlineStr">
+      <c r="J14" s="6" t="inlineStr">
         <is>
           <t>Back End</t>
         </is>
       </c>
-      <c r="J14" s="6" t="n"/>
-      <c r="K14" s="6" t="inlineStr">
+      <c r="K14" s="6" t="n"/>
+      <c r="L14" s="6" t="inlineStr">
         <is>
           <t>A dependência é testar conectividade, não teste funcional.</t>
         </is>
       </c>
-      <c r="L14" s="6" t="inlineStr">
+      <c r="M14" s="6" t="inlineStr">
         <is>
           <t>Logo depois dos workloads desta fila. Confirma que a aplicação enxerga o destino. O teste funcional espera dado, índice e portal.</t>
         </is>
       </c>
-      <c r="M14" s="7" t="inlineStr">
+      <c r="N14" s="7" t="inlineStr">
         <is>
           <t>https://dasa.businessmap.io/ctrl_board/96/cards/424944/details</t>
         </is>
       </c>
-      <c r="N14" s="6" t="n">
+      <c r="O14" s="6" t="n">
         <v>8</v>
       </c>
     </row>
@@ -1485,54 +1530,55 @@
           <t>3. HML — front e back do DP, em paralelo com o Airflow</t>
         </is>
       </c>
-      <c r="C15" s="6" t="inlineStr">
+      <c r="C15" s="6" t="n"/>
+      <c r="D15" s="6" t="inlineStr">
         <is>
           <t>Card da planilha</t>
         </is>
       </c>
-      <c r="D15" s="6" t="inlineStr">
+      <c r="E15" s="6" t="inlineStr">
         <is>
           <t>469049</t>
         </is>
       </c>
-      <c r="E15" s="6" t="inlineStr">
+      <c r="F15" s="6" t="inlineStr">
         <is>
           <t>[DP] Migração GCP | Migrar Backend -&gt; front do DP (adaptações)</t>
         </is>
       </c>
-      <c r="F15" s="6" t="inlineStr">
+      <c r="G15" s="6" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="G15" s="6" t="inlineStr">
+      <c r="H15" s="6" t="inlineStr">
         <is>
           <t>Ajuste de codigo, versao, eventual erro</t>
         </is>
       </c>
-      <c r="H15" s="6" t="n"/>
-      <c r="I15" s="6" t="inlineStr">
+      <c r="I15" s="6" t="n"/>
+      <c r="J15" s="6" t="inlineStr">
         <is>
           <t>Back End</t>
         </is>
       </c>
-      <c r="J15" s="6" t="n"/>
-      <c r="K15" s="6" t="inlineStr">
+      <c r="K15" s="6" t="n"/>
+      <c r="L15" s="6" t="inlineStr">
         <is>
           <t>A documentação aponta o repositório datp-backoffice-backend. O card não cita Airflow. O diagrama tem dp-backoffice-api-prd.</t>
         </is>
       </c>
-      <c r="L15" s="6" t="inlineStr">
+      <c r="M15" s="6" t="inlineStr">
         <is>
           <t>Sobe com as APIs. Não espera carga nem índice. O teste do frontend espera a integração.</t>
         </is>
       </c>
-      <c r="M15" s="7" t="inlineStr">
+      <c r="N15" s="7" t="inlineStr">
         <is>
           <t>https://dasa.businessmap.io/ctrl_board/96/cards/469049/details</t>
         </is>
       </c>
-      <c r="N15" s="6" t="n">
+      <c r="O15" s="6" t="n">
         <v>15</v>
       </c>
     </row>
@@ -1545,58 +1591,59 @@
           <t>3. HML — front e back do DP, em paralelo com o Airflow</t>
         </is>
       </c>
-      <c r="C16" s="6" t="inlineStr">
+      <c r="C16" s="6" t="n"/>
+      <c r="D16" s="6" t="inlineStr">
         <is>
           <t>Card da planilha</t>
         </is>
       </c>
-      <c r="D16" s="6" t="inlineStr">
+      <c r="E16" s="6" t="inlineStr">
         <is>
           <t>469051</t>
         </is>
       </c>
-      <c r="E16" s="6" t="inlineStr">
+      <c r="F16" s="6" t="inlineStr">
         <is>
           <t>[DP] Migração GCP | Migrar Frontend  portal do DP (adaptações)</t>
         </is>
       </c>
-      <c r="F16" s="6" t="inlineStr">
+      <c r="G16" s="6" t="inlineStr">
         <is>
           <t>Média</t>
         </is>
       </c>
-      <c r="G16" s="6" t="inlineStr">
+      <c r="H16" s="6" t="inlineStr">
         <is>
           <t>Ajuste de codigo, versao, eventual erro</t>
         </is>
       </c>
-      <c r="H16" s="6" t="n"/>
-      <c r="I16" s="6" t="inlineStr">
+      <c r="I16" s="6" t="n"/>
+      <c r="J16" s="6" t="inlineStr">
         <is>
           <t>Back End</t>
         </is>
       </c>
-      <c r="J16" s="6" t="inlineStr">
+      <c r="K16" s="6" t="inlineStr">
         <is>
           <t>só é possivel testar o front com tudo integrado.</t>
         </is>
       </c>
-      <c r="K16" s="6" t="inlineStr">
+      <c r="L16" s="6" t="inlineStr">
         <is>
           <t>A documentação cita o frontend em dp-corporate-frontend e o repositório datp-backoffice-frontend. O card 470121, dp-corporate-frontend, está cancelado. A observação deste card fala do teste, que é o 451689.</t>
         </is>
       </c>
-      <c r="L16" s="6" t="inlineStr">
+      <c r="M16" s="6" t="inlineStr">
         <is>
           <t>A adaptação entra aqui. O teste do front fica no fim da HML, com o 451689.</t>
         </is>
       </c>
-      <c r="M16" s="7" t="inlineStr">
+      <c r="N16" s="7" t="inlineStr">
         <is>
           <t>https://dasa.businessmap.io/ctrl_board/96/cards/469051/details</t>
         </is>
       </c>
-      <c r="N16" s="6" t="n">
+      <c r="O16" s="6" t="n">
         <v>14</v>
       </c>
     </row>
@@ -1609,54 +1656,55 @@
           <t>4. HML — índice e exam, em paralelo com o Airflow</t>
         </is>
       </c>
-      <c r="C17" s="8" t="inlineStr">
+      <c r="C17" s="8" t="n"/>
+      <c r="D17" s="8" t="inlineStr">
         <is>
           <t>Card da planilha</t>
         </is>
       </c>
-      <c r="D17" s="8" t="inlineStr">
+      <c r="E17" s="8" t="inlineStr">
         <is>
           <t>451682</t>
         </is>
       </c>
-      <c r="E17" s="8" t="inlineStr">
+      <c r="F17" s="8" t="inlineStr">
         <is>
           <t>[DP] Migração GCP | Index (cognitive search &gt; vertex - adaptar na aplicação)</t>
         </is>
       </c>
-      <c r="F17" s="8" t="inlineStr">
+      <c r="G17" s="8" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="G17" s="8" t="inlineStr">
+      <c r="H17" s="8" t="inlineStr">
         <is>
           <t>Maior Risco, descoberta</t>
         </is>
       </c>
-      <c r="H17" s="8" t="n"/>
-      <c r="I17" s="8" t="inlineStr">
+      <c r="I17" s="8" t="n"/>
+      <c r="J17" s="8" t="inlineStr">
         <is>
           <t>Felipe Paixão | Back End</t>
         </is>
       </c>
-      <c r="J17" s="8" t="n"/>
-      <c r="K17" s="8" t="inlineStr">
+      <c r="K17" s="8" t="n"/>
+      <c r="L17" s="8" t="inlineStr">
         <is>
           <t>No diagrama, busca-search fica entre o Corporate e as APIs. No documento, Cognitive Search é dependência externa, criticidade alta, e 'pode desacoplar' está TBD. O card aponta Vertex e está em descoberta. A planilha só declara a dependência na API de exam e no dp-backend-api cancelado.</t>
         </is>
       </c>
-      <c r="L17" s="8" t="inlineStr">
+      <c r="M17" s="8" t="inlineStr">
         <is>
           <t>Antes da API de exam. As outras APIs não foram colocadas atrás deste card: a planilha não diz que elas leem o índice.</t>
         </is>
       </c>
-      <c r="M17" s="9" t="inlineStr">
+      <c r="N17" s="9" t="inlineStr">
         <is>
           <t>https://dasa.businessmap.io/ctrl_board/96/cards/451682/details</t>
         </is>
       </c>
-      <c r="N17" s="8" t="n">
+      <c r="O17" s="8" t="n">
         <v>41</v>
       </c>
     </row>
@@ -1669,58 +1717,59 @@
           <t>4. HML — índice e exam, em paralelo com o Airflow</t>
         </is>
       </c>
-      <c r="C18" s="8" t="inlineStr">
+      <c r="C18" s="8" t="n"/>
+      <c r="D18" s="8" t="inlineStr">
         <is>
           <t>Card da planilha</t>
         </is>
       </c>
-      <c r="D18" s="8" t="inlineStr">
+      <c r="E18" s="8" t="inlineStr">
         <is>
           <t>470114</t>
         </is>
       </c>
-      <c r="E18" s="8" t="inlineStr">
+      <c r="F18" s="8" t="inlineStr">
         <is>
           <t>Criação de Workloads do projeto BUSCA -&gt; datp-searcher-api-exam</t>
         </is>
       </c>
-      <c r="F18" s="8" t="inlineStr">
+      <c r="G18" s="8" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="G18" s="8" t="inlineStr">
+      <c r="H18" s="8" t="inlineStr">
         <is>
           <t>Backend Hj a conectividade está por IP, isso é errado</t>
         </is>
       </c>
-      <c r="H18" s="8" t="n"/>
-      <c r="I18" s="8" t="inlineStr">
+      <c r="I18" s="8" t="n"/>
+      <c r="J18" s="8" t="inlineStr">
         <is>
           <t>Back End</t>
         </is>
       </c>
-      <c r="J18" s="8" t="inlineStr">
+      <c r="K18" s="8" t="inlineStr">
         <is>
           <t>depende cognitiveSearch</t>
         </is>
       </c>
-      <c r="K18" s="8" t="inlineStr">
+      <c r="L18" s="8" t="inlineStr">
         <is>
           <t>API de exam do documento. Observação: depende de Cognitive Search. Também registra conectividade por IP errada.</t>
         </is>
       </c>
-      <c r="L18" s="8" t="inlineStr">
+      <c r="M18" s="8" t="inlineStr">
         <is>
           <t>Depois do 451682 e depois da conectividade.</t>
         </is>
       </c>
-      <c r="M18" s="9" t="inlineStr">
+      <c r="N18" s="9" t="inlineStr">
         <is>
           <t>https://dasa.businessmap.io/ctrl_board/96/cards/470114/details</t>
         </is>
       </c>
-      <c r="N18" s="8" t="n">
+      <c r="O18" s="8" t="n">
         <v>18</v>
       </c>
     </row>
@@ -1733,62 +1782,63 @@
           <t>5. HML — migrar o Airflow da Azure para a GCP</t>
         </is>
       </c>
-      <c r="C19" s="10" t="inlineStr">
+      <c r="C19" s="10" t="n"/>
+      <c r="D19" s="10" t="inlineStr">
         <is>
           <t>Card da planilha</t>
         </is>
       </c>
-      <c r="D19" s="10" t="inlineStr">
+      <c r="E19" s="10" t="inlineStr">
         <is>
           <t>478326</t>
         </is>
       </c>
-      <c r="E19" s="10" t="inlineStr">
+      <c r="F19" s="10" t="inlineStr">
         <is>
           <t>Spike -&gt; Airflow na versao mais nova do airflow</t>
         </is>
       </c>
-      <c r="F19" s="10" t="inlineStr">
+      <c r="G19" s="10" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="G19" s="10" t="inlineStr">
+      <c r="H19" s="10" t="inlineStr">
         <is>
           <t>Victor, subir um docker e testar ambienteLocal</t>
         </is>
       </c>
-      <c r="H19" s="10" t="inlineStr">
+      <c r="I19" s="10" t="inlineStr">
         <is>
           <t>20/10/26</t>
         </is>
       </c>
-      <c r="I19" s="10" t="inlineStr">
+      <c r="J19" s="10" t="inlineStr">
         <is>
           <t>Back End</t>
         </is>
       </c>
-      <c r="J19" s="10" t="inlineStr">
+      <c r="K19" s="10" t="inlineStr">
         <is>
           <t>Aqui já vai ser possivel pegar imcompatibilidade de versao</t>
         </is>
       </c>
-      <c r="K19" s="10" t="inlineStr">
+      <c r="L19" s="10" t="inlineStr">
         <is>
           <t>O Airflow de partida já está na Azure. A dependência deste card é docker local. A documentação registra a versão 2.2.5 como baixa demais para a versão do Google.</t>
         </is>
       </c>
-      <c r="L19" s="10" t="inlineStr">
+      <c r="M19" s="10" t="inlineStr">
         <is>
           <t>Primeira linha desta frente, em paralelo com as APIs da etapa 3. A spike existe por causa da versão, antes de migrar o Airflow da Azure para a GCP. Carga, Blob e portal esperam essa migração. A data 20/10/26 não posiciona o resto.</t>
         </is>
       </c>
-      <c r="M19" s="11" t="inlineStr">
+      <c r="N19" s="11" t="inlineStr">
         <is>
           <t>https://dasa.businessmap.io/ctrl_board/96/cards/478326/details</t>
         </is>
       </c>
-      <c r="N19" s="10" t="n">
+      <c r="O19" s="10" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1801,46 +1851,47 @@
           <t>5. HML — migrar o Airflow da Azure para a GCP</t>
         </is>
       </c>
-      <c r="C20" s="10" t="inlineStr">
+      <c r="C20" s="10" t="n"/>
+      <c r="D20" s="10" t="inlineStr">
         <is>
           <t>Card da planilha</t>
         </is>
       </c>
-      <c r="D20" s="10" t="n"/>
-      <c r="E20" s="10" t="inlineStr">
+      <c r="E20" s="10" t="n"/>
+      <c r="F20" s="10" t="inlineStr">
         <is>
           <t>Criar historia adequação airflow, vinculada ao fim da poc do Victor =&gt; necessario devido versao de airflow</t>
         </is>
       </c>
-      <c r="F20" s="10" t="inlineStr">
+      <c r="G20" s="10" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="G20" s="10" t="inlineStr">
+      <c r="H20" s="10" t="inlineStr">
         <is>
           <t>as adequações levarão tempo, pode ser a maior data.</t>
         </is>
       </c>
-      <c r="H20" s="10" t="inlineStr">
+      <c r="I20" s="10" t="inlineStr">
         <is>
           <t>entre março e abril de 2027</t>
         </is>
       </c>
-      <c r="I20" s="10" t="n"/>
       <c r="J20" s="10" t="n"/>
-      <c r="K20" s="10" t="inlineStr">
+      <c r="K20" s="10" t="n"/>
+      <c r="L20" s="10" t="inlineStr">
         <is>
           <t>Linha da planilha, sem Card ID. É a migração do Airflow que já roda na Azure para a GCP. A adequação existe por causa da versão. Portal, Blob e backoffice citam Airflow como dependência. Os workloads com prd no nome ficam na produção.</t>
         </is>
       </c>
-      <c r="L20" s="10" t="inlineStr">
+      <c r="M20" s="10" t="inlineStr">
         <is>
           <t>Depois da spike. A janela de março–abril de 2027 fica registrada e não empurra esta linha para o fim. Blob e portal ficam depois porque dependem do Airflow já na GCP.</t>
         </is>
       </c>
-      <c r="M20" s="10" t="n"/>
-      <c r="N20" s="10" t="n">
+      <c r="N20" s="10" t="n"/>
+      <c r="O20" s="10" t="n">
         <v>13</v>
       </c>
     </row>
@@ -1853,96 +1904,102 @@
           <t>6. HML — dado, depois do Airflow e do backend</t>
         </is>
       </c>
-      <c r="C21" s="12" t="inlineStr">
+      <c r="C21" s="13" t="inlineStr">
+        <is>
+          <t>Inclusa por IA — gap identificado</t>
+        </is>
+      </c>
+      <c r="D21" s="12" t="inlineStr">
         <is>
           <t>Lacuna — documentação</t>
         </is>
       </c>
-      <c r="D21" s="12" t="n"/>
-      <c r="E21" s="12" t="inlineStr">
+      <c r="E21" s="12" t="n"/>
+      <c r="F21" s="12" t="inlineStr">
         <is>
           <t>Carga, no banco de HML, dos dados de exame, unidade e convênio que hoje estão no Corporate</t>
         </is>
       </c>
-      <c r="F21" s="12" t="n"/>
       <c r="G21" s="12" t="n"/>
       <c r="H21" s="12" t="n"/>
       <c r="I21" s="12" t="n"/>
       <c r="J21" s="12" t="n"/>
-      <c r="K21" s="12" t="inlineStr">
+      <c r="K21" s="12" t="n"/>
+      <c r="L21" s="12" t="inlineStr">
         <is>
           <t>O DP serve exame, unidade e convênio para NAV e CDC. O diagrama leva as fontes ao Corporate, e o Corporate às APIs. Existe CORPORATE_HOM na documentação. O card 451661 cria o banco e está concluído. O card 451676, migrar SQL Server, está abortado. Não há card de carga.</t>
         </is>
       </c>
-      <c r="L21" s="12" t="inlineStr">
+      <c r="M21" s="12" t="inlineStr">
         <is>
           <t>Antes do teste funcional e depois da migração do Airflow para a GCP. Se o banco criado já tiver esses dados, esta linha sai.</t>
         </is>
       </c>
-      <c r="M21" s="12" t="n"/>
       <c r="N21" s="12" t="n"/>
+      <c r="O21" s="12" t="n"/>
     </row>
     <row r="22" ht="52" customHeight="1">
-      <c r="A22" s="13" t="n">
+      <c r="A22" s="14" t="n">
         <v>21</v>
       </c>
-      <c r="B22" s="13" t="inlineStr">
+      <c r="B22" s="14" t="inlineStr">
         <is>
           <t>6. HML — dado, depois do Airflow e do backend</t>
         </is>
       </c>
-      <c r="C22" s="13" t="inlineStr">
+      <c r="C22" s="14" t="n"/>
+      <c r="D22" s="14" t="inlineStr">
         <is>
           <t>Card da planilha</t>
         </is>
       </c>
-      <c r="D22" s="13" t="inlineStr">
+      <c r="E22" s="14" t="inlineStr">
         <is>
           <t>451688</t>
         </is>
       </c>
-      <c r="E22" s="13" t="inlineStr">
+      <c r="F22" s="14" t="inlineStr">
         <is>
           <t>[DP] Migração GCP | Blob Storage (adaptações na aplicação)</t>
         </is>
       </c>
-      <c r="F22" s="13" t="inlineStr">
+      <c r="G22" s="14" t="inlineStr">
         <is>
           <t>Média</t>
         </is>
       </c>
-      <c r="G22" s="13" t="inlineStr">
+      <c r="H22" s="14" t="inlineStr">
         <is>
           <t>Criado, depende de airFlow, backend e frontEnd</t>
         </is>
       </c>
-      <c r="H22" s="13" t="inlineStr">
+      <c r="I22" s="14" t="inlineStr">
         <is>
           <t>03/02/27</t>
         </is>
       </c>
-      <c r="I22" s="13" t="inlineStr">
+      <c r="J22" s="14" t="inlineStr">
         <is>
           <t>Back End | Dados</t>
         </is>
       </c>
-      <c r="J22" s="13" t="n"/>
-      <c r="K22" s="13" t="inlineStr">
+      <c r="K22" s="14" t="n"/>
+      <c r="L22" s="14" t="inlineStr">
         <is>
           <t>A documentação registra 269 GB de Blob. A dependência do card pede Airflow, backend e frontend. A data 03/02/27 não define a posição.</t>
         </is>
       </c>
-      <c r="L22" s="13" t="inlineStr">
+      <c r="M22" s="14" t="inlineStr">
         <is>
           <t>Depois do Airflow de HML e depois do backend e do frontend do DP. A planilha não diz se o download D+1 lê este Blob; por isso o D+1 não foi colocado obrigatoriamente depois.</t>
         </is>
       </c>
-      <c r="M22" s="14" t="inlineStr">
+      <c r="N22" s="15" t="inlineStr">
         <is>
           <t>https://dasa.businessmap.io/ctrl_board/96/cards/451688/details</t>
         </is>
       </c>
-      <c r="N22" s="13" t="n">
+      <c r="O22" s="14" t="n">
         <v>10</v>
       </c>
     </row>
@@ -1955,34 +2012,39 @@
           <t>6. HML — dado, depois do Airflow e do backend</t>
         </is>
       </c>
-      <c r="C23" s="12" t="inlineStr">
+      <c r="C23" s="13" t="inlineStr">
+        <is>
+          <t>Inclusa por IA — gap identificado</t>
+        </is>
+      </c>
+      <c r="D23" s="12" t="inlineStr">
         <is>
           <t>Lacuna — dependência citada no card</t>
         </is>
       </c>
-      <c r="D23" s="12" t="n"/>
-      <c r="E23" s="12" t="inlineStr">
+      <c r="E23" s="12" t="n"/>
+      <c r="F23" s="12" t="inlineStr">
         <is>
           <t>Cargas de cadastro</t>
         </is>
       </c>
-      <c r="F23" s="12" t="n"/>
       <c r="G23" s="12" t="n"/>
       <c r="H23" s="12" t="n"/>
       <c r="I23" s="12" t="n"/>
       <c r="J23" s="12" t="n"/>
-      <c r="K23" s="12" t="inlineStr">
+      <c r="K23" s="12" t="n"/>
+      <c r="L23" s="12" t="inlineStr">
         <is>
           <t>Dependência escrita nos cards 470165 e 470100: 'Depende do airFlow pronto, cargas cadastro e D+1 (dowloads Cadastro)'. O diagrama tem o Portal de Cadastros como consumidor e, no desenho GCP, Excel do Portal Cadastro como fonte.</t>
         </is>
       </c>
-      <c r="L23" s="12" t="inlineStr">
+      <c r="M23" s="12" t="inlineStr">
         <is>
           <t>Antes dos workloads de portal que citam essa carga. Não há card, responsável nem prazo.</t>
         </is>
       </c>
-      <c r="M23" s="12" t="n"/>
       <c r="N23" s="12" t="n"/>
+      <c r="O23" s="12" t="n"/>
     </row>
     <row r="24" ht="52" customHeight="1">
       <c r="A24" s="12" t="n">
@@ -1993,1621 +2055,1367 @@
           <t>6. HML — dado, depois do Airflow e do backend</t>
         </is>
       </c>
-      <c r="C24" s="12" t="inlineStr">
+      <c r="C24" s="13" t="inlineStr">
+        <is>
+          <t>Inclusa por IA — gap identificado</t>
+        </is>
+      </c>
+      <c r="D24" s="12" t="inlineStr">
         <is>
           <t>Lacuna — dependência citada no card</t>
         </is>
       </c>
-      <c r="D24" s="12" t="n"/>
-      <c r="E24" s="12" t="inlineStr">
+      <c r="E24" s="12" t="n"/>
+      <c r="F24" s="12" t="inlineStr">
         <is>
           <t>Downloads D+1 de cadastro</t>
         </is>
       </c>
-      <c r="F24" s="12" t="n"/>
       <c r="G24" s="12" t="n"/>
       <c r="H24" s="12" t="n"/>
       <c r="I24" s="12" t="n"/>
       <c r="J24" s="12" t="n"/>
-      <c r="K24" s="12" t="inlineStr">
+      <c r="K24" s="12" t="n"/>
+      <c r="L24" s="12" t="inlineStr">
         <is>
           <t>Mesma dependência dos cards 470165 e 470100. Não há card só para o D+1.</t>
         </is>
       </c>
-      <c r="L24" s="12" t="inlineStr">
+      <c r="M24" s="12" t="inlineStr">
         <is>
           <t>No mesmo bloco das cargas de cadastro. A ordem entre D+1 e Blob não está escrita.</t>
         </is>
       </c>
-      <c r="M24" s="12" t="n"/>
       <c r="N24" s="12" t="n"/>
+      <c r="O24" s="12" t="n"/>
     </row>
     <row r="25" ht="52" customHeight="1">
-      <c r="A25" s="13" t="n">
+      <c r="A25" s="14" t="n">
         <v>24</v>
       </c>
-      <c r="B25" s="13" t="inlineStr">
+      <c r="B25" s="14" t="inlineStr">
         <is>
           <t>7. HML — portal, depois da carga que ele cita</t>
         </is>
       </c>
-      <c r="C25" s="13" t="inlineStr">
+      <c r="C25" s="14" t="n"/>
+      <c r="D25" s="14" t="inlineStr">
         <is>
           <t>Card da planilha</t>
         </is>
       </c>
-      <c r="D25" s="13" t="inlineStr">
+      <c r="E25" s="14" t="inlineStr">
         <is>
           <t>468966</t>
         </is>
       </c>
-      <c r="E25" s="13" t="inlineStr">
+      <c r="F25" s="14" t="inlineStr">
         <is>
           <t>Criação de Workloads do projeto BUSCA -&gt; datp-backoffice-backend</t>
         </is>
       </c>
-      <c r="F25" s="13" t="inlineStr">
+      <c r="G25" s="14" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="G25" s="13" t="inlineStr">
+      <c r="H25" s="14" t="inlineStr">
         <is>
           <t>Ajuste de codigo, versao, eventual erro</t>
         </is>
       </c>
-      <c r="H25" s="13" t="n"/>
-      <c r="I25" s="13" t="inlineStr">
+      <c r="I25" s="14" t="n"/>
+      <c r="J25" s="14" t="inlineStr">
         <is>
           <t>Back End</t>
         </is>
       </c>
-      <c r="J25" s="13" t="inlineStr">
+      <c r="K25" s="14" t="inlineStr">
         <is>
           <t>depende do airFlow</t>
         </is>
       </c>
-      <c r="K25" s="13" t="inlineStr">
+      <c r="L25" s="14" t="inlineStr">
         <is>
           <t>Observação do card: depende do Airflow. Não cita a carga de cadastro.</t>
         </is>
       </c>
-      <c r="L25" s="13" t="inlineStr">
+      <c r="M25" s="14" t="inlineStr">
         <is>
           <t>Depois do Airflow de HML. Antes do teste integrado.</t>
         </is>
       </c>
-      <c r="M25" s="14" t="inlineStr">
+      <c r="N25" s="15" t="inlineStr">
         <is>
           <t>https://dasa.businessmap.io/ctrl_board/96/cards/468966/details</t>
         </is>
       </c>
-      <c r="N25" s="13" t="n">
+      <c r="O25" s="14" t="n">
         <v>22</v>
       </c>
     </row>
     <row r="26" ht="52" customHeight="1">
-      <c r="A26" s="13" t="n">
+      <c r="A26" s="14" t="n">
         <v>25</v>
       </c>
-      <c r="B26" s="13" t="inlineStr">
+      <c r="B26" s="14" t="inlineStr">
         <is>
           <t>7. HML — portal, depois da carga que ele cita</t>
         </is>
       </c>
-      <c r="C26" s="13" t="inlineStr">
+      <c r="C26" s="14" t="n"/>
+      <c r="D26" s="14" t="inlineStr">
         <is>
           <t>Card da planilha</t>
         </is>
       </c>
-      <c r="D26" s="13" t="inlineStr">
+      <c r="E26" s="14" t="inlineStr">
         <is>
           <t>470165</t>
         </is>
       </c>
-      <c r="E26" s="13" t="inlineStr">
+      <c r="F26" s="14" t="inlineStr">
         <is>
           <t>Criação de Workloads do projeto PORTAL-CADASTRO -&gt; portal-cadastro-web</t>
         </is>
       </c>
-      <c r="F26" s="13" t="inlineStr">
+      <c r="G26" s="14" t="inlineStr">
         <is>
           <t>Média</t>
         </is>
       </c>
-      <c r="G26" s="13" t="inlineStr">
+      <c r="H26" s="14" t="inlineStr">
         <is>
           <t>Depende do airFlow pronto, cargas cadastro e D+1 (dowloads Cadastro)</t>
         </is>
       </c>
-      <c r="H26" s="13" t="n"/>
-      <c r="I26" s="13" t="inlineStr">
+      <c r="I26" s="14" t="n"/>
+      <c r="J26" s="14" t="inlineStr">
         <is>
           <t>Back End | Dados | Infra</t>
         </is>
       </c>
-      <c r="J26" s="13" t="inlineStr">
+      <c r="K26" s="14" t="inlineStr">
         <is>
           <t>depende do airFlow</t>
         </is>
       </c>
-      <c r="K26" s="13" t="inlineStr">
+      <c r="L26" s="14" t="inlineStr">
         <is>
           <t>A documentação cita o frontend do portal de cadastro e o repositório datp-backoffice-frontend-portal. O card desse repositório, 468985, está cancelado.</t>
         </is>
       </c>
-      <c r="L26" s="13" t="inlineStr">
+      <c r="M26" s="14" t="inlineStr">
         <is>
           <t>Depois de Airflow, cargas de cadastro e D+1, como a dependência escreve.</t>
         </is>
       </c>
-      <c r="M26" s="14" t="inlineStr">
+      <c r="N26" s="15" t="inlineStr">
         <is>
           <t>https://dasa.businessmap.io/ctrl_board/96/cards/470165/details</t>
         </is>
       </c>
-      <c r="N26" s="13" t="n">
+      <c r="O26" s="14" t="n">
         <v>19</v>
       </c>
     </row>
     <row r="27" ht="52" customHeight="1">
-      <c r="A27" s="13" t="n">
+      <c r="A27" s="14" t="n">
         <v>26</v>
       </c>
-      <c r="B27" s="13" t="inlineStr">
+      <c r="B27" s="14" t="inlineStr">
         <is>
           <t>7. HML — portal, depois da carga que ele cita</t>
         </is>
       </c>
-      <c r="C27" s="13" t="inlineStr">
+      <c r="C27" s="14" t="n"/>
+      <c r="D27" s="14" t="inlineStr">
         <is>
           <t>Card da planilha</t>
         </is>
       </c>
-      <c r="D27" s="13" t="inlineStr">
+      <c r="E27" s="14" t="inlineStr">
         <is>
           <t>470100</t>
         </is>
       </c>
-      <c r="E27" s="13" t="inlineStr">
+      <c r="F27" s="14" t="inlineStr">
         <is>
           <t>Criação de Workloads do projeto BUSCA -&gt; datp-backoffice-frontend</t>
         </is>
       </c>
-      <c r="F27" s="13" t="inlineStr">
+      <c r="G27" s="14" t="inlineStr">
         <is>
           <t>Média</t>
         </is>
       </c>
-      <c r="G27" s="13" t="inlineStr">
+      <c r="H27" s="14" t="inlineStr">
         <is>
           <t>Depende do airFlow pronto, cargas cadastro e D+1 (dowloads Cadastro)</t>
         </is>
       </c>
-      <c r="H27" s="13" t="n"/>
-      <c r="I27" s="13" t="inlineStr">
+      <c r="I27" s="14" t="n"/>
+      <c r="J27" s="14" t="inlineStr">
         <is>
           <t>Back End | Dados | Infra</t>
         </is>
       </c>
-      <c r="J27" s="13" t="inlineStr">
+      <c r="K27" s="14" t="inlineStr">
         <is>
           <t>depende do airFlow</t>
         </is>
       </c>
-      <c r="K27" s="13" t="inlineStr">
+      <c r="L27" s="14" t="inlineStr">
         <is>
           <t>Mesma dependência do 470165.</t>
         </is>
       </c>
-      <c r="L27" s="13" t="inlineStr">
+      <c r="M27" s="14" t="inlineStr">
         <is>
           <t>Junto do portal-cadastro-web.</t>
         </is>
       </c>
-      <c r="M27" s="14" t="inlineStr">
+      <c r="N27" s="15" t="inlineStr">
         <is>
           <t>https://dasa.businessmap.io/ctrl_board/96/cards/470100/details</t>
         </is>
       </c>
-      <c r="N27" s="13" t="n">
+      <c r="O27" s="14" t="n">
         <v>21</v>
       </c>
     </row>
     <row r="28" ht="52" customHeight="1">
-      <c r="A28" s="13" t="n">
+      <c r="A28" s="14" t="n">
         <v>27</v>
       </c>
-      <c r="B28" s="13" t="inlineStr">
+      <c r="B28" s="14" t="inlineStr">
         <is>
           <t>7. HML — portal, depois da carga que ele cita</t>
         </is>
       </c>
-      <c r="C28" s="13" t="inlineStr">
+      <c r="C28" s="14" t="n"/>
+      <c r="D28" s="14" t="inlineStr">
         <is>
           <t>Card da planilha</t>
         </is>
       </c>
-      <c r="D28" s="13" t="inlineStr">
+      <c r="E28" s="14" t="inlineStr">
         <is>
           <t>451681</t>
         </is>
       </c>
-      <c r="E28" s="13" t="inlineStr">
+      <c r="F28" s="14" t="inlineStr">
         <is>
           <t>[DP] Migração GCP | Migrar Backend -&gt; portal de cadastro (adaptações)</t>
         </is>
       </c>
-      <c r="F28" s="13" t="inlineStr">
+      <c r="G28" s="14" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="G28" s="13" t="inlineStr">
+      <c r="H28" s="14" t="inlineStr">
         <is>
           <t>Ajuste de codigo, versao, eventual erro</t>
         </is>
       </c>
-      <c r="H28" s="13" t="inlineStr">
+      <c r="I28" s="14" t="inlineStr">
         <is>
           <t>10/02/27</t>
         </is>
       </c>
-      <c r="I28" s="13" t="inlineStr">
+      <c r="J28" s="14" t="inlineStr">
         <is>
           <t>Back End</t>
         </is>
       </c>
-      <c r="J28" s="13" t="n"/>
-      <c r="K28" s="13" t="inlineStr">
+      <c r="K28" s="14" t="n"/>
+      <c r="L28" s="14" t="inlineStr">
         <is>
           <t>Adaptação do backend do portal. A data 10/02/27 não define a posição. O card não cita Airflow no texto; o workload do portal cita.</t>
         </is>
       </c>
-      <c r="L28" s="13" t="inlineStr">
+      <c r="M28" s="14" t="inlineStr">
         <is>
           <t>No bloco do portal, junto dos workloads que a planilha amarra à carga. A data de fevereiro ficou para trás da adequação do Airflow de propósito.</t>
         </is>
       </c>
-      <c r="M28" s="14" t="inlineStr">
+      <c r="N28" s="15" t="inlineStr">
         <is>
           <t>https://dasa.businessmap.io/ctrl_board/96/cards/451681/details</t>
         </is>
       </c>
-      <c r="N28" s="13" t="n">
+      <c r="O28" s="14" t="n">
         <v>12</v>
       </c>
     </row>
     <row r="29" ht="52" customHeight="1">
-      <c r="A29" s="13" t="n">
+      <c r="A29" s="14" t="n">
         <v>28</v>
       </c>
-      <c r="B29" s="13" t="inlineStr">
+      <c r="B29" s="14" t="inlineStr">
         <is>
           <t>7. HML — portal, depois da carga que ele cita</t>
         </is>
       </c>
-      <c r="C29" s="13" t="inlineStr">
+      <c r="C29" s="14" t="n"/>
+      <c r="D29" s="14" t="inlineStr">
         <is>
           <t>Card da planilha</t>
         </is>
       </c>
-      <c r="D29" s="13" t="inlineStr">
+      <c r="E29" s="14" t="inlineStr">
         <is>
           <t>451677</t>
         </is>
       </c>
-      <c r="E29" s="13" t="inlineStr">
+      <c r="F29" s="14" t="inlineStr">
         <is>
           <t>[DP] Migração GCP | Migrar Frontend  Protal de cadastro (adaptações)</t>
         </is>
       </c>
-      <c r="F29" s="13" t="inlineStr">
+      <c r="G29" s="14" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="G29" s="13" t="inlineStr">
+      <c r="H29" s="14" t="inlineStr">
         <is>
           <t>Ajuste de codigo, versao, eventual erro</t>
         </is>
       </c>
-      <c r="H29" s="13" t="inlineStr">
+      <c r="I29" s="14" t="inlineStr">
         <is>
           <t>07/02/27</t>
         </is>
       </c>
-      <c r="I29" s="13" t="inlineStr">
+      <c r="J29" s="14" t="inlineStr">
         <is>
           <t>Back End</t>
         </is>
       </c>
-      <c r="J29" s="13" t="inlineStr">
+      <c r="K29" s="14" t="inlineStr">
         <is>
           <t>só é possivel testar o front com tudo integrado.</t>
         </is>
       </c>
-      <c r="K29" s="13" t="inlineStr">
+      <c r="L29" s="14" t="inlineStr">
         <is>
           <t>A observação condiciona o teste à integração. A data 07/02/27 não define a posição.</t>
         </is>
       </c>
-      <c r="L29" s="13" t="inlineStr">
+      <c r="M29" s="14" t="inlineStr">
         <is>
           <t>A adaptação fica neste bloco. O teste do front é o card 451689.</t>
         </is>
       </c>
-      <c r="M29" s="14" t="inlineStr">
+      <c r="N29" s="15" t="inlineStr">
         <is>
           <t>https://dasa.businessmap.io/ctrl_board/96/cards/451677/details</t>
         </is>
       </c>
-      <c r="N29" s="13" t="n">
+      <c r="O29" s="14" t="n">
         <v>11</v>
       </c>
     </row>
     <row r="30" ht="52" customHeight="1">
-      <c r="A30" s="15" t="n">
+      <c r="A30" s="16" t="n">
         <v>29</v>
       </c>
-      <c r="B30" s="15" t="inlineStr">
+      <c r="B30" s="16" t="inlineStr">
         <is>
           <t>8. HML — teste funcional, e em seguida carga</t>
         </is>
       </c>
-      <c r="C30" s="15" t="inlineStr">
+      <c r="C30" s="16" t="n"/>
+      <c r="D30" s="16" t="inlineStr">
         <is>
           <t>Card da planilha</t>
         </is>
       </c>
-      <c r="D30" s="15" t="inlineStr">
+      <c r="E30" s="16" t="inlineStr">
         <is>
           <t>451689</t>
         </is>
       </c>
-      <c r="E30" s="15" t="inlineStr">
+      <c r="F30" s="16" t="inlineStr">
         <is>
           <t>[DP] Migração GCP | Testes Integrados, Homologação &amp; Plano de Rollback</t>
         </is>
       </c>
-      <c r="F30" s="15" t="inlineStr">
+      <c r="G30" s="16" t="inlineStr">
         <is>
           <t>Sem Definição de Escopo</t>
         </is>
       </c>
-      <c r="G30" s="15" t="inlineStr">
+      <c r="H30" s="16" t="inlineStr">
         <is>
           <t>??</t>
         </is>
       </c>
-      <c r="H30" s="15" t="n"/>
-      <c r="I30" s="15" t="n"/>
-      <c r="J30" s="15" t="n"/>
-      <c r="K30" s="15" t="inlineStr">
+      <c r="I30" s="16" t="n"/>
+      <c r="J30" s="16" t="n"/>
+      <c r="K30" s="16" t="n"/>
+      <c r="L30" s="16" t="inlineStr">
         <is>
           <t>Único card de teste. Não cita teste de carga. Sem definição de escopo. O template do documento lista teste funcional, performance, segurança e DR, todos sem conteúdo. Os fronts 451677 e 469051 dizem que só testam com tudo integrado.</t>
         </is>
       </c>
-      <c r="L30" s="15" t="inlineStr">
+      <c r="M30" s="16" t="inlineStr">
         <is>
           <t>Fecha o que a planilha chama de homologação. Produção só começa depois deste card e do teste de carga.</t>
         </is>
       </c>
-      <c r="M30" s="16" t="inlineStr">
+      <c r="N30" s="17" t="inlineStr">
         <is>
           <t>https://dasa.businessmap.io/ctrl_board/96/cards/451689/details</t>
         </is>
       </c>
-      <c r="N30" s="15" t="n">
+      <c r="O30" s="16" t="n">
         <v>36</v>
       </c>
     </row>
     <row r="31" ht="52" customHeight="1">
-      <c r="A31" s="17" t="n">
+      <c r="A31" s="18" t="n">
         <v>30</v>
       </c>
-      <c r="B31" s="17" t="inlineStr">
+      <c r="B31" s="18" t="inlineStr">
         <is>
           <t>8. HML — teste funcional, e em seguida carga</t>
         </is>
       </c>
-      <c r="C31" s="17" t="inlineStr">
+      <c r="C31" s="19" t="inlineStr">
+        <is>
+          <t>Inclusa por IA — gap identificado</t>
+        </is>
+      </c>
+      <c r="D31" s="18" t="inlineStr">
         <is>
           <t>Marco pedido, sem card</t>
         </is>
       </c>
-      <c r="D31" s="17" t="n"/>
-      <c r="E31" s="17" t="inlineStr">
+      <c r="E31" s="18" t="n"/>
+      <c r="F31" s="18" t="inlineStr">
         <is>
           <t>Teste de carga em HML</t>
         </is>
       </c>
-      <c r="F31" s="17" t="n"/>
-      <c r="G31" s="17" t="n"/>
-      <c r="H31" s="17" t="n"/>
-      <c r="I31" s="17" t="n"/>
-      <c r="J31" s="17" t="n"/>
-      <c r="K31" s="17" t="inlineStr">
+      <c r="G31" s="18" t="n"/>
+      <c r="H31" s="18" t="n"/>
+      <c r="I31" s="18" t="n"/>
+      <c r="J31" s="18" t="n"/>
+      <c r="K31" s="18" t="n"/>
+      <c r="L31" s="18" t="inlineStr">
         <is>
           <t>Pedido desta ordenação: ter tudo em HML para testes funcionais e de carga antes de planejar produção. O documento cita Performance no template de testes e não define volume, API nem meta. Nenhum card descreve o teste.</t>
         </is>
       </c>
-      <c r="L31" s="17" t="inlineStr">
+      <c r="M31" s="18" t="inlineStr">
         <is>
           <t>Depois do teste funcional. Sem cenário, volume ou API. Não é um card do BusinessMap.</t>
         </is>
       </c>
-      <c r="M31" s="17" t="n"/>
-      <c r="N31" s="17" t="n"/>
+      <c r="N31" s="18" t="n"/>
+      <c r="O31" s="18" t="n"/>
     </row>
     <row r="32" ht="52" customHeight="1">
-      <c r="A32" s="18" t="n">
+      <c r="A32" s="20" t="n">
         <v>31</v>
       </c>
-      <c r="B32" s="18" t="inlineStr">
-        <is>
-          <t>9. Produção — planejar depois do teste de HML</t>
-        </is>
-      </c>
-      <c r="C32" s="18" t="inlineStr">
+      <c r="B32" s="20" t="inlineStr">
+        <is>
+          <t>9. HML — Databricks na GCP, antes da produção</t>
+        </is>
+      </c>
+      <c r="C32" s="21" t="inlineStr">
+        <is>
+          <t>Inclusa por IA — gap identificado</t>
+        </is>
+      </c>
+      <c r="D32" s="20" t="inlineStr">
         <is>
           <t>Lacuna — documentação</t>
         </is>
       </c>
-      <c r="D32" s="18" t="n"/>
-      <c r="E32" s="18" t="inlineStr">
+      <c r="E32" s="20" t="n"/>
+      <c r="F32" s="20" t="inlineStr">
+        <is>
+          <t>Workspaces Databricks de HML e de PRD na GCP</t>
+        </is>
+      </c>
+      <c r="G32" s="20" t="n"/>
+      <c r="H32" s="20" t="n"/>
+      <c r="I32" s="20" t="n"/>
+      <c r="J32" s="20" t="n"/>
+      <c r="K32" s="20" t="n"/>
+      <c r="L32" s="20" t="inlineStr">
+        <is>
+          <t>A documentação lista o workspace de PRD adb-7665073515379548 e o de HML adb-887971986833958. Não há jobs, notebooks nem tabelas de saída. Não há card para levar esses workspaces à GCP. O card 478328, que pede BigQuery, está na aba de discussão.</t>
+        </is>
+      </c>
+      <c r="M32" s="20" t="inlineStr">
+        <is>
+          <t>Entra porque a decisão é levar o Databricks para a GCP e a documentação comprova que os workspaces existem. Fica depois do teste funcional: o diagrama até as APIs não passa pelo Databricks, então o teste não espera esta linha. Produção começa depois dela.</t>
+        </is>
+      </c>
+      <c r="N32" s="20" t="n"/>
+      <c r="O32" s="20" t="n"/>
+    </row>
+    <row r="33" ht="52" customHeight="1">
+      <c r="A33" s="22" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="22" t="inlineStr">
+        <is>
+          <t>10. Produção — planejar depois do teste de HML</t>
+        </is>
+      </c>
+      <c r="C33" s="23" t="inlineStr">
+        <is>
+          <t>Inclusa por IA — gap identificado</t>
+        </is>
+      </c>
+      <c r="D33" s="22" t="inlineStr">
+        <is>
+          <t>Lacuna — documentação</t>
+        </is>
+      </c>
+      <c r="E33" s="22" t="n"/>
+      <c r="F33" s="22" t="inlineStr">
         <is>
           <t>GKE de produção</t>
         </is>
       </c>
-      <c r="F32" s="18" t="n"/>
-      <c r="G32" s="18" t="n"/>
-      <c r="H32" s="18" t="n"/>
-      <c r="I32" s="18" t="n"/>
-      <c r="J32" s="18" t="n"/>
-      <c r="K32" s="18" t="inlineStr">
+      <c r="G33" s="22" t="n"/>
+      <c r="H33" s="22" t="n"/>
+      <c r="I33" s="22" t="n"/>
+      <c r="J33" s="22" t="n"/>
+      <c r="K33" s="22" t="n"/>
+      <c r="L33" s="22" t="inlineStr">
         <is>
           <t>A documentação cita o cluster aks-prd-cadastro01, namespaces busca, dataprovider-data e portal-cadastro. O único card de GKE é o de HML, concluído.</t>
         </is>
       </c>
-      <c r="L32" s="18" t="inlineStr">
+      <c r="M33" s="22" t="inlineStr">
         <is>
           <t>Primeiro item de produção porque a HML já tem cluster e a produção, no documento, também tem. Não há card.</t>
         </is>
       </c>
-      <c r="M32" s="18" t="n"/>
-      <c r="N32" s="18" t="n"/>
-    </row>
-    <row r="33" ht="52" customHeight="1">
-      <c r="A33" s="19" t="n">
-        <v>32</v>
-      </c>
-      <c r="B33" s="19" t="inlineStr">
-        <is>
-          <t>9. Produção — planejar depois do teste de HML</t>
-        </is>
-      </c>
-      <c r="C33" s="19" t="inlineStr">
+      <c r="N33" s="22" t="n"/>
+      <c r="O33" s="22" t="n"/>
+    </row>
+    <row r="34" ht="52" customHeight="1">
+      <c r="A34" s="24" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="24" t="inlineStr">
+        <is>
+          <t>10. Produção — planejar depois do teste de HML</t>
+        </is>
+      </c>
+      <c r="C34" s="24" t="n"/>
+      <c r="D34" s="24" t="inlineStr">
         <is>
           <t>Card da planilha</t>
         </is>
       </c>
-      <c r="D33" s="19" t="inlineStr">
+      <c r="E34" s="24" t="inlineStr">
         <is>
           <t>470150</t>
         </is>
       </c>
-      <c r="E33" s="19" t="inlineStr">
+      <c r="F34" s="24" t="inlineStr">
         <is>
           <t>Criação de Workloads do projeto DATAPROVIDER-DATA -&gt; dp-data-stack-airflow-prd-worker-statefulset</t>
         </is>
       </c>
-      <c r="F33" s="19" t="inlineStr">
+      <c r="G34" s="24" t="inlineStr">
         <is>
           <t>Média</t>
         </is>
       </c>
-      <c r="G33" s="19" t="inlineStr">
+      <c r="H34" s="24" t="inlineStr">
         <is>
           <t>infra managedAirFlow - infra =&gt; sem data depende de infra</t>
         </is>
       </c>
-      <c r="H33" s="19" t="inlineStr">
+      <c r="I34" s="24" t="inlineStr">
         <is>
           <t>09/10/26</t>
         </is>
       </c>
-      <c r="I33" s="19" t="inlineStr">
+      <c r="J34" s="24" t="inlineStr">
         <is>
           <t>Infra</t>
         </is>
       </c>
-      <c r="J33" s="19" t="inlineStr">
+      <c r="K34" s="24" t="inlineStr">
         <is>
           <t>infra</t>
         </is>
       </c>
-      <c r="K33" s="19" t="inlineStr">
+      <c r="L34" s="24" t="inlineStr">
         <is>
           <t>Nome com prd. Data escrita 09/10/26. A dependência é infra, não a POC do Airflow.</t>
         </is>
       </c>
-      <c r="L33" s="19" t="inlineStr">
+      <c r="M34" s="24" t="inlineStr">
         <is>
           <t>Produção, pelo nome. A data 09/10/26 não trouxe este card para antes da HML.</t>
         </is>
       </c>
-      <c r="M33" s="20" t="inlineStr">
+      <c r="N34" s="25" t="inlineStr">
         <is>
           <t>https://dasa.businessmap.io/ctrl_board/96/cards/470150/details</t>
         </is>
       </c>
-      <c r="N33" s="19" t="n">
+      <c r="O34" s="24" t="n">
         <v>23</v>
       </c>
     </row>
-    <row r="34" ht="52" customHeight="1">
-      <c r="A34" s="19" t="n">
-        <v>33</v>
-      </c>
-      <c r="B34" s="19" t="inlineStr">
-        <is>
-          <t>9. Produção — planejar depois do teste de HML</t>
-        </is>
-      </c>
-      <c r="C34" s="19" t="inlineStr">
+    <row r="35" ht="52" customHeight="1">
+      <c r="A35" s="24" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="24" t="inlineStr">
+        <is>
+          <t>10. Produção — planejar depois do teste de HML</t>
+        </is>
+      </c>
+      <c r="C35" s="24" t="n"/>
+      <c r="D35" s="24" t="inlineStr">
         <is>
           <t>Card da planilha</t>
         </is>
       </c>
-      <c r="D34" s="19" t="inlineStr">
+      <c r="E35" s="24" t="inlineStr">
         <is>
           <t>470149</t>
         </is>
       </c>
-      <c r="E34" s="19" t="inlineStr">
+      <c r="F35" s="24" t="inlineStr">
         <is>
           <t>Criação de Workloads do projeto DATAPROVIDER-DATA -&gt; dp-data-stack-airflow-prd</t>
         </is>
       </c>
-      <c r="F34" s="19" t="inlineStr">
+      <c r="G35" s="24" t="inlineStr">
         <is>
           <t>Média</t>
         </is>
       </c>
-      <c r="G34" s="19" t="inlineStr">
+      <c r="H35" s="24" t="inlineStr">
         <is>
           <t>infra managedAirFlow - infra =&gt; sem data depende de infra</t>
         </is>
       </c>
-      <c r="H34" s="19" t="inlineStr">
+      <c r="I35" s="24" t="inlineStr">
         <is>
           <t>09/10/26</t>
         </is>
       </c>
-      <c r="I34" s="19" t="inlineStr">
+      <c r="J35" s="24" t="inlineStr">
         <is>
           <t>Infra</t>
         </is>
       </c>
-      <c r="J34" s="19" t="inlineStr">
+      <c r="K35" s="24" t="inlineStr">
         <is>
           <t>infra</t>
         </is>
       </c>
-      <c r="K34" s="19" t="inlineStr">
+      <c r="L35" s="24" t="inlineStr">
         <is>
           <t>Nome com prd. Data escrita 09/10/26.</t>
         </is>
       </c>
-      <c r="L34" s="19" t="inlineStr">
+      <c r="M35" s="24" t="inlineStr">
         <is>
           <t>No bloco de produção, na ordem em que a planilha lista os workloads de Airflow.</t>
         </is>
       </c>
-      <c r="M34" s="20" t="inlineStr">
+      <c r="N35" s="25" t="inlineStr">
         <is>
           <t>https://dasa.businessmap.io/ctrl_board/96/cards/470149/details</t>
         </is>
       </c>
-      <c r="N34" s="19" t="n">
+      <c r="O35" s="24" t="n">
         <v>24</v>
       </c>
     </row>
-    <row r="35" ht="52" customHeight="1">
-      <c r="A35" s="19" t="n">
+    <row r="36" ht="52" customHeight="1">
+      <c r="A36" s="24" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="24" t="inlineStr">
+        <is>
+          <t>10. Produção — planejar depois do teste de HML</t>
+        </is>
+      </c>
+      <c r="C36" s="24" t="n"/>
+      <c r="D36" s="24" t="inlineStr">
+        <is>
+          <t>Card da planilha</t>
+        </is>
+      </c>
+      <c r="E36" s="24" t="inlineStr">
+        <is>
+          <t>470148</t>
+        </is>
+      </c>
+      <c r="F36" s="24" t="inlineStr">
+        <is>
+          <t>Criação de Workloads do projeto DATAPROVIDER-DATA -&gt; dp-data-stack-airflow-prd-sync-users</t>
+        </is>
+      </c>
+      <c r="G36" s="24" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="H36" s="24" t="inlineStr">
+        <is>
+          <t>infra managedAirFlow - infra =&gt; sem data depende de infra</t>
+        </is>
+      </c>
+      <c r="I36" s="24" t="inlineStr">
+        <is>
+          <t>09/10/26</t>
+        </is>
+      </c>
+      <c r="J36" s="24" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="K36" s="24" t="inlineStr">
+        <is>
+          <t>infra</t>
+        </is>
+      </c>
+      <c r="L36" s="24" t="inlineStr">
+        <is>
+          <t>Nome com prd. Data escrita 09/10/26.</t>
+        </is>
+      </c>
+      <c r="M36" s="24" t="inlineStr">
+        <is>
+          <t>No bloco de produção, na ordem original.</t>
+        </is>
+      </c>
+      <c r="N36" s="25" t="inlineStr">
+        <is>
+          <t>https://dasa.businessmap.io/ctrl_board/96/cards/470148/details</t>
+        </is>
+      </c>
+      <c r="O36" s="24" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="37" ht="52" customHeight="1">
+      <c r="A37" s="24" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="24" t="inlineStr">
+        <is>
+          <t>10. Produção — planejar depois do teste de HML</t>
+        </is>
+      </c>
+      <c r="C37" s="24" t="n"/>
+      <c r="D37" s="24" t="inlineStr">
+        <is>
+          <t>Card da planilha</t>
+        </is>
+      </c>
+      <c r="E37" s="24" t="inlineStr">
+        <is>
+          <t>470146</t>
+        </is>
+      </c>
+      <c r="F37" s="24" t="inlineStr">
+        <is>
+          <t>Criação de Workloads do projeto DATAPROVIDER-DATA -&gt; dp-data-stack-airflow-prd-scheduler</t>
+        </is>
+      </c>
+      <c r="G37" s="24" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="H37" s="24" t="inlineStr">
+        <is>
+          <t>infra managedAirFlow - infra =&gt; sem data depende de infra</t>
+        </is>
+      </c>
+      <c r="I37" s="24" t="inlineStr">
+        <is>
+          <t>09/10/26</t>
+        </is>
+      </c>
+      <c r="J37" s="24" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="K37" s="24" t="inlineStr">
+        <is>
+          <t>infra</t>
+        </is>
+      </c>
+      <c r="L37" s="24" t="inlineStr">
+        <is>
+          <t>Nome com prd. Data escrita 09/10/26.</t>
+        </is>
+      </c>
+      <c r="M37" s="24" t="inlineStr">
+        <is>
+          <t>No bloco de produção, na ordem original.</t>
+        </is>
+      </c>
+      <c r="N37" s="25" t="inlineStr">
+        <is>
+          <t>https://dasa.businessmap.io/ctrl_board/96/cards/470146/details</t>
+        </is>
+      </c>
+      <c r="O37" s="24" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="38" ht="52" customHeight="1">
+      <c r="A38" s="24" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="24" t="inlineStr">
+        <is>
+          <t>10. Produção — planejar depois do teste de HML</t>
+        </is>
+      </c>
+      <c r="C38" s="24" t="n"/>
+      <c r="D38" s="24" t="inlineStr">
+        <is>
+          <t>Card da planilha</t>
+        </is>
+      </c>
+      <c r="E38" s="24" t="inlineStr">
+        <is>
+          <t>470145</t>
+        </is>
+      </c>
+      <c r="F38" s="24" t="inlineStr">
+        <is>
+          <t>Criação de Workloads do projeto DATAPROVIDER-DATA -&gt; dp-data-stack-airflow-prd-flower</t>
+        </is>
+      </c>
+      <c r="G38" s="24" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="H38" s="24" t="inlineStr">
+        <is>
+          <t>infra managedAirFlow - infra =&gt; sem data depende de infra</t>
+        </is>
+      </c>
+      <c r="I38" s="24" t="inlineStr">
+        <is>
+          <t>09/10/26</t>
+        </is>
+      </c>
+      <c r="J38" s="24" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="K38" s="24" t="inlineStr">
+        <is>
+          <t>infra</t>
+        </is>
+      </c>
+      <c r="L38" s="24" t="inlineStr">
+        <is>
+          <t>Nome com prd. Data escrita 09/10/26.</t>
+        </is>
+      </c>
+      <c r="M38" s="24" t="inlineStr">
+        <is>
+          <t>No bloco de produção, na ordem original.</t>
+        </is>
+      </c>
+      <c r="N38" s="25" t="inlineStr">
+        <is>
+          <t>https://dasa.businessmap.io/ctrl_board/96/cards/470145/details</t>
+        </is>
+      </c>
+      <c r="O38" s="24" t="n">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="39" ht="52" customHeight="1">
+      <c r="A39" s="24" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="24" t="inlineStr">
+        <is>
+          <t>10. Produção — planejar depois do teste de HML</t>
+        </is>
+      </c>
+      <c r="C39" s="24" t="n"/>
+      <c r="D39" s="24" t="inlineStr">
+        <is>
+          <t>Card da planilha</t>
+        </is>
+      </c>
+      <c r="E39" s="24" t="inlineStr">
+        <is>
+          <t>468978</t>
+        </is>
+      </c>
+      <c r="F39" s="24" t="inlineStr">
+        <is>
+          <t>Criação de Workloads do projeto DATAPROVIDER-DATA -&gt; dp-data-stack-airflow-prd-db-migrations</t>
+        </is>
+      </c>
+      <c r="G39" s="24" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="H39" s="24" t="inlineStr">
+        <is>
+          <t>infra managedAirFlow - infra</t>
+        </is>
+      </c>
+      <c r="I39" s="24" t="inlineStr">
+        <is>
+          <t>09/10/26</t>
+        </is>
+      </c>
+      <c r="J39" s="24" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="K39" s="24" t="inlineStr">
+        <is>
+          <t>infra</t>
+        </is>
+      </c>
+      <c r="L39" s="24" t="inlineStr">
+        <is>
+          <t>Nome com prd. Data escrita 09/10/26.</t>
+        </is>
+      </c>
+      <c r="M39" s="24" t="inlineStr">
+        <is>
+          <t>No bloco de produção, na ordem original.</t>
+        </is>
+      </c>
+      <c r="N39" s="25" t="inlineStr">
+        <is>
+          <t>https://dasa.businessmap.io/ctrl_board/96/cards/468978/details</t>
+        </is>
+      </c>
+      <c r="O39" s="24" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="40" ht="52" customHeight="1">
+      <c r="A40" s="24" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="24" t="inlineStr">
+        <is>
+          <t>10. Produção — planejar depois do teste de HML</t>
+        </is>
+      </c>
+      <c r="C40" s="24" t="n"/>
+      <c r="D40" s="24" t="inlineStr">
+        <is>
+          <t>Card da planilha</t>
+        </is>
+      </c>
+      <c r="E40" s="24" t="inlineStr">
+        <is>
+          <t>451683</t>
+        </is>
+      </c>
+      <c r="F40" s="24" t="inlineStr">
+        <is>
+          <t>[DP] Migração GCP | Event Hub para Pub/Sub</t>
+        </is>
+      </c>
+      <c r="G40" s="24" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="H40" s="24" t="inlineStr">
+        <is>
+          <t>Ultima demanda, por ultimo -&gt; falar depois</t>
+        </is>
+      </c>
+      <c r="I40" s="24" t="n"/>
+      <c r="J40" s="24" t="inlineStr">
+        <is>
+          <t>BD</t>
+        </is>
+      </c>
+      <c r="K40" s="24" t="inlineStr">
+        <is>
+          <t>pode ficar por ultimo</t>
+        </is>
+      </c>
+      <c r="L40" s="24" t="inlineStr">
+        <is>
+          <t>A documentação lista o Event Hub data-provider-prd. O desenho GCP tem Pub/Sub na ingestão. A planilha manda deixar por último. Nenhuma API cita Event Hub como dependência.</t>
+        </is>
+      </c>
+      <c r="M40" s="24" t="inlineStr">
+        <is>
+          <t>No fim da produção, antes do cutover. Fora do teste funcional de HML, como o card pede.</t>
+        </is>
+      </c>
+      <c r="N40" s="25" t="inlineStr">
+        <is>
+          <t>https://dasa.businessmap.io/ctrl_board/96/cards/451683/details</t>
+        </is>
+      </c>
+      <c r="O40" s="24" t="n">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="41" ht="52" customHeight="1">
+      <c r="A41" s="24" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="24" t="inlineStr">
+        <is>
+          <t>10. Produção — planejar depois do teste de HML</t>
+        </is>
+      </c>
+      <c r="C41" s="24" t="n"/>
+      <c r="D41" s="24" t="inlineStr">
+        <is>
+          <t>Card da planilha</t>
+        </is>
+      </c>
+      <c r="E41" s="24" t="inlineStr">
+        <is>
+          <t>451691</t>
+        </is>
+      </c>
+      <c r="F41" s="24" t="inlineStr">
+        <is>
+          <t>[DP] Migração GCP | Cutover &amp; Go-Live</t>
+        </is>
+      </c>
+      <c r="G41" s="24" t="inlineStr">
+        <is>
+          <t>Sem Definição de Escopo</t>
+        </is>
+      </c>
+      <c r="H41" s="24" t="inlineStr">
+        <is>
+          <t>??</t>
+        </is>
+      </c>
+      <c r="I41" s="24" t="n"/>
+      <c r="J41" s="24" t="n"/>
+      <c r="K41" s="24" t="n"/>
+      <c r="L41" s="24" t="inlineStr">
+        <is>
+          <t>Sem definição de escopo. O template do documento deixa em branco big bang ou gradual, DNS e janela.</t>
+        </is>
+      </c>
+      <c r="M41" s="24" t="inlineStr">
+        <is>
+          <t>Última linha de produção. Sem escopo preenchido.</t>
+        </is>
+      </c>
+      <c r="N41" s="25" t="inlineStr">
+        <is>
+          <t>https://dasa.businessmap.io/ctrl_board/96/cards/451691/details</t>
+        </is>
+      </c>
+      <c r="O41" s="24" t="n">
         <v>34</v>
       </c>
-      <c r="B35" s="19" t="inlineStr">
-        <is>
-          <t>9. Produção — planejar depois do teste de HML</t>
-        </is>
-      </c>
-      <c r="C35" s="19" t="inlineStr">
+    </row>
+    <row r="42" ht="52" customHeight="1">
+      <c r="A42" s="26" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="26" t="inlineStr">
+        <is>
+          <t>Encerrada pela equipe</t>
+        </is>
+      </c>
+      <c r="C42" s="26" t="inlineStr">
+        <is>
+          <t>Equipe — encerrada</t>
+        </is>
+      </c>
+      <c r="D42" s="26" t="inlineStr">
         <is>
           <t>Card da planilha</t>
         </is>
       </c>
-      <c r="D35" s="19" t="inlineStr">
-        <is>
-          <t>470148</t>
-        </is>
-      </c>
-      <c r="E35" s="19" t="inlineStr">
-        <is>
-          <t>Criação de Workloads do projeto DATAPROVIDER-DATA -&gt; dp-data-stack-airflow-prd-sync-users</t>
-        </is>
-      </c>
-      <c r="F35" s="19" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="G35" s="19" t="inlineStr">
-        <is>
-          <t>infra managedAirFlow - infra =&gt; sem data depende de infra</t>
-        </is>
-      </c>
-      <c r="H35" s="19" t="inlineStr">
-        <is>
-          <t>09/10/26</t>
-        </is>
-      </c>
-      <c r="I35" s="19" t="inlineStr">
-        <is>
-          <t>Infra</t>
-        </is>
-      </c>
-      <c r="J35" s="19" t="inlineStr">
-        <is>
-          <t>infra</t>
-        </is>
-      </c>
-      <c r="K35" s="19" t="inlineStr">
-        <is>
-          <t>Nome com prd. Data escrita 09/10/26.</t>
-        </is>
-      </c>
-      <c r="L35" s="19" t="inlineStr">
-        <is>
-          <t>No bloco de produção, na ordem original.</t>
-        </is>
-      </c>
-      <c r="M35" s="20" t="inlineStr">
-        <is>
-          <t>https://dasa.businessmap.io/ctrl_board/96/cards/470148/details</t>
-        </is>
-      </c>
-      <c r="N35" s="19" t="n">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="36" ht="52" customHeight="1">
-      <c r="A36" s="19" t="n">
-        <v>35</v>
-      </c>
-      <c r="B36" s="19" t="inlineStr">
-        <is>
-          <t>9. Produção — planejar depois do teste de HML</t>
-        </is>
-      </c>
-      <c r="C36" s="19" t="inlineStr">
+      <c r="E42" s="26" t="inlineStr">
+        <is>
+          <t>470119</t>
+        </is>
+      </c>
+      <c r="F42" s="26" t="inlineStr">
+        <is>
+          <t>Criação de Workloads do projeto BUSCA -&gt; dp-backend-api</t>
+        </is>
+      </c>
+      <c r="G42" s="26" t="inlineStr">
+        <is>
+          <t>Cancelado</t>
+        </is>
+      </c>
+      <c r="H42" s="26" t="n"/>
+      <c r="I42" s="26" t="n"/>
+      <c r="J42" s="26" t="n"/>
+      <c r="K42" s="26" t="inlineStr">
+        <is>
+          <t>depende cognitiveSearch</t>
+        </is>
+      </c>
+      <c r="L42" s="26" t="inlineStr">
+        <is>
+          <t>Complexidade Cancelado. A observação cita Cognitive Search.</t>
+        </is>
+      </c>
+      <c r="M42" s="26" t="inlineStr">
+        <is>
+          <t>Cancelado pela equipe. Os backends 469049 e 468966 continuam no caminho. O documento não descreve este card além da observação de Cognitive Search.</t>
+        </is>
+      </c>
+      <c r="N42" s="27" t="inlineStr">
+        <is>
+          <t>https://dasa.businessmap.io/ctrl_board/96/cards/470119/details</t>
+        </is>
+      </c>
+      <c r="O42" s="26" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="43" ht="52" customHeight="1">
+      <c r="A43" s="26" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="26" t="inlineStr">
+        <is>
+          <t>Encerrada pela equipe</t>
+        </is>
+      </c>
+      <c r="C43" s="26" t="inlineStr">
+        <is>
+          <t>Equipe — encerrada</t>
+        </is>
+      </c>
+      <c r="D43" s="26" t="inlineStr">
         <is>
           <t>Card da planilha</t>
         </is>
       </c>
-      <c r="D36" s="19" t="inlineStr">
-        <is>
-          <t>470146</t>
-        </is>
-      </c>
-      <c r="E36" s="19" t="inlineStr">
-        <is>
-          <t>Criação de Workloads do projeto DATAPROVIDER-DATA -&gt; dp-data-stack-airflow-prd-scheduler</t>
-        </is>
-      </c>
-      <c r="F36" s="19" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="G36" s="19" t="inlineStr">
-        <is>
-          <t>infra managedAirFlow - infra =&gt; sem data depende de infra</t>
-        </is>
-      </c>
-      <c r="H36" s="19" t="inlineStr">
-        <is>
-          <t>09/10/26</t>
-        </is>
-      </c>
-      <c r="I36" s="19" t="inlineStr">
-        <is>
-          <t>Infra</t>
-        </is>
-      </c>
-      <c r="J36" s="19" t="inlineStr">
-        <is>
-          <t>infra</t>
-        </is>
-      </c>
-      <c r="K36" s="19" t="inlineStr">
-        <is>
-          <t>Nome com prd. Data escrita 09/10/26.</t>
-        </is>
-      </c>
-      <c r="L36" s="19" t="inlineStr">
-        <is>
-          <t>No bloco de produção, na ordem original.</t>
-        </is>
-      </c>
-      <c r="M36" s="20" t="inlineStr">
-        <is>
-          <t>https://dasa.businessmap.io/ctrl_board/96/cards/470146/details</t>
-        </is>
-      </c>
-      <c r="N36" s="19" t="n">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="37" ht="52" customHeight="1">
-      <c r="A37" s="19" t="n">
-        <v>36</v>
-      </c>
-      <c r="B37" s="19" t="inlineStr">
-        <is>
-          <t>9. Produção — planejar depois do teste de HML</t>
-        </is>
-      </c>
-      <c r="C37" s="19" t="inlineStr">
+      <c r="E43" s="26" t="inlineStr">
+        <is>
+          <t>451674</t>
+        </is>
+      </c>
+      <c r="F43" s="26" t="inlineStr">
+        <is>
+          <t>[DP] Migração GCP | Converter ETL's (DataBricks)</t>
+        </is>
+      </c>
+      <c r="G43" s="26" t="inlineStr">
+        <is>
+          <t>Cancelado</t>
+        </is>
+      </c>
+      <c r="H43" s="26" t="n"/>
+      <c r="I43" s="26" t="n"/>
+      <c r="J43" s="26" t="n"/>
+      <c r="K43" s="26" t="n"/>
+      <c r="L43" s="26" t="inlineStr">
+        <is>
+          <t>Complexidade Cancelado.</t>
+        </is>
+      </c>
+      <c r="M43" s="26" t="inlineStr">
+        <is>
+          <t>Fora da ordem.</t>
+        </is>
+      </c>
+      <c r="N43" s="27" t="inlineStr">
+        <is>
+          <t>https://dasa.businessmap.io/ctrl_board/96/cards/451674/details</t>
+        </is>
+      </c>
+      <c r="O43" s="26" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="44" ht="52" customHeight="1">
+      <c r="A44" s="26" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="26" t="inlineStr">
+        <is>
+          <t>Encerrada pela equipe</t>
+        </is>
+      </c>
+      <c r="C44" s="26" t="inlineStr">
+        <is>
+          <t>Equipe — encerrada</t>
+        </is>
+      </c>
+      <c r="D44" s="26" t="inlineStr">
         <is>
           <t>Card da planilha</t>
         </is>
       </c>
-      <c r="D37" s="19" t="inlineStr">
-        <is>
-          <t>470145</t>
-        </is>
-      </c>
-      <c r="E37" s="19" t="inlineStr">
-        <is>
-          <t>Criação de Workloads do projeto DATAPROVIDER-DATA -&gt; dp-data-stack-airflow-prd-flower</t>
-        </is>
-      </c>
-      <c r="F37" s="19" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="G37" s="19" t="inlineStr">
-        <is>
-          <t>infra managedAirFlow - infra =&gt; sem data depende de infra</t>
-        </is>
-      </c>
-      <c r="H37" s="19" t="inlineStr">
-        <is>
-          <t>09/10/26</t>
-        </is>
-      </c>
-      <c r="I37" s="19" t="inlineStr">
-        <is>
-          <t>Infra</t>
-        </is>
-      </c>
-      <c r="J37" s="19" t="inlineStr">
-        <is>
-          <t>infra</t>
-        </is>
-      </c>
-      <c r="K37" s="19" t="inlineStr">
-        <is>
-          <t>Nome com prd. Data escrita 09/10/26.</t>
-        </is>
-      </c>
-      <c r="L37" s="19" t="inlineStr">
-        <is>
-          <t>No bloco de produção, na ordem original.</t>
-        </is>
-      </c>
-      <c r="M37" s="20" t="inlineStr">
-        <is>
-          <t>https://dasa.businessmap.io/ctrl_board/96/cards/470145/details</t>
-        </is>
-      </c>
-      <c r="N37" s="19" t="n">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="38" ht="52" customHeight="1">
-      <c r="A38" s="19" t="n">
+      <c r="E44" s="26" t="inlineStr">
+        <is>
+          <t>424941</t>
+        </is>
+      </c>
+      <c r="F44" s="26" t="inlineStr">
+        <is>
+          <t>[DP] PostgreSQL - Levantamento de recursos para reescrita de código</t>
+        </is>
+      </c>
+      <c r="G44" s="26" t="inlineStr">
+        <is>
+          <t>Cancelado</t>
+        </is>
+      </c>
+      <c r="H44" s="26" t="n"/>
+      <c r="I44" s="26" t="n"/>
+      <c r="J44" s="26" t="n"/>
+      <c r="K44" s="26" t="n"/>
+      <c r="L44" s="26" t="inlineStr">
+        <is>
+          <t>Complexidade Cancelado.</t>
+        </is>
+      </c>
+      <c r="M44" s="26" t="inlineStr">
+        <is>
+          <t>Fora da ordem.</t>
+        </is>
+      </c>
+      <c r="N44" s="27" t="inlineStr">
+        <is>
+          <t>https://dasa.businessmap.io/ctrl_board/96/cards/424941/details</t>
+        </is>
+      </c>
+      <c r="O44" s="26" t="n">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="45" ht="52" customHeight="1">
+      <c r="A45" s="26" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="26" t="inlineStr">
+        <is>
+          <t>Encerrada pela equipe</t>
+        </is>
+      </c>
+      <c r="C45" s="26" t="inlineStr">
+        <is>
+          <t>Equipe — encerrada</t>
+        </is>
+      </c>
+      <c r="D45" s="26" t="inlineStr">
+        <is>
+          <t>Card da planilha</t>
+        </is>
+      </c>
+      <c r="E45" s="26" t="inlineStr">
+        <is>
+          <t>451676</t>
+        </is>
+      </c>
+      <c r="F45" s="26" t="inlineStr">
+        <is>
+          <t>[DP] Migração GCP | Migrar banco de dados SQL Server -- ABORTADO</t>
+        </is>
+      </c>
+      <c r="G45" s="26" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="H45" s="26" t="n"/>
+      <c r="I45" s="26" t="n"/>
+      <c r="J45" s="26" t="n"/>
+      <c r="K45" s="26" t="n"/>
+      <c r="L45" s="26" t="inlineStr">
+        <is>
+          <t>Título ABORTADO e status Concluído. A documentação diz que a réplica 3 não será migrada e está desligada. Master com 10 vCores, réplica com 18, HML com 6, staging com 2. Tamanho citado: 461 GB.</t>
+        </is>
+      </c>
+      <c r="M45" s="26" t="inlineStr">
+        <is>
+          <t>Fora do caminho. A existência de réplica em produção não virou atividade.</t>
+        </is>
+      </c>
+      <c r="N45" s="27" t="inlineStr">
+        <is>
+          <t>https://dasa.businessmap.io/ctrl_board/96/cards/451676/details</t>
+        </is>
+      </c>
+      <c r="O45" s="26" t="n">
         <v>37</v>
       </c>
-      <c r="B38" s="19" t="inlineStr">
-        <is>
-          <t>9. Produção — planejar depois do teste de HML</t>
-        </is>
-      </c>
-      <c r="C38" s="19" t="inlineStr">
-        <is>
-          <t>Card da planilha</t>
-        </is>
-      </c>
-      <c r="D38" s="19" t="inlineStr">
-        <is>
-          <t>468978</t>
-        </is>
-      </c>
-      <c r="E38" s="19" t="inlineStr">
-        <is>
-          <t>Criação de Workloads do projeto DATAPROVIDER-DATA -&gt; dp-data-stack-airflow-prd-db-migrations</t>
-        </is>
-      </c>
-      <c r="F38" s="19" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="G38" s="19" t="inlineStr">
-        <is>
-          <t>infra managedAirFlow - infra</t>
-        </is>
-      </c>
-      <c r="H38" s="19" t="inlineStr">
-        <is>
-          <t>09/10/26</t>
-        </is>
-      </c>
-      <c r="I38" s="19" t="inlineStr">
-        <is>
-          <t>Infra</t>
-        </is>
-      </c>
-      <c r="J38" s="19" t="inlineStr">
-        <is>
-          <t>infra</t>
-        </is>
-      </c>
-      <c r="K38" s="19" t="inlineStr">
-        <is>
-          <t>Nome com prd. Data escrita 09/10/26.</t>
-        </is>
-      </c>
-      <c r="L38" s="19" t="inlineStr">
-        <is>
-          <t>No bloco de produção, na ordem original.</t>
-        </is>
-      </c>
-      <c r="M38" s="20" t="inlineStr">
-        <is>
-          <t>https://dasa.businessmap.io/ctrl_board/96/cards/468978/details</t>
-        </is>
-      </c>
-      <c r="N38" s="19" t="n">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="39" ht="52" customHeight="1">
-      <c r="A39" s="19" t="n">
-        <v>38</v>
-      </c>
-      <c r="B39" s="19" t="inlineStr">
-        <is>
-          <t>9. Produção — planejar depois do teste de HML</t>
-        </is>
-      </c>
-      <c r="C39" s="19" t="inlineStr">
-        <is>
-          <t>Card da planilha</t>
-        </is>
-      </c>
-      <c r="D39" s="19" t="inlineStr">
-        <is>
-          <t>451683</t>
-        </is>
-      </c>
-      <c r="E39" s="19" t="inlineStr">
-        <is>
-          <t>[DP] Migração GCP | Event Hub para Pub/Sub</t>
-        </is>
-      </c>
-      <c r="F39" s="19" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="G39" s="19" t="inlineStr">
-        <is>
-          <t>Ultima demanda, por ultimo -&gt; falar depois</t>
-        </is>
-      </c>
-      <c r="H39" s="19" t="n"/>
-      <c r="I39" s="19" t="inlineStr">
-        <is>
-          <t>BD</t>
-        </is>
-      </c>
-      <c r="J39" s="19" t="inlineStr">
-        <is>
-          <t>pode ficar por ultimo</t>
-        </is>
-      </c>
-      <c r="K39" s="19" t="inlineStr">
-        <is>
-          <t>A documentação lista o Event Hub data-provider-prd. O desenho GCP tem Pub/Sub na ingestão. A planilha manda deixar por último. Nenhuma API cita Event Hub como dependência.</t>
-        </is>
-      </c>
-      <c r="L39" s="19" t="inlineStr">
-        <is>
-          <t>No fim da produção, antes do cutover. Fora do teste funcional de HML, como o card pede.</t>
-        </is>
-      </c>
-      <c r="M39" s="20" t="inlineStr">
-        <is>
-          <t>https://dasa.businessmap.io/ctrl_board/96/cards/451683/details</t>
-        </is>
-      </c>
-      <c r="N39" s="19" t="n">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="40" ht="52" customHeight="1">
-      <c r="A40" s="19" t="n">
-        <v>39</v>
-      </c>
-      <c r="B40" s="19" t="inlineStr">
-        <is>
-          <t>9. Produção — planejar depois do teste de HML</t>
-        </is>
-      </c>
-      <c r="C40" s="19" t="inlineStr">
-        <is>
-          <t>Card da planilha</t>
-        </is>
-      </c>
-      <c r="D40" s="19" t="inlineStr">
-        <is>
-          <t>451691</t>
-        </is>
-      </c>
-      <c r="E40" s="19" t="inlineStr">
-        <is>
-          <t>[DP] Migração GCP | Cutover &amp; Go-Live</t>
-        </is>
-      </c>
-      <c r="F40" s="19" t="inlineStr">
-        <is>
-          <t>Sem Definição de Escopo</t>
-        </is>
-      </c>
-      <c r="G40" s="19" t="inlineStr">
-        <is>
-          <t>??</t>
-        </is>
-      </c>
-      <c r="H40" s="19" t="n"/>
-      <c r="I40" s="19" t="n"/>
-      <c r="J40" s="19" t="n"/>
-      <c r="K40" s="19" t="inlineStr">
-        <is>
-          <t>Sem definição de escopo. O template do documento deixa em branco big bang ou gradual, DNS e janela.</t>
-        </is>
-      </c>
-      <c r="L40" s="19" t="inlineStr">
-        <is>
-          <t>Última linha de produção. Sem escopo preenchido.</t>
-        </is>
-      </c>
-      <c r="M40" s="20" t="inlineStr">
-        <is>
-          <t>https://dasa.businessmap.io/ctrl_board/96/cards/451691/details</t>
-        </is>
-      </c>
-      <c r="N40" s="19" t="n">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="41" ht="52" customHeight="1">
-      <c r="A41" s="21" t="n">
-        <v>40</v>
-      </c>
-      <c r="B41" s="21" t="inlineStr">
-        <is>
-          <t>10. Documentado, fora deste caminho</t>
-        </is>
-      </c>
-      <c r="C41" s="21" t="inlineStr">
-        <is>
-          <t>Card da planilha</t>
-        </is>
-      </c>
-      <c r="D41" s="21" t="inlineStr">
-        <is>
-          <t>478328</t>
-        </is>
-      </c>
-      <c r="E41" s="21" t="inlineStr">
-        <is>
-          <t>BigQuery =&gt; substituir dataBricks</t>
-        </is>
-      </c>
-      <c r="F41" s="21" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="G41" s="21" t="inlineStr">
-        <is>
-          <t>Galerinha de dados DP</t>
-        </is>
-      </c>
-      <c r="H41" s="21" t="inlineStr">
-        <is>
-          <t>29/01/27</t>
-        </is>
-      </c>
-      <c r="I41" s="21" t="inlineStr">
-        <is>
-          <t>Dados</t>
-        </is>
-      </c>
-      <c r="J41" s="21" t="inlineStr">
-        <is>
-          <t>Levar toda a orquestração do dataBricks para o BigQuery</t>
-        </is>
-      </c>
-      <c r="K41" s="21" t="inlineStr">
-        <is>
-          <t>Card mantido com o texto original. A decisão registrada é levar o Databricks para a GCP. O diagrama AS IS não desenha o Databricks no caminho até as APIs. O documento lista os workspaces de HML e de PRD e não descreve jobs. O card 451674, converter ETLs, está cancelado. O desenho GCP é uma plataforma genérica com BigQuery bronze, silver e gold; a matriz de estratégia do documento está em branco.</t>
-        </is>
-      </c>
-      <c r="L41" s="21" t="inlineStr">
-        <is>
-          <t>Fora da fila de HML e fora da produção. Nenhum outro card o cita. A data 29/01/27 não o coloca entre dezembro e fevereiro.</t>
-        </is>
-      </c>
-      <c r="M41" s="22" t="inlineStr">
-        <is>
-          <t>https://dasa.businessmap.io/ctrl_board/96/cards/478328/details</t>
-        </is>
-      </c>
-      <c r="N41" s="21" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="42" ht="52" customHeight="1">
-      <c r="A42" s="23" t="n">
-        <v>41</v>
-      </c>
-      <c r="B42" s="23" t="inlineStr">
-        <is>
-          <t>10. Documentado, fora deste caminho</t>
-        </is>
-      </c>
-      <c r="C42" s="23" t="inlineStr">
-        <is>
-          <t>Lacuna — documentação</t>
-        </is>
-      </c>
-      <c r="D42" s="23" t="n"/>
-      <c r="E42" s="23" t="inlineStr">
-        <is>
-          <t>Workspaces Databricks de HML e de PRD na GCP</t>
-        </is>
-      </c>
-      <c r="F42" s="23" t="n"/>
-      <c r="G42" s="23" t="n"/>
-      <c r="H42" s="23" t="n"/>
-      <c r="I42" s="23" t="n"/>
-      <c r="J42" s="23" t="n"/>
-      <c r="K42" s="23" t="inlineStr">
-        <is>
-          <t>A documentação lista o workspace de PRD adb-7665073515379548 e o de HML adb-887971986833958. Não há jobs, notebooks nem tabelas de saída. Não há card para levar esses workspaces à GCP. O card existente, 478328, pede BigQuery.</t>
-        </is>
-      </c>
-      <c r="L42" s="23" t="inlineStr">
-        <is>
-          <t>Não entrou na frente do teste funcional. O diagrama até as APIs não passa pelo Databricks. Sem a lista do que ele entrega, não há como saber se a API ou o portal esperam essa saída.</t>
-        </is>
-      </c>
-      <c r="M42" s="23" t="n"/>
-      <c r="N42" s="23" t="n"/>
-    </row>
-    <row r="43" ht="52" customHeight="1">
-      <c r="A43" s="23" t="n">
-        <v>42</v>
-      </c>
-      <c r="B43" s="23" t="inlineStr">
-        <is>
-          <t>10. Documentado, fora deste caminho</t>
-        </is>
-      </c>
-      <c r="C43" s="23" t="inlineStr">
-        <is>
-          <t>Lacuna — documentação</t>
-        </is>
-      </c>
-      <c r="D43" s="23" t="n"/>
-      <c r="E43" s="23" t="inlineStr">
-        <is>
-          <t>Staging SQL do caminho de ETL</t>
-        </is>
-      </c>
-      <c r="F43" s="23" t="n"/>
-      <c r="G43" s="23" t="n"/>
-      <c r="H43" s="23" t="n"/>
-      <c r="I43" s="23" t="n"/>
-      <c r="J43" s="23" t="n"/>
-      <c r="K43" s="23" t="inlineStr">
-        <is>
-          <t>A documentação lista STAGING_PRD, 2 vCores. O diagrama antigo coloca Staging no caminho de ETL. Não há card de staging.</t>
-        </is>
-      </c>
-      <c r="L43" s="23" t="inlineStr">
-        <is>
-          <t>Não sequenciado. A documentação não diz se o staging continua no Airflow que vai para a GCP.</t>
-        </is>
-      </c>
-      <c r="M43" s="23" t="n"/>
-      <c r="N43" s="23" t="n"/>
-    </row>
-    <row r="44" ht="52" customHeight="1">
-      <c r="A44" s="23" t="n">
-        <v>43</v>
-      </c>
-      <c r="B44" s="23" t="inlineStr">
-        <is>
-          <t>10. Documentado, fora deste caminho</t>
-        </is>
-      </c>
-      <c r="C44" s="23" t="inlineStr">
-        <is>
-          <t>Lacuna — documentação</t>
-        </is>
-      </c>
-      <c r="D44" s="23" t="n"/>
-      <c r="E44" s="23" t="inlineStr">
-        <is>
-          <t>dp-api-gtw e dp-cad-proxy do diagrama AS IS</t>
-        </is>
-      </c>
-      <c r="F44" s="23" t="n"/>
-      <c r="G44" s="23" t="n"/>
-      <c r="H44" s="23" t="n"/>
-      <c r="I44" s="23" t="n"/>
-      <c r="J44" s="23" t="n"/>
-      <c r="K44" s="23" t="inlineStr">
-        <is>
-          <t>O diagrama AS IS nomeia dp-api-gtw e dp-cad-proxy. O gateway com card é o Zuul (470109). dp-backend-api (470119) está cancelado. Não há card com esses dois nomes.</t>
-        </is>
-      </c>
-      <c r="L44" s="23" t="inlineStr">
-        <is>
-          <t>Não sequenciado. O diagrama não diz o que cada um faz nem se o Zuul os cobre.</t>
-        </is>
-      </c>
-      <c r="M44" s="23" t="n"/>
-      <c r="N44" s="23" t="n"/>
-    </row>
-    <row r="45" ht="52" customHeight="1">
-      <c r="A45" s="24" t="n">
-        <v>44</v>
-      </c>
-      <c r="B45" s="24" t="inlineStr">
-        <is>
-          <t>11. Fora da linha do tempo</t>
-        </is>
-      </c>
-      <c r="C45" s="24" t="inlineStr">
-        <is>
-          <t>Card da planilha</t>
-        </is>
-      </c>
-      <c r="D45" s="24" t="inlineStr">
-        <is>
-          <t>470119</t>
-        </is>
-      </c>
-      <c r="E45" s="24" t="inlineStr">
-        <is>
-          <t>Criação de Workloads do projeto BUSCA -&gt; dp-backend-api</t>
-        </is>
-      </c>
-      <c r="F45" s="24" t="inlineStr">
-        <is>
-          <t>Cancelado</t>
-        </is>
-      </c>
-      <c r="G45" s="24" t="n"/>
-      <c r="H45" s="24" t="n"/>
-      <c r="I45" s="24" t="n"/>
-      <c r="J45" s="24" t="inlineStr">
-        <is>
-          <t>depende cognitiveSearch</t>
-        </is>
-      </c>
-      <c r="K45" s="24" t="inlineStr">
-        <is>
-          <t>Complexidade Cancelado. A observação cita Cognitive Search.</t>
-        </is>
-      </c>
-      <c r="L45" s="24" t="inlineStr">
-        <is>
-          <t>Fora da ordem.</t>
-        </is>
-      </c>
-      <c r="M45" s="25" t="inlineStr">
-        <is>
-          <t>https://dasa.businessmap.io/ctrl_board/96/cards/470119/details</t>
-        </is>
-      </c>
-      <c r="N45" s="24" t="n">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="46" ht="52" customHeight="1">
-      <c r="A46" s="24" t="n">
-        <v>45</v>
-      </c>
-      <c r="B46" s="24" t="inlineStr">
-        <is>
-          <t>11. Fora da linha do tempo</t>
-        </is>
-      </c>
-      <c r="C46" s="24" t="inlineStr">
-        <is>
-          <t>Card da planilha</t>
-        </is>
-      </c>
-      <c r="D46" s="24" t="inlineStr">
-        <is>
-          <t>468985</t>
-        </is>
-      </c>
-      <c r="E46" s="24" t="inlineStr">
-        <is>
-          <t>Criação de Workloads do projeto PORTAL-CADASTRO -&gt; datp-backoffice-frontend-portal</t>
-        </is>
-      </c>
-      <c r="F46" s="24" t="inlineStr">
-        <is>
-          <t>Cancelado</t>
-        </is>
-      </c>
-      <c r="G46" s="24" t="n"/>
-      <c r="H46" s="24" t="n"/>
-      <c r="I46" s="24" t="n"/>
-      <c r="J46" s="24" t="inlineStr">
-        <is>
-          <t>depende do airFlow</t>
-        </is>
-      </c>
-      <c r="K46" s="24" t="inlineStr">
-        <is>
-          <t>Complexidade Cancelado.</t>
-        </is>
-      </c>
-      <c r="L46" s="24" t="inlineStr">
-        <is>
-          <t>Fora da ordem. O repositório correspondente continua citado na documentação.</t>
-        </is>
-      </c>
-      <c r="M46" s="25" t="inlineStr">
-        <is>
-          <t>https://dasa.businessmap.io/ctrl_board/96/cards/468985/details</t>
-        </is>
-      </c>
-      <c r="N46" s="24" t="n">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="47" ht="52" customHeight="1">
-      <c r="A47" s="24" t="n">
-        <v>46</v>
-      </c>
-      <c r="B47" s="24" t="inlineStr">
-        <is>
-          <t>11. Fora da linha do tempo</t>
-        </is>
-      </c>
-      <c r="C47" s="24" t="inlineStr">
-        <is>
-          <t>Card da planilha</t>
-        </is>
-      </c>
-      <c r="D47" s="24" t="inlineStr">
-        <is>
-          <t>470121</t>
-        </is>
-      </c>
-      <c r="E47" s="24" t="inlineStr">
-        <is>
-          <t>Criação de Workloads do projeto BUSCA -&gt; dp-corporate-frontend</t>
-        </is>
-      </c>
-      <c r="F47" s="24" t="inlineStr">
-        <is>
-          <t>Cancelado</t>
-        </is>
-      </c>
-      <c r="G47" s="24" t="n"/>
-      <c r="H47" s="24" t="n"/>
-      <c r="I47" s="24" t="n"/>
-      <c r="J47" s="24" t="n"/>
-      <c r="K47" s="24" t="inlineStr">
-        <is>
-          <t>Complexidade Cancelado. A documentação ainda cita a URL dp-corporate-frontend.</t>
-        </is>
-      </c>
-      <c r="L47" s="24" t="inlineStr">
-        <is>
-          <t>Fora da ordem. Não foi fundido com o card 469051.</t>
-        </is>
-      </c>
-      <c r="M47" s="25" t="inlineStr">
-        <is>
-          <t>https://dasa.businessmap.io/ctrl_board/96/cards/470121/details</t>
-        </is>
-      </c>
-      <c r="N47" s="24" t="n">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="48" ht="52" customHeight="1">
-      <c r="A48" s="24" t="n">
-        <v>47</v>
-      </c>
-      <c r="B48" s="24" t="inlineStr">
-        <is>
-          <t>11. Fora da linha do tempo</t>
-        </is>
-      </c>
-      <c r="C48" s="24" t="inlineStr">
-        <is>
-          <t>Card da planilha</t>
-        </is>
-      </c>
-      <c r="D48" s="24" t="inlineStr">
-        <is>
-          <t>451674</t>
-        </is>
-      </c>
-      <c r="E48" s="24" t="inlineStr">
-        <is>
-          <t>[DP] Migração GCP | Converter ETL's (DataBricks)</t>
-        </is>
-      </c>
-      <c r="F48" s="24" t="inlineStr">
-        <is>
-          <t>Cancelado</t>
-        </is>
-      </c>
-      <c r="G48" s="24" t="n"/>
-      <c r="H48" s="24" t="n"/>
-      <c r="I48" s="24" t="n"/>
-      <c r="J48" s="24" t="n"/>
-      <c r="K48" s="24" t="inlineStr">
-        <is>
-          <t>Complexidade Cancelado.</t>
-        </is>
-      </c>
-      <c r="L48" s="24" t="inlineStr">
-        <is>
-          <t>Fora da ordem.</t>
-        </is>
-      </c>
-      <c r="M48" s="25" t="inlineStr">
-        <is>
-          <t>https://dasa.businessmap.io/ctrl_board/96/cards/451674/details</t>
-        </is>
-      </c>
-      <c r="N48" s="24" t="n">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="49" ht="52" customHeight="1">
-      <c r="A49" s="24" t="n">
-        <v>48</v>
-      </c>
-      <c r="B49" s="24" t="inlineStr">
-        <is>
-          <t>11. Fora da linha do tempo</t>
-        </is>
-      </c>
-      <c r="C49" s="24" t="inlineStr">
-        <is>
-          <t>Card da planilha</t>
-        </is>
-      </c>
-      <c r="D49" s="24" t="inlineStr">
-        <is>
-          <t>424941</t>
-        </is>
-      </c>
-      <c r="E49" s="24" t="inlineStr">
-        <is>
-          <t>[DP] PostgreSQL - Levantamento de recursos para reescrita de código</t>
-        </is>
-      </c>
-      <c r="F49" s="24" t="inlineStr">
-        <is>
-          <t>Cancelado</t>
-        </is>
-      </c>
-      <c r="G49" s="24" t="n"/>
-      <c r="H49" s="24" t="n"/>
-      <c r="I49" s="24" t="n"/>
-      <c r="J49" s="24" t="n"/>
-      <c r="K49" s="24" t="inlineStr">
-        <is>
-          <t>Complexidade Cancelado.</t>
-        </is>
-      </c>
-      <c r="L49" s="24" t="inlineStr">
-        <is>
-          <t>Fora da ordem.</t>
-        </is>
-      </c>
-      <c r="M49" s="25" t="inlineStr">
-        <is>
-          <t>https://dasa.businessmap.io/ctrl_board/96/cards/424941/details</t>
-        </is>
-      </c>
-      <c r="N49" s="24" t="n">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="50" ht="52" customHeight="1">
-      <c r="A50" s="24" t="n">
-        <v>49</v>
-      </c>
-      <c r="B50" s="24" t="inlineStr">
-        <is>
-          <t>11. Fora da linha do tempo</t>
-        </is>
-      </c>
-      <c r="C50" s="24" t="inlineStr">
-        <is>
-          <t>Card da planilha</t>
-        </is>
-      </c>
-      <c r="D50" s="24" t="inlineStr">
-        <is>
-          <t>451676</t>
-        </is>
-      </c>
-      <c r="E50" s="24" t="inlineStr">
-        <is>
-          <t>[DP] Migração GCP | Migrar banco de dados SQL Server -- ABORTADO</t>
-        </is>
-      </c>
-      <c r="F50" s="24" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="G50" s="24" t="n"/>
-      <c r="H50" s="24" t="n"/>
-      <c r="I50" s="24" t="n"/>
-      <c r="J50" s="24" t="n"/>
-      <c r="K50" s="24" t="inlineStr">
-        <is>
-          <t>Título ABORTADO e status Concluído. A documentação diz que a réplica 3 não será migrada e está desligada. Master com 10 vCores, réplica com 18, HML com 6, staging com 2. Tamanho citado: 461 GB.</t>
-        </is>
-      </c>
-      <c r="L50" s="24" t="inlineStr">
-        <is>
-          <t>Fora do caminho. A existência de réplica em produção não virou atividade.</t>
-        </is>
-      </c>
-      <c r="M50" s="25" t="inlineStr">
-        <is>
-          <t>https://dasa.businessmap.io/ctrl_board/96/cards/451676/details</t>
-        </is>
-      </c>
-      <c r="N50" s="24" t="n">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="51" ht="52" customHeight="1">
-      <c r="A51" s="24" t="n">
-        <v>50</v>
-      </c>
-      <c r="B51" s="24" t="inlineStr">
-        <is>
-          <t>11. Fora da linha do tempo</t>
-        </is>
-      </c>
-      <c r="C51" s="24" t="inlineStr">
-        <is>
-          <t>Card da planilha</t>
-        </is>
-      </c>
-      <c r="D51" s="24" t="inlineStr">
-        <is>
-          <t>476063</t>
-        </is>
-      </c>
-      <c r="E51" s="24" t="inlineStr">
-        <is>
-          <t>[DATP] DasaLogs -&gt; api local - unidades</t>
-        </is>
-      </c>
-      <c r="F51" s="24" t="inlineStr">
-        <is>
-          <t>Stand By</t>
-        </is>
-      </c>
-      <c r="G51" s="24" t="n"/>
-      <c r="H51" s="24" t="n"/>
-      <c r="I51" s="24" t="n"/>
-      <c r="J51" s="24" t="n"/>
-      <c r="K51" s="24" t="inlineStr">
-        <is>
-          <t>Complexidade Stand By.</t>
-        </is>
-      </c>
-      <c r="L51" s="24" t="inlineStr">
-        <is>
-          <t>Fora da ordem.</t>
-        </is>
-      </c>
-      <c r="M51" s="25" t="inlineStr">
-        <is>
-          <t>https://dasa.businessmap.io/ctrl_board/96/cards/476063/details</t>
-        </is>
-      </c>
-      <c r="N51" s="24" t="n">
-        <v>33</v>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N51">
-    <sortState ref="A1:N51">
+  <autoFilter ref="A1:O45">
+    <sortState ref="A1:O45">
       <sortCondition descending="0" ref="A2:A200"/>
     </sortState>
   </autoFilter>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M9" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M10" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M11" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M12" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M13" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M14" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M15" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M16" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M17" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M18" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M19" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M22" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M25" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M26" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M27" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M28" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M29" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M30" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M33" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M34" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M35" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M36" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M37" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M38" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M39" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M40" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M41" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M45" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M46" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M47" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M48" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M49" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M50" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M51" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N22" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N25" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N26" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N27" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N28" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N29" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N30" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N34" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N35" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N36" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N37" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N38" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N39" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N40" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N41" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N42" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N43" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N44" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N45" r:id="rId37"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.6" bottom="0.6" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" scale="70" fitToHeight="0" fitToWidth="1"/>
@@ -3628,73 +3436,263 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="150" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="62" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="36" customWidth="1" min="8" max="8"/>
+    <col width="70" customWidth="1" min="9" max="9"/>
+    <col width="42" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="26" t="inlineStr">
-        <is>
-          <t>Como a aba foi ordenada</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="48" customHeight="1">
-      <c r="A3" s="27" t="inlineStr">
-        <is>
-          <t>A ordem segue dependência e arquitetura. A coluna Cronograma original guarda a data da planilha e não foi usada para ordenar. Várias datas se contradizem: portal e Blob em fevereiro de 2027, adequação do Airflow em março–abril de 2027, Airflow com nome prd em 09/10/26.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="48" customHeight="1">
-      <c r="A4" s="27" t="inlineStr">
-        <is>
-          <t>HML termina no teste funcional (card 451689) e no teste de carga, que não tem card. Produção começa depois. O único cluster concluído é o GKE de HML.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="48" customHeight="1">
-      <c r="A5" s="27" t="inlineStr">
-        <is>
-          <t>A passagem do Data Factory para o Airflow não entra nesta aba. Está concluída e é pré-requisito de outro projeto. O Airflow de partida está na Azure. Nesta lista a frente é migrar esse Airflow para a GCP: primeiro a spike, por causa da versão 2.2.5, depois a adequação. Carga, Blob e portal esperam essa migração. As APIs que não citam Airflow nem Cognitive Search não esperam.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="48" customHeight="1">
-      <c r="A6" s="27" t="inlineStr">
-        <is>
-          <t>Exam fica depois do índice. As outras APIs não foram colocadas atrás do índice: só a exam e o dp-backend-api cancelado citam Cognitive Search. O diagrama desenha busca-search na frente do conjunto de APIs, e essa diferença está na aba Dúvidas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="48" customHeight="1">
-      <c r="A7" s="27" t="inlineStr">
-        <is>
-          <t>Lacuna só entra quando a documentação nomeia o componente ou quando um card cita a dependência e não existe card para ela. Lacuna não tem Card ID, responsável, complexidade nem prazo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="48" customHeight="1">
-      <c r="A8" s="27" t="inlineStr">
-        <is>
-          <t>BigQuery no lugar do Databricks ficou fora do caminho. A decisão é levar o Databricks para a GCP, o diagrama AS IS não o coloca até a API, e a documentação não lista o que os workspaces executam.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="48" customHeight="1">
-      <c r="A9" s="27" t="inlineStr">
-        <is>
-          <t>Cancelado, Stand By e o SQL Server abortado ficam no fim, para a lista original continuar completa.</t>
-        </is>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Ordem</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Card ID</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Descrição</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Complexidade</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Depêndencia</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Cronograma original</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Recurso Responsável</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Observações</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Por que não entra neste caminho</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Card URL</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Linha na planilha original</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="60" customHeight="1">
+      <c r="A2" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="28" t="inlineStr">
+        <is>
+          <t>478328</t>
+        </is>
+      </c>
+      <c r="C2" s="28" t="inlineStr">
+        <is>
+          <t>BigQuery =&gt; substituir dataBricks</t>
+        </is>
+      </c>
+      <c r="D2" s="28" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="E2" s="28" t="inlineStr">
+        <is>
+          <t>Galerinha de dados DP</t>
+        </is>
+      </c>
+      <c r="F2" s="28" t="inlineStr">
+        <is>
+          <t>29/01/27</t>
+        </is>
+      </c>
+      <c r="G2" s="28" t="inlineStr">
+        <is>
+          <t>Dados</t>
+        </is>
+      </c>
+      <c r="H2" s="28" t="inlineStr">
+        <is>
+          <t>Levar toda a orquestração do dataBricks para o BigQuery</t>
+        </is>
+      </c>
+      <c r="I2" s="28" t="inlineStr">
+        <is>
+          <t>A equipe pediu levar a orquestração do Databricks para o BigQuery. O diagrama AS IS não passa pelo Databricks até as APIs. A ida para a GCP não exige essa troca: a decisão deste plano é levar os workspaces, e o card de converter os ETLs já está cancelado. O desenho com bronze, silver e gold está no documento sem a estratégia preenchida.</t>
+        </is>
+      </c>
+      <c r="J2" s="29" t="inlineStr">
+        <is>
+          <t>https://dasa.businessmap.io/ctrl_board/96/cards/478328/details</t>
+        </is>
+      </c>
+      <c r="K2" s="28" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" ht="60" customHeight="1">
+      <c r="A3" s="28" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="28" t="inlineStr">
+        <is>
+          <t>476063</t>
+        </is>
+      </c>
+      <c r="C3" s="28" t="inlineStr">
+        <is>
+          <t>[DATP] DasaLogs -&gt; api local - unidades</t>
+        </is>
+      </c>
+      <c r="D3" s="28" t="inlineStr">
+        <is>
+          <t>Stand By</t>
+        </is>
+      </c>
+      <c r="E3" s="28" t="n"/>
+      <c r="F3" s="28" t="n"/>
+      <c r="G3" s="28" t="n"/>
+      <c r="H3" s="28" t="n"/>
+      <c r="I3" s="28" t="inlineStr">
+        <is>
+          <t>A equipe deixou em stand-by. O documento de arquitetura não cita DasaLogs no caminho de exame, unidade e convênio, nem nas APIs, no Airflow ou na busca.</t>
+        </is>
+      </c>
+      <c r="J3" s="29" t="inlineStr">
+        <is>
+          <t>https://dasa.businessmap.io/ctrl_board/96/cards/476063/details</t>
+        </is>
+      </c>
+      <c r="K3" s="28" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="4" ht="60" customHeight="1">
+      <c r="A4" s="28" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="28" t="inlineStr">
+        <is>
+          <t>470121</t>
+        </is>
+      </c>
+      <c r="C4" s="28" t="inlineStr">
+        <is>
+          <t>Criação de Workloads do projeto BUSCA -&gt; dp-corporate-frontend</t>
+        </is>
+      </c>
+      <c r="D4" s="28" t="inlineStr">
+        <is>
+          <t>Cancelado</t>
+        </is>
+      </c>
+      <c r="E4" s="28" t="n"/>
+      <c r="F4" s="28" t="n"/>
+      <c r="G4" s="28" t="n"/>
+      <c r="H4" s="28" t="n"/>
+      <c r="I4" s="28" t="inlineStr">
+        <is>
+          <t>A equipe cancelou o workload dp-corporate-frontend. A documentação ainda aponta essa URL como frontend do DP. O card 469051 segue no caminho com outro nome. Os dois não foram tratados como o mesmo frontend.</t>
+        </is>
+      </c>
+      <c r="J4" s="29" t="inlineStr">
+        <is>
+          <t>https://dasa.businessmap.io/ctrl_board/96/cards/470121/details</t>
+        </is>
+      </c>
+      <c r="K4" s="28" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5" ht="60" customHeight="1">
+      <c r="A5" s="28" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="28" t="inlineStr">
+        <is>
+          <t>468985</t>
+        </is>
+      </c>
+      <c r="C5" s="28" t="inlineStr">
+        <is>
+          <t>Criação de Workloads do projeto PORTAL-CADASTRO -&gt; datp-backoffice-frontend-portal</t>
+        </is>
+      </c>
+      <c r="D5" s="28" t="inlineStr">
+        <is>
+          <t>Cancelado</t>
+        </is>
+      </c>
+      <c r="E5" s="28" t="n"/>
+      <c r="F5" s="28" t="n"/>
+      <c r="G5" s="28" t="n"/>
+      <c r="H5" s="28" t="inlineStr">
+        <is>
+          <t>depende do airFlow</t>
+        </is>
+      </c>
+      <c r="I5" s="28" t="inlineStr">
+        <is>
+          <t>A equipe cancelou o workload do repositório datp-backoffice-frontend-portal. A documentação cita esse repositório como frontend do portal de cadastro. Os cards 470165 e 451677 seguem no caminho com outros nomes.</t>
+        </is>
+      </c>
+      <c r="J5" s="29" t="inlineStr">
+        <is>
+          <t>https://dasa.businessmap.io/ctrl_board/96/cards/468985/details</t>
+        </is>
+      </c>
+      <c r="K5" s="28" t="n">
+        <v>20</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
+  <autoFilter ref="A1:K5">
+    <sortState ref="A1:K5">
+      <sortCondition descending="0" ref="A2:A200"/>
+    </sortState>
+  </autoFilter>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J5" r:id="rId4"/>
+  </hyperlinks>
+  <pageMargins left="0.4" right="0.4" top="0.6" bottom="0.6" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" scale="70" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
-    <oddHeader/>
+    <oddHeader>&amp;LDiscutir com a equipe</oddHeader>
     <oddFooter>&amp;RPágina &amp;P de &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -3710,6 +3708,95 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
+  <dimension ref="A1:A10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="150" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="30" t="inlineStr">
+        <is>
+          <t>Como a aba foi ordenada</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="48" customHeight="1">
+      <c r="A3" s="31" t="inlineStr">
+        <is>
+          <t>A ordem segue dependência e arquitetura. A coluna Cronograma original guarda a data da planilha e não foi usada para ordenar. Várias datas se contradizem: portal e Blob em fevereiro de 2027, adequação do Airflow em março–abril de 2027, Airflow com nome prd em 09/10/26.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="48" customHeight="1">
+      <c r="A4" s="31" t="inlineStr">
+        <is>
+          <t>O teste funcional (card 451689) e o teste de carga fecham o que a HML precisa para testar. A linha de Databricks na GCP fica depois desse teste e antes da produção, e não bloqueia o teste. O único cluster concluído é o GKE de HML.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="48" customHeight="1">
+      <c r="A5" s="31" t="inlineStr">
+        <is>
+          <t>A passagem do Data Factory para o Airflow não entra nesta aba. Está concluída e é pré-requisito de outro projeto. O Airflow de partida está na Azure. Nesta lista a frente é migrar esse Airflow para a GCP: primeiro a spike, por causa da versão 2.2.5, depois a adequação. Carga, Blob e portal esperam essa migração. As APIs que não citam Airflow nem Cognitive Search não esperam.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="48" customHeight="1">
+      <c r="A6" s="31" t="inlineStr">
+        <is>
+          <t>Exam fica depois do índice. As outras APIs não foram colocadas atrás do índice: só a exam e o dp-backend-api cancelado citam Cognitive Search. O diagrama desenha busca-search na frente do conjunto de APIs, e essa diferença está na aba Dúvidas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="48" customHeight="1">
+      <c r="A7" s="31" t="inlineStr">
+        <is>
+          <t>Lacuna só entra quando a documentação nomeia o componente ou quando um card cita a dependência e não existe card para ela. Lacuna não tem Card ID, responsável, complexidade nem prazo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="48" customHeight="1">
+      <c r="A8" s="31" t="inlineStr">
+        <is>
+          <t>A coluna Indicação fica vazia quando a atividade é da equipe e permanece no caminho. O texto 'Inclusa por IA — gap identificado' marca o que não tinha card: a documentação ou a dependência de um card mostrou a falta. Nada disso recebeu responsável, prazo ou Card ID.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="48" customHeight="1">
+      <c r="A9" s="31" t="inlineStr">
+        <is>
+          <t>O card de BigQuery no lugar do Databricks, o DasaLogs, o frontend dp-corporate-frontend e o repositório datp-backoffice-frontend-portal foram para a aba Discutir com a equipe. São itens da planilha que não se sustentam neste caminho.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="48" customHeight="1">
+      <c r="A10" s="31" t="inlineStr">
+        <is>
+          <t>Cards cancelados ou abortados que não entram nessa discussão ficam no fim, com Indicação 'Equipe — encerrada'.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;RPágina &amp;P de &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -3736,204 +3823,204 @@
       </c>
     </row>
     <row r="2" ht="48" customHeight="1">
-      <c r="A2" s="28" t="inlineStr">
+      <c r="A2" s="32" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B2" s="28" t="inlineStr">
+      <c r="B2" s="32" t="inlineStr">
         <is>
           <t>O banco criado no card 451661 já tem, em HML, exame, unidade e convênio?</t>
         </is>
       </c>
-      <c r="C2" s="28" t="inlineStr">
+      <c r="C2" s="32" t="inlineStr">
         <is>
           <t>Se já tiver, a lacuna de carga sai da frente do teste funcional. Se não tiver, ela continua depois da migração do Airflow da Azure para a GCP. A migração do SQL Server está abortada.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="48" customHeight="1">
-      <c r="A3" s="28" t="inlineStr">
+      <c r="A3" s="32" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B3" s="28" t="inlineStr">
+      <c r="B3" s="32" t="inlineStr">
         <is>
           <t>Quais APIs leem o Cognitive Search além da exam?</t>
         </is>
       </c>
-      <c r="C3" s="28" t="inlineStr">
+      <c r="C3" s="32" t="inlineStr">
         <is>
           <t>O diagrama coloca busca-search na frente das APIs. A planilha só trava a exam e o dp-backend-api cancelado. Se brand, local, health insurance, elegibility ou commons leem o índice, elas saem da etapa 3 e vão para depois do card 451682.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="48" customHeight="1">
-      <c r="A4" s="28" t="inlineStr">
+      <c r="A4" s="32" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="B4" s="28" t="inlineStr">
+      <c r="B4" s="32" t="inlineStr">
         <is>
           <t>O que o Databricks de HML entrega para a API ou para o portal?</t>
         </is>
       </c>
-      <c r="C4" s="28" t="inlineStr">
-        <is>
-          <t>A documentação só lista os workspaces. Sem jobs ou tabelas de saída, ele ficou fora da frente do teste. Se alguma carga do Corporate ou do cadastro sair de lá, ele entra antes do teste funcional.</t>
+      <c r="C4" s="32" t="inlineStr">
+        <is>
+          <t>A linha dos workspaces foi inclusa por gap e ficou depois do teste funcional, porque o diagrama até as APIs não passa pelo Databricks. Se a API ou o portal consomem a saída, ela sobe para antes do card 451689.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="48" customHeight="1">
-      <c r="A5" s="28" t="inlineStr">
+      <c r="A5" s="32" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="B5" s="28" t="inlineStr">
+      <c r="B5" s="32" t="inlineStr">
         <is>
           <t>datp-searcher-api-elegibility é a API de agendamento do documento?</t>
         </is>
       </c>
-      <c r="C5" s="28" t="inlineStr">
+      <c r="C5" s="32" t="inlineStr">
         <is>
           <t>O documento lista agendamento entre as seis APIs. O diagrama nomeia busca-agendamento-backend. A planilha tem elegibility e não tem card chamado agendamento. Se forem duas APIs, falta o workload de agendamento.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="48" customHeight="1">
-      <c r="A6" s="28" t="inlineStr">
+      <c r="A6" s="32" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="B6" s="28" t="inlineStr">
+      <c r="B6" s="32" t="inlineStr">
         <is>
           <t>O card cancelado dp-corporate-frontend (470121) é o mesmo frontend do card 469051?</t>
         </is>
       </c>
-      <c r="C6" s="28" t="inlineStr">
+      <c r="C6" s="32" t="inlineStr">
         <is>
           <t>A documentação cita a URL dp-corporate-frontend e o repositório datp-backoffice-frontend. Um card está cancelado e o outro está na fila de HML. Sem essa resposta os dois não foram unidos.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="48" customHeight="1">
-      <c r="A7" s="28" t="inlineStr">
+      <c r="A7" s="32" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="B7" s="28" t="inlineStr">
+      <c r="B7" s="32" t="inlineStr">
         <is>
           <t>O download D+1 de cadastro lê o Blob?</t>
         </is>
       </c>
-      <c r="C7" s="28" t="inlineStr">
+      <c r="C7" s="32" t="inlineStr">
         <is>
           <t>O Blob depende de Airflow, backend e frontend. O portal depende de Airflow, cargas de cadastro e D+1. A planilha não liga um ao outro. Se o D+1 ler o Blob, o card 451688 fica antes das cargas.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="48" customHeight="1">
-      <c r="A8" s="28" t="inlineStr">
+      <c r="A8" s="32" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="B8" s="28" t="inlineStr">
+      <c r="B8" s="32" t="inlineStr">
         <is>
           <t>A conectividade do card 424949 inclui as fontes do diagrama?</t>
         </is>
       </c>
-      <c r="C8" s="28" t="inlineStr">
+      <c r="C8" s="32" t="inlineStr">
         <is>
           <t>K2/Gliese, base federada, MDM, GSC, hospitais e MV estão no desenho. A seção de rede do documento está vazia. O texto dos workloads fala só do IP da aplicação. Se as fontes forem outro trabalho, falta uma atividade antes da carga.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="48" customHeight="1">
-      <c r="A9" s="28" t="inlineStr">
+      <c r="A9" s="32" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="B9" s="28" t="inlineStr">
+      <c r="B9" s="32" t="inlineStr">
         <is>
           <t>No teste de HML a autenticação continua como está?</t>
         </is>
       </c>
-      <c r="C9" s="28" t="inlineStr">
+      <c r="C9" s="32" t="inlineStr">
         <is>
           <t>O documento marca Azure AD como dependência interna que não pode ser desacoplada. Frontend do DP usa AD, portal usa SSO, APIs usam API key. O template GCP escreve Azure AD para Google IAM e não foi preenchido. Nenhuma atividade de identidade foi criada.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="48" customHeight="1">
-      <c r="A10" s="28" t="inlineStr">
+      <c r="A10" s="32" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="B10" s="28" t="inlineStr">
+      <c r="B10" s="32" t="inlineStr">
         <is>
           <t>O que entra no teste de carga?</t>
         </is>
       </c>
-      <c r="C10" s="28" t="inlineStr">
+      <c r="C10" s="32" t="inlineStr">
         <is>
           <t>Não há card, volume, API nem meta. O template do documento cita Performance sem conteúdo. A linha está depois do teste funcional e antes da produção, sem cenário.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="48" customHeight="1">
-      <c r="A11" s="28" t="inlineStr">
+      <c r="A11" s="32" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="B11" s="28" t="inlineStr">
+      <c r="B11" s="32" t="inlineStr">
         <is>
           <t>dp-api-gtw e dp-cad-proxy entram nesta migração?</t>
         </is>
       </c>
-      <c r="C11" s="28" t="inlineStr">
+      <c r="C11" s="32" t="inlineStr">
         <is>
           <t>Estão no diagrama AS IS e não têm card. Ficaram fora do caminho. O Zuul tem card próprio.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="48" customHeight="1">
-      <c r="A12" s="28" t="inlineStr">
+      <c r="A12" s="32" t="inlineStr">
         <is>
           <t>11</t>
         </is>
       </c>
-      <c r="B12" s="28" t="inlineStr">
+      <c r="B12" s="32" t="inlineStr">
         <is>
           <t>O staging SQL ainda faz parte do caminho em HML?</t>
         </is>
       </c>
-      <c r="C12" s="28" t="inlineStr">
+      <c r="C12" s="32" t="inlineStr">
         <is>
           <t>STAGING_PRD está na documentação e não há card. Ficou fora do caminho.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="48" customHeight="1">
-      <c r="A13" s="28" t="inlineStr">
+      <c r="A13" s="32" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="B13" s="28" t="inlineStr">
+      <c r="B13" s="32" t="inlineStr">
         <is>
           <t>Event Hub entra no teste funcional de algum canal?</t>
         </is>
       </c>
-      <c r="C13" s="28" t="inlineStr">
+      <c r="C13" s="32" t="inlineStr">
         <is>
           <t>O card manda deixar por último e nenhuma API o cita. Ele está no fim da produção. Se NAV ou CDC dependem do evento para o teste de HML, ele sobe para antes do card 451689.</t>
         </is>

</xml_diff>

<commit_message>
Separa status de complexidade e reorganiza as colunas.
A coluna original misturava Alta, Média e Baixa com Concluído, Cancelado, Stand By e sem escopo. A descrição fica ao lado da etapa, a origem marca lacuna com - IA, e o motivo da posição fica ao lado das observações.

Co-authored-by: waneron <waneron@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/BM-GCP-Atividades-DP-ordem-temporal.xlsx
+++ b/BM-GCP-Atividades-DP-ordem-temporal.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'BM - GCP Atividades - DP'!$A$1:$O$45</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'BM - GCP Atividades - DP'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Discutir com a equipe'!$A$1:$K$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Discutir com a equipe'!$A$1:$L$5</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Discutir com a equipe'!$1:$1</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Regra de ordem'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Dúvidas'!$A$1:$C$13</definedName>
@@ -640,11 +640,11 @@
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="46" customWidth="1" min="2" max="2"/>
-    <col width="38" customWidth="1" min="3" max="3"/>
-    <col width="36" customWidth="1" min="4" max="4"/>
+    <col width="62" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="62" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
     <col width="46" customWidth="1" min="8" max="8"/>
     <col width="28" customWidth="1" min="9" max="9"/>
     <col width="26" customWidth="1" min="10" max="10"/>
@@ -668,7 +668,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Indicação</t>
+          <t>Descrição</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -683,7 +683,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Descrição</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -713,12 +713,12 @@
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
+          <t>Por que nesta posição</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
           <t>Base na planilha ou na documentação</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Por que nesta posição</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
@@ -741,7 +741,11 @@
           <t>1. HML — base já concluída</t>
         </is>
       </c>
-      <c r="C2" s="2" t="n"/>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>[DP] Provisionar ambiente GKE HML</t>
+        </is>
+      </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
           <t>Card da planilha</t>
@@ -754,26 +758,22 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>[DP] Provisionar ambiente GKE HML</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
           <t>Concluído</t>
         </is>
       </c>
+      <c r="G2" s="2" t="n"/>
       <c r="H2" s="2" t="n"/>
       <c r="I2" s="2" t="n"/>
       <c r="J2" s="2" t="n"/>
       <c r="K2" s="2" t="n"/>
       <c r="L2" s="2" t="inlineStr">
         <is>
+          <t>Ponto de partida. O pedido é sair da homologação.</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
           <t>Status Concluído. Único card de ambiente, nome HML. A documentação cita o cluster Azure de homologação azr-hml02, namespaces busca, dataprovider-data e portal-cadastro.</t>
-        </is>
-      </c>
-      <c r="M2" s="2" t="inlineStr">
-        <is>
-          <t>Ponto de partida. O pedido é sair da homologação.</t>
         </is>
       </c>
       <c r="N2" s="3" t="inlineStr">
@@ -794,7 +794,11 @@
           <t>1. HML — base já concluída</t>
         </is>
       </c>
-      <c r="C3" s="2" t="n"/>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>[DP] Migração GCP | Criar banco de dados</t>
+        </is>
+      </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
           <t>Card da planilha</t>
@@ -807,26 +811,22 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>[DP] Migração GCP | Criar banco de dados</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
           <t>Concluído</t>
         </is>
       </c>
+      <c r="G3" s="2" t="n"/>
       <c r="H3" s="2" t="n"/>
       <c r="I3" s="2" t="n"/>
       <c r="J3" s="2" t="n"/>
       <c r="K3" s="2" t="n"/>
       <c r="L3" s="2" t="inlineStr">
         <is>
+          <t>O banco existe. A carga desse banco não tem card e entra mais adiante, antes do teste funcional.</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
           <t>Status Concluído. O card de migrar o SQL Server está abortado. A documentação descreve o Corporate (HML, master, réplica e staging) como o banco que serve as APIs.</t>
-        </is>
-      </c>
-      <c r="M3" s="2" t="inlineStr">
-        <is>
-          <t>O banco existe. A carga desse banco não tem card e entra mais adiante, antes do teste funcional.</t>
         </is>
       </c>
       <c r="N3" s="3" t="inlineStr">
@@ -847,7 +847,11 @@
           <t>1. HML — base já concluída</t>
         </is>
       </c>
-      <c r="C4" s="2" t="n"/>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>[DP] Migração GCP | Redis</t>
+        </is>
+      </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
           <t>Card da planilha</t>
@@ -860,14 +864,10 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>[DP] Migração GCP | Redis</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
           <t>Concluído</t>
         </is>
       </c>
+      <c r="G4" s="2" t="n"/>
       <c r="H4" s="2" t="inlineStr">
         <is>
           <t>Os pods precisam estar de pé para testar</t>
@@ -882,12 +882,12 @@
       <c r="K4" s="2" t="n"/>
       <c r="L4" s="2" t="inlineStr">
         <is>
+          <t>Concluído. O teste que a dependência pede espera os pods das APIs.</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
           <t>Status Concluído. No diagrama, busca-cache fica entre o Corporate e as APIs. A documentação lista dois Redis de 6 GB: DP Cache PRD e Busca. A planilha não separa HML e PRD.</t>
-        </is>
-      </c>
-      <c r="M4" s="2" t="inlineStr">
-        <is>
-          <t>Concluído. O teste que a dependência pede espera os pods das APIs.</t>
         </is>
       </c>
       <c r="N4" s="3" t="inlineStr">
@@ -908,7 +908,11 @@
           <t>1. HML — base já concluída</t>
         </is>
       </c>
-      <c r="C5" s="2" t="n"/>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Continuação - Criação de Workloads do projeto BUSCA -&gt; datp-searcher-api-commons</t>
+        </is>
+      </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
           <t>Card da planilha</t>
@@ -921,26 +925,22 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Continuação - Criação de Workloads do projeto BUSCA -&gt; datp-searcher-api-commons</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
           <t>Concluído</t>
         </is>
       </c>
+      <c r="G5" s="2" t="n"/>
       <c r="H5" s="2" t="n"/>
       <c r="I5" s="2" t="n"/>
       <c r="J5" s="2" t="n"/>
       <c r="K5" s="2" t="n"/>
       <c r="L5" s="2" t="inlineStr">
         <is>
+          <t>Concluído. O 470112 permanece na fila das APIs.</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
           <t>Status Concluído. O card 470112, da criação do mesmo workload, segue com observação 'atuando'.</t>
-        </is>
-      </c>
-      <c r="M5" s="2" t="inlineStr">
-        <is>
-          <t>Concluído. O 470112 permanece na fila das APIs.</t>
         </is>
       </c>
       <c r="N5" s="3" t="inlineStr">
@@ -961,7 +961,11 @@
           <t>2. HML — antes de subir workload</t>
         </is>
       </c>
-      <c r="C6" s="4" t="n"/>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>[DP] Definir conectividade</t>
+        </is>
+      </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
           <t>Card da planilha</t>
@@ -972,11 +976,7 @@
           <t>424949</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>[DP] Definir conectividade</t>
-        </is>
-      </c>
+      <c r="F6" s="4" t="n"/>
       <c r="G6" s="4" t="n"/>
       <c r="H6" s="4" t="n"/>
       <c r="I6" s="4" t="n"/>
@@ -984,12 +984,12 @@
       <c r="K6" s="4" t="n"/>
       <c r="L6" s="4" t="inlineStr">
         <is>
+          <t>Antes dos workloads. Sem isso a aplicação sobe apontando para IP, que a própria planilha registra como errado.</t>
+        </is>
+      </c>
+      <c r="M6" s="4" t="inlineStr">
+        <is>
           <t>Único card de conectividade. Os workloads de busca registram que a conectividade por IP está errada. A seção de rede do documento (VNet, subnet, VPN, DNS, firewall) está vazia. O diagrama mostra as fontes K2/Gliese, base federada, MDM, GSC, hospitais e MV.</t>
-        </is>
-      </c>
-      <c r="M6" s="4" t="inlineStr">
-        <is>
-          <t>Antes dos workloads. Sem isso a aplicação sobe apontando para IP, que a própria planilha registra como errado.</t>
         </is>
       </c>
       <c r="N6" s="5" t="inlineStr">
@@ -1010,7 +1010,11 @@
           <t>2. HML — antes de subir workload</t>
         </is>
       </c>
-      <c r="C7" s="4" t="n"/>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>[DP] Adequação de pipelines CI/CD</t>
+        </is>
+      </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
           <t>Card da planilha</t>
@@ -1021,11 +1025,7 @@
           <t>424942</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr">
-        <is>
-          <t>[DP] Adequação de pipelines CI/CD</t>
-        </is>
-      </c>
+      <c r="F7" s="4" t="n"/>
       <c r="G7" s="4" t="inlineStr">
         <is>
           <t>Alta</t>
@@ -1049,12 +1049,12 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
+          <t>Em paralelo com a conectividade. A planilha não diz que este card bloqueia a criação do workload.</t>
+        </is>
+      </c>
+      <c r="M7" s="4" t="inlineStr">
+        <is>
           <t>Card de esteira, sem data. Nenhum workload cita este número como dependência.</t>
-        </is>
-      </c>
-      <c r="M7" s="4" t="inlineStr">
-        <is>
-          <t>Em paralelo com a conectividade. A planilha não diz que este card bloqueia a criação do workload.</t>
         </is>
       </c>
       <c r="N7" s="5" t="inlineStr">
@@ -1075,7 +1075,11 @@
           <t>3. HML — APIs e gateway, em paralelo com o Airflow</t>
         </is>
       </c>
-      <c r="C8" s="6" t="n"/>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>Criação de Workloads do projeto BUSCA -&gt; datp-searcher-api-brand</t>
+        </is>
+      </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
           <t>Card da planilha</t>
@@ -1086,11 +1090,7 @@
           <t>470110</t>
         </is>
       </c>
-      <c r="F8" s="6" t="inlineStr">
-        <is>
-          <t>Criação de Workloads do projeto BUSCA -&gt; datp-searcher-api-brand</t>
-        </is>
-      </c>
+      <c r="F8" s="6" t="n"/>
       <c r="G8" s="6" t="inlineStr">
         <is>
           <t>Baixa</t>
@@ -1114,12 +1114,12 @@
       <c r="K8" s="6" t="n"/>
       <c r="L8" s="6" t="inlineStr">
         <is>
+          <t>Depois da conectividade. Não espera o Airflow. A data 20/10/26 foi ignorada na ordenação.</t>
+        </is>
+      </c>
+      <c r="M8" s="6" t="inlineStr">
+        <is>
           <t>Uma das seis APIs do documento: exam, healthinsurance, commons, agendamento, local e brand. Este card não cita Airflow nem Cognitive Search.</t>
-        </is>
-      </c>
-      <c r="M8" s="6" t="inlineStr">
-        <is>
-          <t>Depois da conectividade. Não espera o Airflow. A data 20/10/26 foi ignorada na ordenação.</t>
         </is>
       </c>
       <c r="N8" s="7" t="inlineStr">
@@ -1140,7 +1140,11 @@
           <t>3. HML — APIs e gateway, em paralelo com o Airflow</t>
         </is>
       </c>
-      <c r="C9" s="6" t="n"/>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>Criação de Workloads do projeto BUSCA -&gt; datp-infra-gateway -&gt; (ZUUL)</t>
+        </is>
+      </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
           <t>Card da planilha</t>
@@ -1151,11 +1155,7 @@
           <t>470109</t>
         </is>
       </c>
-      <c r="F9" s="6" t="inlineStr">
-        <is>
-          <t>Criação de Workloads do projeto BUSCA -&gt; datp-infra-gateway -&gt; (ZUUL)</t>
-        </is>
-      </c>
+      <c r="F9" s="6" t="n"/>
       <c r="G9" s="6" t="inlineStr">
         <is>
           <t>Média</t>
@@ -1179,12 +1179,12 @@
       <c r="K9" s="6" t="n"/>
       <c r="L9" s="6" t="inlineStr">
         <is>
+          <t>Junto das APIs, depois da conectividade. A documentação não separa o gateway da entrada das APIs.</t>
+        </is>
+      </c>
+      <c r="M9" s="6" t="inlineStr">
+        <is>
           <t>No diagrama o gateway aparece como dp-zuul-proxy, ao lado de autorização, rate limit e WAF. Não há card separado para WAF, rate limit ou API key.</t>
-        </is>
-      </c>
-      <c r="M9" s="6" t="inlineStr">
-        <is>
-          <t>Junto das APIs, depois da conectividade. A documentação não separa o gateway da entrada das APIs.</t>
         </is>
       </c>
       <c r="N9" s="7" t="inlineStr">
@@ -1205,7 +1205,11 @@
           <t>3. HML — APIs e gateway, em paralelo com o Airflow</t>
         </is>
       </c>
-      <c r="C10" s="6" t="n"/>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>Criação de Workloads do projeto BUSCA -&gt; datp-searcher-api-local</t>
+        </is>
+      </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
           <t>Card da planilha</t>
@@ -1216,11 +1220,7 @@
           <t>470118</t>
         </is>
       </c>
-      <c r="F10" s="6" t="inlineStr">
-        <is>
-          <t>Criação de Workloads do projeto BUSCA -&gt; datp-searcher-api-local</t>
-        </is>
-      </c>
+      <c r="F10" s="6" t="n"/>
       <c r="G10" s="6" t="inlineStr">
         <is>
           <t>Média</t>
@@ -1244,12 +1244,12 @@
       <c r="K10" s="6" t="n"/>
       <c r="L10" s="6" t="inlineStr">
         <is>
+          <t>Depois da conectividade. Data da planilha ignorada na ordenação.</t>
+        </is>
+      </c>
+      <c r="M10" s="6" t="inlineStr">
+        <is>
           <t>API local do documento. Não cita Airflow nem Cognitive Search.</t>
-        </is>
-      </c>
-      <c r="M10" s="6" t="inlineStr">
-        <is>
-          <t>Depois da conectividade. Data da planilha ignorada na ordenação.</t>
         </is>
       </c>
       <c r="N10" s="7" t="inlineStr">
@@ -1270,7 +1270,11 @@
           <t>3. HML — APIs e gateway, em paralelo com o Airflow</t>
         </is>
       </c>
-      <c r="C11" s="6" t="n"/>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>Criação de Workloads do projeto BUSCA -&gt; datp-searcher-api-healthinsurance</t>
+        </is>
+      </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
           <t>Card da planilha</t>
@@ -1281,11 +1285,7 @@
           <t>470115</t>
         </is>
       </c>
-      <c r="F11" s="6" t="inlineStr">
-        <is>
-          <t>Criação de Workloads do projeto BUSCA -&gt; datp-searcher-api-healthinsurance</t>
-        </is>
-      </c>
+      <c r="F11" s="6" t="n"/>
       <c r="G11" s="6" t="inlineStr">
         <is>
           <t>Alta</t>
@@ -1309,12 +1309,12 @@
       <c r="K11" s="6" t="n"/>
       <c r="L11" s="6" t="inlineStr">
         <is>
+          <t>Depois da conectividade. Data da planilha ignorada na ordenação.</t>
+        </is>
+      </c>
+      <c r="M11" s="6" t="inlineStr">
+        <is>
           <t>API de convênio do documento. Não cita Airflow nem Cognitive Search.</t>
-        </is>
-      </c>
-      <c r="M11" s="6" t="inlineStr">
-        <is>
-          <t>Depois da conectividade. Data da planilha ignorada na ordenação.</t>
         </is>
       </c>
       <c r="N11" s="7" t="inlineStr">
@@ -1335,7 +1335,11 @@
           <t>3. HML — APIs e gateway, em paralelo com o Airflow</t>
         </is>
       </c>
-      <c r="C12" s="6" t="n"/>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>Criação de Workloads do projeto BUSCA -&gt; datp-searcher-api-elegibility</t>
+        </is>
+      </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
           <t>Card da planilha</t>
@@ -1346,11 +1350,7 @@
           <t>470113</t>
         </is>
       </c>
-      <c r="F12" s="6" t="inlineStr">
-        <is>
-          <t>Criação de Workloads do projeto BUSCA -&gt; datp-searcher-api-elegibility</t>
-        </is>
-      </c>
+      <c r="F12" s="6" t="n"/>
       <c r="G12" s="6" t="inlineStr">
         <is>
           <t>Alta</t>
@@ -1374,12 +1374,12 @@
       <c r="K12" s="6" t="n"/>
       <c r="L12" s="6" t="inlineStr">
         <is>
+          <t>Permanece nesta fila porque o card não cita Airflow nem Cognitive Search. Não foi tratado como a API de agendamento.</t>
+        </is>
+      </c>
+      <c r="M12" s="6" t="inlineStr">
+        <is>
           <t>O documento e o diagrama nomeiam busca-agendamento. A planilha nomeia elegibility. Não há outro card com o nome agendamento.</t>
-        </is>
-      </c>
-      <c r="M12" s="6" t="inlineStr">
-        <is>
-          <t>Permanece nesta fila porque o card não cita Airflow nem Cognitive Search. Não foi tratado como a API de agendamento.</t>
         </is>
       </c>
       <c r="N12" s="7" t="inlineStr">
@@ -1400,7 +1400,11 @@
           <t>3. HML — APIs e gateway, em paralelo com o Airflow</t>
         </is>
       </c>
-      <c r="C13" s="6" t="n"/>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>Criação de Workloads do projeto BUSCA -&gt; datp-searcher-api-commons</t>
+        </is>
+      </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
           <t>Card da planilha</t>
@@ -1411,11 +1415,7 @@
           <t>470112</t>
         </is>
       </c>
-      <c r="F13" s="6" t="inlineStr">
-        <is>
-          <t>Criação de Workloads do projeto BUSCA -&gt; datp-searcher-api-commons</t>
-        </is>
-      </c>
+      <c r="F13" s="6" t="n"/>
       <c r="G13" s="6" t="inlineStr">
         <is>
           <t>Baixa</t>
@@ -1439,12 +1439,12 @@
       </c>
       <c r="L13" s="6" t="inlineStr">
         <is>
+          <t>Na mesma fila das outras APIs de busca que não citam índice.</t>
+        </is>
+      </c>
+      <c r="M13" s="6" t="inlineStr">
+        <is>
           <t>API commons do documento. A continuação 476416 está concluída. Este card segue 'atuando'.</t>
-        </is>
-      </c>
-      <c r="M13" s="6" t="inlineStr">
-        <is>
-          <t>Na mesma fila das outras APIs de busca que não citam índice.</t>
         </is>
       </c>
       <c r="N13" s="7" t="inlineStr">
@@ -1465,7 +1465,11 @@
           <t>3. HML — APIs e gateway, em paralelo com o Airflow</t>
         </is>
       </c>
-      <c r="C14" s="6" t="n"/>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>[DP] Migração de aplicações, APIs</t>
+        </is>
+      </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
           <t>Card da planilha</t>
@@ -1476,11 +1480,7 @@
           <t>424944</t>
         </is>
       </c>
-      <c r="F14" s="6" t="inlineStr">
-        <is>
-          <t>[DP] Migração de aplicações, APIs</t>
-        </is>
-      </c>
+      <c r="F14" s="6" t="n"/>
       <c r="G14" s="6" t="inlineStr">
         <is>
           <t>Baixa</t>
@@ -1504,12 +1504,12 @@
       <c r="K14" s="6" t="n"/>
       <c r="L14" s="6" t="inlineStr">
         <is>
+          <t>Logo depois dos workloads desta fila. Confirma que a aplicação enxerga o destino. O teste funcional espera dado, índice e portal.</t>
+        </is>
+      </c>
+      <c r="M14" s="6" t="inlineStr">
+        <is>
           <t>A dependência é testar conectividade, não teste funcional.</t>
-        </is>
-      </c>
-      <c r="M14" s="6" t="inlineStr">
-        <is>
-          <t>Logo depois dos workloads desta fila. Confirma que a aplicação enxerga o destino. O teste funcional espera dado, índice e portal.</t>
         </is>
       </c>
       <c r="N14" s="7" t="inlineStr">
@@ -1530,7 +1530,11 @@
           <t>3. HML — front e back do DP, em paralelo com o Airflow</t>
         </is>
       </c>
-      <c r="C15" s="6" t="n"/>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>[DP] Migração GCP | Migrar Backend -&gt; front do DP (adaptações)</t>
+        </is>
+      </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
           <t>Card da planilha</t>
@@ -1541,11 +1545,7 @@
           <t>469049</t>
         </is>
       </c>
-      <c r="F15" s="6" t="inlineStr">
-        <is>
-          <t>[DP] Migração GCP | Migrar Backend -&gt; front do DP (adaptações)</t>
-        </is>
-      </c>
+      <c r="F15" s="6" t="n"/>
       <c r="G15" s="6" t="inlineStr">
         <is>
           <t>Alta</t>
@@ -1565,12 +1565,12 @@
       <c r="K15" s="6" t="n"/>
       <c r="L15" s="6" t="inlineStr">
         <is>
+          <t>Sobe com as APIs. Não espera carga nem índice. O teste do frontend espera a integração.</t>
+        </is>
+      </c>
+      <c r="M15" s="6" t="inlineStr">
+        <is>
           <t>A documentação aponta o repositório datp-backoffice-backend. O card não cita Airflow. O diagrama tem dp-backoffice-api-prd.</t>
-        </is>
-      </c>
-      <c r="M15" s="6" t="inlineStr">
-        <is>
-          <t>Sobe com as APIs. Não espera carga nem índice. O teste do frontend espera a integração.</t>
         </is>
       </c>
       <c r="N15" s="7" t="inlineStr">
@@ -1591,7 +1591,11 @@
           <t>3. HML — front e back do DP, em paralelo com o Airflow</t>
         </is>
       </c>
-      <c r="C16" s="6" t="n"/>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>[DP] Migração GCP | Migrar Frontend  portal do DP (adaptações)</t>
+        </is>
+      </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
           <t>Card da planilha</t>
@@ -1602,11 +1606,7 @@
           <t>469051</t>
         </is>
       </c>
-      <c r="F16" s="6" t="inlineStr">
-        <is>
-          <t>[DP] Migração GCP | Migrar Frontend  portal do DP (adaptações)</t>
-        </is>
-      </c>
+      <c r="F16" s="6" t="n"/>
       <c r="G16" s="6" t="inlineStr">
         <is>
           <t>Média</t>
@@ -1630,12 +1630,12 @@
       </c>
       <c r="L16" s="6" t="inlineStr">
         <is>
+          <t>A adaptação entra aqui. O teste do front fica no fim da HML, com o 451689.</t>
+        </is>
+      </c>
+      <c r="M16" s="6" t="inlineStr">
+        <is>
           <t>A documentação cita o frontend em dp-corporate-frontend e o repositório datp-backoffice-frontend. O card 470121, dp-corporate-frontend, está cancelado. A observação deste card fala do teste, que é o 451689.</t>
-        </is>
-      </c>
-      <c r="M16" s="6" t="inlineStr">
-        <is>
-          <t>A adaptação entra aqui. O teste do front fica no fim da HML, com o 451689.</t>
         </is>
       </c>
       <c r="N16" s="7" t="inlineStr">
@@ -1656,7 +1656,11 @@
           <t>4. HML — índice e exam, em paralelo com o Airflow</t>
         </is>
       </c>
-      <c r="C17" s="8" t="n"/>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>[DP] Migração GCP | Index (cognitive search &gt; vertex - adaptar na aplicação)</t>
+        </is>
+      </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
           <t>Card da planilha</t>
@@ -1667,11 +1671,7 @@
           <t>451682</t>
         </is>
       </c>
-      <c r="F17" s="8" t="inlineStr">
-        <is>
-          <t>[DP] Migração GCP | Index (cognitive search &gt; vertex - adaptar na aplicação)</t>
-        </is>
-      </c>
+      <c r="F17" s="8" t="n"/>
       <c r="G17" s="8" t="inlineStr">
         <is>
           <t>Alta</t>
@@ -1691,12 +1691,12 @@
       <c r="K17" s="8" t="n"/>
       <c r="L17" s="8" t="inlineStr">
         <is>
+          <t>Antes da API de exam. As outras APIs não foram colocadas atrás deste card: a planilha não diz que elas leem o índice.</t>
+        </is>
+      </c>
+      <c r="M17" s="8" t="inlineStr">
+        <is>
           <t>No diagrama, busca-search fica entre o Corporate e as APIs. No documento, Cognitive Search é dependência externa, criticidade alta, e 'pode desacoplar' está TBD. O card aponta Vertex e está em descoberta. A planilha só declara a dependência na API de exam e no dp-backend-api cancelado.</t>
-        </is>
-      </c>
-      <c r="M17" s="8" t="inlineStr">
-        <is>
-          <t>Antes da API de exam. As outras APIs não foram colocadas atrás deste card: a planilha não diz que elas leem o índice.</t>
         </is>
       </c>
       <c r="N17" s="9" t="inlineStr">
@@ -1717,7 +1717,11 @@
           <t>4. HML — índice e exam, em paralelo com o Airflow</t>
         </is>
       </c>
-      <c r="C18" s="8" t="n"/>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>Criação de Workloads do projeto BUSCA -&gt; datp-searcher-api-exam</t>
+        </is>
+      </c>
       <c r="D18" s="8" t="inlineStr">
         <is>
           <t>Card da planilha</t>
@@ -1728,11 +1732,7 @@
           <t>470114</t>
         </is>
       </c>
-      <c r="F18" s="8" t="inlineStr">
-        <is>
-          <t>Criação de Workloads do projeto BUSCA -&gt; datp-searcher-api-exam</t>
-        </is>
-      </c>
+      <c r="F18" s="8" t="n"/>
       <c r="G18" s="8" t="inlineStr">
         <is>
           <t>Alta</t>
@@ -1756,12 +1756,12 @@
       </c>
       <c r="L18" s="8" t="inlineStr">
         <is>
+          <t>Depois do 451682 e depois da conectividade.</t>
+        </is>
+      </c>
+      <c r="M18" s="8" t="inlineStr">
+        <is>
           <t>API de exam do documento. Observação: depende de Cognitive Search. Também registra conectividade por IP errada.</t>
-        </is>
-      </c>
-      <c r="M18" s="8" t="inlineStr">
-        <is>
-          <t>Depois do 451682 e depois da conectividade.</t>
         </is>
       </c>
       <c r="N18" s="9" t="inlineStr">
@@ -1782,7 +1782,11 @@
           <t>5. HML — migrar o Airflow da Azure para a GCP</t>
         </is>
       </c>
-      <c r="C19" s="10" t="n"/>
+      <c r="C19" s="10" t="inlineStr">
+        <is>
+          <t>Spike -&gt; Airflow na versao mais nova do airflow</t>
+        </is>
+      </c>
       <c r="D19" s="10" t="inlineStr">
         <is>
           <t>Card da planilha</t>
@@ -1793,11 +1797,7 @@
           <t>478326</t>
         </is>
       </c>
-      <c r="F19" s="10" t="inlineStr">
-        <is>
-          <t>Spike -&gt; Airflow na versao mais nova do airflow</t>
-        </is>
-      </c>
+      <c r="F19" s="10" t="n"/>
       <c r="G19" s="10" t="inlineStr">
         <is>
           <t>Alta</t>
@@ -1825,12 +1825,12 @@
       </c>
       <c r="L19" s="10" t="inlineStr">
         <is>
+          <t>Primeira linha desta frente, em paralelo com as APIs da etapa 3. A spike existe por causa da versão, antes de migrar o Airflow da Azure para a GCP. Carga, Blob e portal esperam essa migração. A data 20/10/26 não posiciona o resto.</t>
+        </is>
+      </c>
+      <c r="M19" s="10" t="inlineStr">
+        <is>
           <t>O Airflow de partida já está na Azure. A dependência deste card é docker local. A documentação registra a versão 2.2.5 como baixa demais para a versão do Google.</t>
-        </is>
-      </c>
-      <c r="M19" s="10" t="inlineStr">
-        <is>
-          <t>Primeira linha desta frente, em paralelo com as APIs da etapa 3. A spike existe por causa da versão, antes de migrar o Airflow da Azure para a GCP. Carga, Blob e portal esperam essa migração. A data 20/10/26 não posiciona o resto.</t>
         </is>
       </c>
       <c r="N19" s="11" t="inlineStr">
@@ -1851,18 +1851,18 @@
           <t>5. HML — migrar o Airflow da Azure para a GCP</t>
         </is>
       </c>
-      <c r="C20" s="10" t="n"/>
+      <c r="C20" s="10" t="inlineStr">
+        <is>
+          <t>Criar historia adequação airflow, vinculada ao fim da poc do Victor =&gt; necessario devido versao de airflow</t>
+        </is>
+      </c>
       <c r="D20" s="10" t="inlineStr">
         <is>
           <t>Card da planilha</t>
         </is>
       </c>
       <c r="E20" s="10" t="n"/>
-      <c r="F20" s="10" t="inlineStr">
-        <is>
-          <t>Criar historia adequação airflow, vinculada ao fim da poc do Victor =&gt; necessario devido versao de airflow</t>
-        </is>
-      </c>
+      <c r="F20" s="10" t="n"/>
       <c r="G20" s="10" t="inlineStr">
         <is>
           <t>Alta</t>
@@ -1882,12 +1882,12 @@
       <c r="K20" s="10" t="n"/>
       <c r="L20" s="10" t="inlineStr">
         <is>
+          <t>Depois da spike. A janela de março–abril de 2027 fica registrada e não empurra esta linha para o fim. Blob e portal ficam depois porque dependem do Airflow já na GCP.</t>
+        </is>
+      </c>
+      <c r="M20" s="10" t="inlineStr">
+        <is>
           <t>Linha da planilha, sem Card ID. É a migração do Airflow que já roda na Azure para a GCP. A adequação existe por causa da versão. Portal, Blob e backoffice citam Airflow como dependência. Os workloads com prd no nome ficam na produção.</t>
-        </is>
-      </c>
-      <c r="M20" s="10" t="inlineStr">
-        <is>
-          <t>Depois da spike. A janela de março–abril de 2027 fica registrada e não empurra esta linha para o fim. Blob e portal ficam depois porque dependem do Airflow já na GCP.</t>
         </is>
       </c>
       <c r="N20" s="10" t="n"/>
@@ -1904,22 +1904,18 @@
           <t>6. HML — dado, depois do Airflow e do backend</t>
         </is>
       </c>
-      <c r="C21" s="13" t="inlineStr">
-        <is>
-          <t>Inclusa por IA — gap identificado</t>
-        </is>
-      </c>
-      <c r="D21" s="12" t="inlineStr">
-        <is>
-          <t>Lacuna — documentação</t>
+      <c r="C21" s="12" t="inlineStr">
+        <is>
+          <t>Carga, no banco de HML, dos dados de exame, unidade e convênio que hoje estão no Corporate</t>
+        </is>
+      </c>
+      <c r="D21" s="13" t="inlineStr">
+        <is>
+          <t>Lacuna — documentação - IA</t>
         </is>
       </c>
       <c r="E21" s="12" t="n"/>
-      <c r="F21" s="12" t="inlineStr">
-        <is>
-          <t>Carga, no banco de HML, dos dados de exame, unidade e convênio que hoje estão no Corporate</t>
-        </is>
-      </c>
+      <c r="F21" s="12" t="n"/>
       <c r="G21" s="12" t="n"/>
       <c r="H21" s="12" t="n"/>
       <c r="I21" s="12" t="n"/>
@@ -1927,12 +1923,12 @@
       <c r="K21" s="12" t="n"/>
       <c r="L21" s="12" t="inlineStr">
         <is>
+          <t>Antes do teste funcional e depois da migração do Airflow para a GCP. Se o banco criado já tiver esses dados, esta linha sai.</t>
+        </is>
+      </c>
+      <c r="M21" s="12" t="inlineStr">
+        <is>
           <t>O DP serve exame, unidade e convênio para NAV e CDC. O diagrama leva as fontes ao Corporate, e o Corporate às APIs. Existe CORPORATE_HOM na documentação. O card 451661 cria o banco e está concluído. O card 451676, migrar SQL Server, está abortado. Não há card de carga.</t>
-        </is>
-      </c>
-      <c r="M21" s="12" t="inlineStr">
-        <is>
-          <t>Antes do teste funcional e depois da migração do Airflow para a GCP. Se o banco criado já tiver esses dados, esta linha sai.</t>
         </is>
       </c>
       <c r="N21" s="12" t="n"/>
@@ -1947,7 +1943,11 @@
           <t>6. HML — dado, depois do Airflow e do backend</t>
         </is>
       </c>
-      <c r="C22" s="14" t="n"/>
+      <c r="C22" s="14" t="inlineStr">
+        <is>
+          <t>[DP] Migração GCP | Blob Storage (adaptações na aplicação)</t>
+        </is>
+      </c>
       <c r="D22" s="14" t="inlineStr">
         <is>
           <t>Card da planilha</t>
@@ -1958,11 +1958,7 @@
           <t>451688</t>
         </is>
       </c>
-      <c r="F22" s="14" t="inlineStr">
-        <is>
-          <t>[DP] Migração GCP | Blob Storage (adaptações na aplicação)</t>
-        </is>
-      </c>
+      <c r="F22" s="14" t="n"/>
       <c r="G22" s="14" t="inlineStr">
         <is>
           <t>Média</t>
@@ -1986,12 +1982,12 @@
       <c r="K22" s="14" t="n"/>
       <c r="L22" s="14" t="inlineStr">
         <is>
+          <t>Depois do Airflow de HML e depois do backend e do frontend do DP. A planilha não diz se o download D+1 lê este Blob; por isso o D+1 não foi colocado obrigatoriamente depois.</t>
+        </is>
+      </c>
+      <c r="M22" s="14" t="inlineStr">
+        <is>
           <t>A documentação registra 269 GB de Blob. A dependência do card pede Airflow, backend e frontend. A data 03/02/27 não define a posição.</t>
-        </is>
-      </c>
-      <c r="M22" s="14" t="inlineStr">
-        <is>
-          <t>Depois do Airflow de HML e depois do backend e do frontend do DP. A planilha não diz se o download D+1 lê este Blob; por isso o D+1 não foi colocado obrigatoriamente depois.</t>
         </is>
       </c>
       <c r="N22" s="15" t="inlineStr">
@@ -2012,22 +2008,18 @@
           <t>6. HML — dado, depois do Airflow e do backend</t>
         </is>
       </c>
-      <c r="C23" s="13" t="inlineStr">
-        <is>
-          <t>Inclusa por IA — gap identificado</t>
-        </is>
-      </c>
-      <c r="D23" s="12" t="inlineStr">
-        <is>
-          <t>Lacuna — dependência citada no card</t>
+      <c r="C23" s="12" t="inlineStr">
+        <is>
+          <t>Cargas de cadastro</t>
+        </is>
+      </c>
+      <c r="D23" s="13" t="inlineStr">
+        <is>
+          <t>Lacuna — dependência citada no card - IA</t>
         </is>
       </c>
       <c r="E23" s="12" t="n"/>
-      <c r="F23" s="12" t="inlineStr">
-        <is>
-          <t>Cargas de cadastro</t>
-        </is>
-      </c>
+      <c r="F23" s="12" t="n"/>
       <c r="G23" s="12" t="n"/>
       <c r="H23" s="12" t="n"/>
       <c r="I23" s="12" t="n"/>
@@ -2035,12 +2027,12 @@
       <c r="K23" s="12" t="n"/>
       <c r="L23" s="12" t="inlineStr">
         <is>
+          <t>Antes dos workloads de portal que citam essa carga. Não há card, responsável nem prazo.</t>
+        </is>
+      </c>
+      <c r="M23" s="12" t="inlineStr">
+        <is>
           <t>Dependência escrita nos cards 470165 e 470100: 'Depende do airFlow pronto, cargas cadastro e D+1 (dowloads Cadastro)'. O diagrama tem o Portal de Cadastros como consumidor e, no desenho GCP, Excel do Portal Cadastro como fonte.</t>
-        </is>
-      </c>
-      <c r="M23" s="12" t="inlineStr">
-        <is>
-          <t>Antes dos workloads de portal que citam essa carga. Não há card, responsável nem prazo.</t>
         </is>
       </c>
       <c r="N23" s="12" t="n"/>
@@ -2055,22 +2047,18 @@
           <t>6. HML — dado, depois do Airflow e do backend</t>
         </is>
       </c>
-      <c r="C24" s="13" t="inlineStr">
-        <is>
-          <t>Inclusa por IA — gap identificado</t>
-        </is>
-      </c>
-      <c r="D24" s="12" t="inlineStr">
-        <is>
-          <t>Lacuna — dependência citada no card</t>
+      <c r="C24" s="12" t="inlineStr">
+        <is>
+          <t>Downloads D+1 de cadastro</t>
+        </is>
+      </c>
+      <c r="D24" s="13" t="inlineStr">
+        <is>
+          <t>Lacuna — dependência citada no card - IA</t>
         </is>
       </c>
       <c r="E24" s="12" t="n"/>
-      <c r="F24" s="12" t="inlineStr">
-        <is>
-          <t>Downloads D+1 de cadastro</t>
-        </is>
-      </c>
+      <c r="F24" s="12" t="n"/>
       <c r="G24" s="12" t="n"/>
       <c r="H24" s="12" t="n"/>
       <c r="I24" s="12" t="n"/>
@@ -2078,12 +2066,12 @@
       <c r="K24" s="12" t="n"/>
       <c r="L24" s="12" t="inlineStr">
         <is>
+          <t>No mesmo bloco das cargas de cadastro. A ordem entre D+1 e Blob não está escrita.</t>
+        </is>
+      </c>
+      <c r="M24" s="12" t="inlineStr">
+        <is>
           <t>Mesma dependência dos cards 470165 e 470100. Não há card só para o D+1.</t>
-        </is>
-      </c>
-      <c r="M24" s="12" t="inlineStr">
-        <is>
-          <t>No mesmo bloco das cargas de cadastro. A ordem entre D+1 e Blob não está escrita.</t>
         </is>
       </c>
       <c r="N24" s="12" t="n"/>
@@ -2098,7 +2086,11 @@
           <t>7. HML — portal, depois da carga que ele cita</t>
         </is>
       </c>
-      <c r="C25" s="14" t="n"/>
+      <c r="C25" s="14" t="inlineStr">
+        <is>
+          <t>Criação de Workloads do projeto BUSCA -&gt; datp-backoffice-backend</t>
+        </is>
+      </c>
       <c r="D25" s="14" t="inlineStr">
         <is>
           <t>Card da planilha</t>
@@ -2109,11 +2101,7 @@
           <t>468966</t>
         </is>
       </c>
-      <c r="F25" s="14" t="inlineStr">
-        <is>
-          <t>Criação de Workloads do projeto BUSCA -&gt; datp-backoffice-backend</t>
-        </is>
-      </c>
+      <c r="F25" s="14" t="n"/>
       <c r="G25" s="14" t="inlineStr">
         <is>
           <t>Alta</t>
@@ -2137,12 +2125,12 @@
       </c>
       <c r="L25" s="14" t="inlineStr">
         <is>
+          <t>Depois do Airflow de HML. Antes do teste integrado.</t>
+        </is>
+      </c>
+      <c r="M25" s="14" t="inlineStr">
+        <is>
           <t>Observação do card: depende do Airflow. Não cita a carga de cadastro.</t>
-        </is>
-      </c>
-      <c r="M25" s="14" t="inlineStr">
-        <is>
-          <t>Depois do Airflow de HML. Antes do teste integrado.</t>
         </is>
       </c>
       <c r="N25" s="15" t="inlineStr">
@@ -2163,7 +2151,11 @@
           <t>7. HML — portal, depois da carga que ele cita</t>
         </is>
       </c>
-      <c r="C26" s="14" t="n"/>
+      <c r="C26" s="14" t="inlineStr">
+        <is>
+          <t>Criação de Workloads do projeto PORTAL-CADASTRO -&gt; portal-cadastro-web</t>
+        </is>
+      </c>
       <c r="D26" s="14" t="inlineStr">
         <is>
           <t>Card da planilha</t>
@@ -2174,11 +2166,7 @@
           <t>470165</t>
         </is>
       </c>
-      <c r="F26" s="14" t="inlineStr">
-        <is>
-          <t>Criação de Workloads do projeto PORTAL-CADASTRO -&gt; portal-cadastro-web</t>
-        </is>
-      </c>
+      <c r="F26" s="14" t="n"/>
       <c r="G26" s="14" t="inlineStr">
         <is>
           <t>Média</t>
@@ -2202,12 +2190,12 @@
       </c>
       <c r="L26" s="14" t="inlineStr">
         <is>
+          <t>Depois de Airflow, cargas de cadastro e D+1, como a dependência escreve.</t>
+        </is>
+      </c>
+      <c r="M26" s="14" t="inlineStr">
+        <is>
           <t>A documentação cita o frontend do portal de cadastro e o repositório datp-backoffice-frontend-portal. O card desse repositório, 468985, está cancelado.</t>
-        </is>
-      </c>
-      <c r="M26" s="14" t="inlineStr">
-        <is>
-          <t>Depois de Airflow, cargas de cadastro e D+1, como a dependência escreve.</t>
         </is>
       </c>
       <c r="N26" s="15" t="inlineStr">
@@ -2228,7 +2216,11 @@
           <t>7. HML — portal, depois da carga que ele cita</t>
         </is>
       </c>
-      <c r="C27" s="14" t="n"/>
+      <c r="C27" s="14" t="inlineStr">
+        <is>
+          <t>Criação de Workloads do projeto BUSCA -&gt; datp-backoffice-frontend</t>
+        </is>
+      </c>
       <c r="D27" s="14" t="inlineStr">
         <is>
           <t>Card da planilha</t>
@@ -2239,11 +2231,7 @@
           <t>470100</t>
         </is>
       </c>
-      <c r="F27" s="14" t="inlineStr">
-        <is>
-          <t>Criação de Workloads do projeto BUSCA -&gt; datp-backoffice-frontend</t>
-        </is>
-      </c>
+      <c r="F27" s="14" t="n"/>
       <c r="G27" s="14" t="inlineStr">
         <is>
           <t>Média</t>
@@ -2267,12 +2255,12 @@
       </c>
       <c r="L27" s="14" t="inlineStr">
         <is>
+          <t>Junto do portal-cadastro-web.</t>
+        </is>
+      </c>
+      <c r="M27" s="14" t="inlineStr">
+        <is>
           <t>Mesma dependência do 470165.</t>
-        </is>
-      </c>
-      <c r="M27" s="14" t="inlineStr">
-        <is>
-          <t>Junto do portal-cadastro-web.</t>
         </is>
       </c>
       <c r="N27" s="15" t="inlineStr">
@@ -2293,7 +2281,11 @@
           <t>7. HML — portal, depois da carga que ele cita</t>
         </is>
       </c>
-      <c r="C28" s="14" t="n"/>
+      <c r="C28" s="14" t="inlineStr">
+        <is>
+          <t>[DP] Migração GCP | Migrar Backend -&gt; portal de cadastro (adaptações)</t>
+        </is>
+      </c>
       <c r="D28" s="14" t="inlineStr">
         <is>
           <t>Card da planilha</t>
@@ -2304,11 +2296,7 @@
           <t>451681</t>
         </is>
       </c>
-      <c r="F28" s="14" t="inlineStr">
-        <is>
-          <t>[DP] Migração GCP | Migrar Backend -&gt; portal de cadastro (adaptações)</t>
-        </is>
-      </c>
+      <c r="F28" s="14" t="n"/>
       <c r="G28" s="14" t="inlineStr">
         <is>
           <t>Alta</t>
@@ -2332,12 +2320,12 @@
       <c r="K28" s="14" t="n"/>
       <c r="L28" s="14" t="inlineStr">
         <is>
+          <t>No bloco do portal, junto dos workloads que a planilha amarra à carga. A data de fevereiro ficou para trás da adequação do Airflow de propósito.</t>
+        </is>
+      </c>
+      <c r="M28" s="14" t="inlineStr">
+        <is>
           <t>Adaptação do backend do portal. A data 10/02/27 não define a posição. O card não cita Airflow no texto; o workload do portal cita.</t>
-        </is>
-      </c>
-      <c r="M28" s="14" t="inlineStr">
-        <is>
-          <t>No bloco do portal, junto dos workloads que a planilha amarra à carga. A data de fevereiro ficou para trás da adequação do Airflow de propósito.</t>
         </is>
       </c>
       <c r="N28" s="15" t="inlineStr">
@@ -2358,7 +2346,11 @@
           <t>7. HML — portal, depois da carga que ele cita</t>
         </is>
       </c>
-      <c r="C29" s="14" t="n"/>
+      <c r="C29" s="14" t="inlineStr">
+        <is>
+          <t>[DP] Migração GCP | Migrar Frontend  Protal de cadastro (adaptações)</t>
+        </is>
+      </c>
       <c r="D29" s="14" t="inlineStr">
         <is>
           <t>Card da planilha</t>
@@ -2369,11 +2361,7 @@
           <t>451677</t>
         </is>
       </c>
-      <c r="F29" s="14" t="inlineStr">
-        <is>
-          <t>[DP] Migração GCP | Migrar Frontend  Protal de cadastro (adaptações)</t>
-        </is>
-      </c>
+      <c r="F29" s="14" t="n"/>
       <c r="G29" s="14" t="inlineStr">
         <is>
           <t>Alta</t>
@@ -2401,12 +2389,12 @@
       </c>
       <c r="L29" s="14" t="inlineStr">
         <is>
+          <t>A adaptação fica neste bloco. O teste do front é o card 451689.</t>
+        </is>
+      </c>
+      <c r="M29" s="14" t="inlineStr">
+        <is>
           <t>A observação condiciona o teste à integração. A data 07/02/27 não define a posição.</t>
-        </is>
-      </c>
-      <c r="M29" s="14" t="inlineStr">
-        <is>
-          <t>A adaptação fica neste bloco. O teste do front é o card 451689.</t>
         </is>
       </c>
       <c r="N29" s="15" t="inlineStr">
@@ -2427,7 +2415,11 @@
           <t>8. HML — teste funcional, e em seguida carga</t>
         </is>
       </c>
-      <c r="C30" s="16" t="n"/>
+      <c r="C30" s="16" t="inlineStr">
+        <is>
+          <t>[DP] Migração GCP | Testes Integrados, Homologação &amp; Plano de Rollback</t>
+        </is>
+      </c>
       <c r="D30" s="16" t="inlineStr">
         <is>
           <t>Card da planilha</t>
@@ -2440,14 +2432,10 @@
       </c>
       <c r="F30" s="16" t="inlineStr">
         <is>
-          <t>[DP] Migração GCP | Testes Integrados, Homologação &amp; Plano de Rollback</t>
-        </is>
-      </c>
-      <c r="G30" s="16" t="inlineStr">
-        <is>
           <t>Sem Definição de Escopo</t>
         </is>
       </c>
+      <c r="G30" s="16" t="n"/>
       <c r="H30" s="16" t="inlineStr">
         <is>
           <t>??</t>
@@ -2458,12 +2446,12 @@
       <c r="K30" s="16" t="n"/>
       <c r="L30" s="16" t="inlineStr">
         <is>
+          <t>Fecha o que a planilha chama de homologação. Produção só começa depois deste card e do teste de carga.</t>
+        </is>
+      </c>
+      <c r="M30" s="16" t="inlineStr">
+        <is>
           <t>Único card de teste. Não cita teste de carga. Sem definição de escopo. O template do documento lista teste funcional, performance, segurança e DR, todos sem conteúdo. Os fronts 451677 e 469051 dizem que só testam com tudo integrado.</t>
-        </is>
-      </c>
-      <c r="M30" s="16" t="inlineStr">
-        <is>
-          <t>Fecha o que a planilha chama de homologação. Produção só começa depois deste card e do teste de carga.</t>
         </is>
       </c>
       <c r="N30" s="17" t="inlineStr">
@@ -2484,22 +2472,18 @@
           <t>8. HML — teste funcional, e em seguida carga</t>
         </is>
       </c>
-      <c r="C31" s="19" t="inlineStr">
-        <is>
-          <t>Inclusa por IA — gap identificado</t>
-        </is>
-      </c>
-      <c r="D31" s="18" t="inlineStr">
-        <is>
-          <t>Marco pedido, sem card</t>
+      <c r="C31" s="18" t="inlineStr">
+        <is>
+          <t>Teste de carga em HML</t>
+        </is>
+      </c>
+      <c r="D31" s="19" t="inlineStr">
+        <is>
+          <t>Marco pedido, sem card - IA</t>
         </is>
       </c>
       <c r="E31" s="18" t="n"/>
-      <c r="F31" s="18" t="inlineStr">
-        <is>
-          <t>Teste de carga em HML</t>
-        </is>
-      </c>
+      <c r="F31" s="18" t="n"/>
       <c r="G31" s="18" t="n"/>
       <c r="H31" s="18" t="n"/>
       <c r="I31" s="18" t="n"/>
@@ -2507,12 +2491,12 @@
       <c r="K31" s="18" t="n"/>
       <c r="L31" s="18" t="inlineStr">
         <is>
+          <t>Depois do teste funcional. Sem cenário, volume ou API. Não é um card do BusinessMap.</t>
+        </is>
+      </c>
+      <c r="M31" s="18" t="inlineStr">
+        <is>
           <t>Pedido desta ordenação: ter tudo em HML para testes funcionais e de carga antes de planejar produção. O documento cita Performance no template de testes e não define volume, API nem meta. Nenhum card descreve o teste.</t>
-        </is>
-      </c>
-      <c r="M31" s="18" t="inlineStr">
-        <is>
-          <t>Depois do teste funcional. Sem cenário, volume ou API. Não é um card do BusinessMap.</t>
         </is>
       </c>
       <c r="N31" s="18" t="n"/>
@@ -2527,22 +2511,18 @@
           <t>9. HML — Databricks na GCP, antes da produção</t>
         </is>
       </c>
-      <c r="C32" s="21" t="inlineStr">
-        <is>
-          <t>Inclusa por IA — gap identificado</t>
-        </is>
-      </c>
-      <c r="D32" s="20" t="inlineStr">
-        <is>
-          <t>Lacuna — documentação</t>
+      <c r="C32" s="20" t="inlineStr">
+        <is>
+          <t>Workspaces Databricks de HML e de PRD na GCP</t>
+        </is>
+      </c>
+      <c r="D32" s="21" t="inlineStr">
+        <is>
+          <t>Lacuna — documentação - IA</t>
         </is>
       </c>
       <c r="E32" s="20" t="n"/>
-      <c r="F32" s="20" t="inlineStr">
-        <is>
-          <t>Workspaces Databricks de HML e de PRD na GCP</t>
-        </is>
-      </c>
+      <c r="F32" s="20" t="n"/>
       <c r="G32" s="20" t="n"/>
       <c r="H32" s="20" t="n"/>
       <c r="I32" s="20" t="n"/>
@@ -2550,12 +2530,12 @@
       <c r="K32" s="20" t="n"/>
       <c r="L32" s="20" t="inlineStr">
         <is>
+          <t>Entra porque a decisão é levar o Databricks para a GCP e a documentação comprova que os workspaces existem. Fica depois do teste funcional: o diagrama até as APIs não passa pelo Databricks, então o teste não espera esta linha. Produção começa depois dela.</t>
+        </is>
+      </c>
+      <c r="M32" s="20" t="inlineStr">
+        <is>
           <t>A documentação lista o workspace de PRD adb-7665073515379548 e o de HML adb-887971986833958. Não há jobs, notebooks nem tabelas de saída. Não há card para levar esses workspaces à GCP. O card 478328, que pede BigQuery, está na aba de discussão.</t>
-        </is>
-      </c>
-      <c r="M32" s="20" t="inlineStr">
-        <is>
-          <t>Entra porque a decisão é levar o Databricks para a GCP e a documentação comprova que os workspaces existem. Fica depois do teste funcional: o diagrama até as APIs não passa pelo Databricks, então o teste não espera esta linha. Produção começa depois dela.</t>
         </is>
       </c>
       <c r="N32" s="20" t="n"/>
@@ -2570,22 +2550,18 @@
           <t>10. Produção — planejar depois do teste de HML</t>
         </is>
       </c>
-      <c r="C33" s="23" t="inlineStr">
-        <is>
-          <t>Inclusa por IA — gap identificado</t>
-        </is>
-      </c>
-      <c r="D33" s="22" t="inlineStr">
-        <is>
-          <t>Lacuna — documentação</t>
+      <c r="C33" s="22" t="inlineStr">
+        <is>
+          <t>GKE de produção</t>
+        </is>
+      </c>
+      <c r="D33" s="23" t="inlineStr">
+        <is>
+          <t>Lacuna — documentação - IA</t>
         </is>
       </c>
       <c r="E33" s="22" t="n"/>
-      <c r="F33" s="22" t="inlineStr">
-        <is>
-          <t>GKE de produção</t>
-        </is>
-      </c>
+      <c r="F33" s="22" t="n"/>
       <c r="G33" s="22" t="n"/>
       <c r="H33" s="22" t="n"/>
       <c r="I33" s="22" t="n"/>
@@ -2593,12 +2569,12 @@
       <c r="K33" s="22" t="n"/>
       <c r="L33" s="22" t="inlineStr">
         <is>
+          <t>Primeiro item de produção porque a HML já tem cluster e a produção, no documento, também tem. Não há card.</t>
+        </is>
+      </c>
+      <c r="M33" s="22" t="inlineStr">
+        <is>
           <t>A documentação cita o cluster aks-prd-cadastro01, namespaces busca, dataprovider-data e portal-cadastro. O único card de GKE é o de HML, concluído.</t>
-        </is>
-      </c>
-      <c r="M33" s="22" t="inlineStr">
-        <is>
-          <t>Primeiro item de produção porque a HML já tem cluster e a produção, no documento, também tem. Não há card.</t>
         </is>
       </c>
       <c r="N33" s="22" t="n"/>
@@ -2613,7 +2589,11 @@
           <t>10. Produção — planejar depois do teste de HML</t>
         </is>
       </c>
-      <c r="C34" s="24" t="n"/>
+      <c r="C34" s="24" t="inlineStr">
+        <is>
+          <t>Criação de Workloads do projeto DATAPROVIDER-DATA -&gt; dp-data-stack-airflow-prd-worker-statefulset</t>
+        </is>
+      </c>
       <c r="D34" s="24" t="inlineStr">
         <is>
           <t>Card da planilha</t>
@@ -2624,11 +2604,7 @@
           <t>470150</t>
         </is>
       </c>
-      <c r="F34" s="24" t="inlineStr">
-        <is>
-          <t>Criação de Workloads do projeto DATAPROVIDER-DATA -&gt; dp-data-stack-airflow-prd-worker-statefulset</t>
-        </is>
-      </c>
+      <c r="F34" s="24" t="n"/>
       <c r="G34" s="24" t="inlineStr">
         <is>
           <t>Média</t>
@@ -2656,12 +2632,12 @@
       </c>
       <c r="L34" s="24" t="inlineStr">
         <is>
+          <t>Produção, pelo nome. A data 09/10/26 não trouxe este card para antes da HML.</t>
+        </is>
+      </c>
+      <c r="M34" s="24" t="inlineStr">
+        <is>
           <t>Nome com prd. Data escrita 09/10/26. A dependência é infra, não a POC do Airflow.</t>
-        </is>
-      </c>
-      <c r="M34" s="24" t="inlineStr">
-        <is>
-          <t>Produção, pelo nome. A data 09/10/26 não trouxe este card para antes da HML.</t>
         </is>
       </c>
       <c r="N34" s="25" t="inlineStr">
@@ -2682,7 +2658,11 @@
           <t>10. Produção — planejar depois do teste de HML</t>
         </is>
       </c>
-      <c r="C35" s="24" t="n"/>
+      <c r="C35" s="24" t="inlineStr">
+        <is>
+          <t>Criação de Workloads do projeto DATAPROVIDER-DATA -&gt; dp-data-stack-airflow-prd</t>
+        </is>
+      </c>
       <c r="D35" s="24" t="inlineStr">
         <is>
           <t>Card da planilha</t>
@@ -2693,11 +2673,7 @@
           <t>470149</t>
         </is>
       </c>
-      <c r="F35" s="24" t="inlineStr">
-        <is>
-          <t>Criação de Workloads do projeto DATAPROVIDER-DATA -&gt; dp-data-stack-airflow-prd</t>
-        </is>
-      </c>
+      <c r="F35" s="24" t="n"/>
       <c r="G35" s="24" t="inlineStr">
         <is>
           <t>Média</t>
@@ -2725,12 +2701,12 @@
       </c>
       <c r="L35" s="24" t="inlineStr">
         <is>
+          <t>No bloco de produção, na ordem em que a planilha lista os workloads de Airflow.</t>
+        </is>
+      </c>
+      <c r="M35" s="24" t="inlineStr">
+        <is>
           <t>Nome com prd. Data escrita 09/10/26.</t>
-        </is>
-      </c>
-      <c r="M35" s="24" t="inlineStr">
-        <is>
-          <t>No bloco de produção, na ordem em que a planilha lista os workloads de Airflow.</t>
         </is>
       </c>
       <c r="N35" s="25" t="inlineStr">
@@ -2751,7 +2727,11 @@
           <t>10. Produção — planejar depois do teste de HML</t>
         </is>
       </c>
-      <c r="C36" s="24" t="n"/>
+      <c r="C36" s="24" t="inlineStr">
+        <is>
+          <t>Criação de Workloads do projeto DATAPROVIDER-DATA -&gt; dp-data-stack-airflow-prd-sync-users</t>
+        </is>
+      </c>
       <c r="D36" s="24" t="inlineStr">
         <is>
           <t>Card da planilha</t>
@@ -2762,11 +2742,7 @@
           <t>470148</t>
         </is>
       </c>
-      <c r="F36" s="24" t="inlineStr">
-        <is>
-          <t>Criação de Workloads do projeto DATAPROVIDER-DATA -&gt; dp-data-stack-airflow-prd-sync-users</t>
-        </is>
-      </c>
+      <c r="F36" s="24" t="n"/>
       <c r="G36" s="24" t="inlineStr">
         <is>
           <t>Média</t>
@@ -2794,12 +2770,12 @@
       </c>
       <c r="L36" s="24" t="inlineStr">
         <is>
+          <t>No bloco de produção, na ordem original.</t>
+        </is>
+      </c>
+      <c r="M36" s="24" t="inlineStr">
+        <is>
           <t>Nome com prd. Data escrita 09/10/26.</t>
-        </is>
-      </c>
-      <c r="M36" s="24" t="inlineStr">
-        <is>
-          <t>No bloco de produção, na ordem original.</t>
         </is>
       </c>
       <c r="N36" s="25" t="inlineStr">
@@ -2820,7 +2796,11 @@
           <t>10. Produção — planejar depois do teste de HML</t>
         </is>
       </c>
-      <c r="C37" s="24" t="n"/>
+      <c r="C37" s="24" t="inlineStr">
+        <is>
+          <t>Criação de Workloads do projeto DATAPROVIDER-DATA -&gt; dp-data-stack-airflow-prd-scheduler</t>
+        </is>
+      </c>
       <c r="D37" s="24" t="inlineStr">
         <is>
           <t>Card da planilha</t>
@@ -2831,11 +2811,7 @@
           <t>470146</t>
         </is>
       </c>
-      <c r="F37" s="24" t="inlineStr">
-        <is>
-          <t>Criação de Workloads do projeto DATAPROVIDER-DATA -&gt; dp-data-stack-airflow-prd-scheduler</t>
-        </is>
-      </c>
+      <c r="F37" s="24" t="n"/>
       <c r="G37" s="24" t="inlineStr">
         <is>
           <t>Média</t>
@@ -2863,12 +2839,12 @@
       </c>
       <c r="L37" s="24" t="inlineStr">
         <is>
+          <t>No bloco de produção, na ordem original.</t>
+        </is>
+      </c>
+      <c r="M37" s="24" t="inlineStr">
+        <is>
           <t>Nome com prd. Data escrita 09/10/26.</t>
-        </is>
-      </c>
-      <c r="M37" s="24" t="inlineStr">
-        <is>
-          <t>No bloco de produção, na ordem original.</t>
         </is>
       </c>
       <c r="N37" s="25" t="inlineStr">
@@ -2889,7 +2865,11 @@
           <t>10. Produção — planejar depois do teste de HML</t>
         </is>
       </c>
-      <c r="C38" s="24" t="n"/>
+      <c r="C38" s="24" t="inlineStr">
+        <is>
+          <t>Criação de Workloads do projeto DATAPROVIDER-DATA -&gt; dp-data-stack-airflow-prd-flower</t>
+        </is>
+      </c>
       <c r="D38" s="24" t="inlineStr">
         <is>
           <t>Card da planilha</t>
@@ -2900,11 +2880,7 @@
           <t>470145</t>
         </is>
       </c>
-      <c r="F38" s="24" t="inlineStr">
-        <is>
-          <t>Criação de Workloads do projeto DATAPROVIDER-DATA -&gt; dp-data-stack-airflow-prd-flower</t>
-        </is>
-      </c>
+      <c r="F38" s="24" t="n"/>
       <c r="G38" s="24" t="inlineStr">
         <is>
           <t>Média</t>
@@ -2932,12 +2908,12 @@
       </c>
       <c r="L38" s="24" t="inlineStr">
         <is>
+          <t>No bloco de produção, na ordem original.</t>
+        </is>
+      </c>
+      <c r="M38" s="24" t="inlineStr">
+        <is>
           <t>Nome com prd. Data escrita 09/10/26.</t>
-        </is>
-      </c>
-      <c r="M38" s="24" t="inlineStr">
-        <is>
-          <t>No bloco de produção, na ordem original.</t>
         </is>
       </c>
       <c r="N38" s="25" t="inlineStr">
@@ -2958,7 +2934,11 @@
           <t>10. Produção — planejar depois do teste de HML</t>
         </is>
       </c>
-      <c r="C39" s="24" t="n"/>
+      <c r="C39" s="24" t="inlineStr">
+        <is>
+          <t>Criação de Workloads do projeto DATAPROVIDER-DATA -&gt; dp-data-stack-airflow-prd-db-migrations</t>
+        </is>
+      </c>
       <c r="D39" s="24" t="inlineStr">
         <is>
           <t>Card da planilha</t>
@@ -2969,11 +2949,7 @@
           <t>468978</t>
         </is>
       </c>
-      <c r="F39" s="24" t="inlineStr">
-        <is>
-          <t>Criação de Workloads do projeto DATAPROVIDER-DATA -&gt; dp-data-stack-airflow-prd-db-migrations</t>
-        </is>
-      </c>
+      <c r="F39" s="24" t="n"/>
       <c r="G39" s="24" t="inlineStr">
         <is>
           <t>Média</t>
@@ -3001,12 +2977,12 @@
       </c>
       <c r="L39" s="24" t="inlineStr">
         <is>
+          <t>No bloco de produção, na ordem original.</t>
+        </is>
+      </c>
+      <c r="M39" s="24" t="inlineStr">
+        <is>
           <t>Nome com prd. Data escrita 09/10/26.</t>
-        </is>
-      </c>
-      <c r="M39" s="24" t="inlineStr">
-        <is>
-          <t>No bloco de produção, na ordem original.</t>
         </is>
       </c>
       <c r="N39" s="25" t="inlineStr">
@@ -3027,7 +3003,11 @@
           <t>10. Produção — planejar depois do teste de HML</t>
         </is>
       </c>
-      <c r="C40" s="24" t="n"/>
+      <c r="C40" s="24" t="inlineStr">
+        <is>
+          <t>[DP] Migração GCP | Event Hub para Pub/Sub</t>
+        </is>
+      </c>
       <c r="D40" s="24" t="inlineStr">
         <is>
           <t>Card da planilha</t>
@@ -3038,11 +3018,7 @@
           <t>451683</t>
         </is>
       </c>
-      <c r="F40" s="24" t="inlineStr">
-        <is>
-          <t>[DP] Migração GCP | Event Hub para Pub/Sub</t>
-        </is>
-      </c>
+      <c r="F40" s="24" t="n"/>
       <c r="G40" s="24" t="inlineStr">
         <is>
           <t>Média</t>
@@ -3066,12 +3042,12 @@
       </c>
       <c r="L40" s="24" t="inlineStr">
         <is>
+          <t>No fim da produção, antes do cutover. Fora do teste funcional de HML, como o card pede.</t>
+        </is>
+      </c>
+      <c r="M40" s="24" t="inlineStr">
+        <is>
           <t>A documentação lista o Event Hub data-provider-prd. O desenho GCP tem Pub/Sub na ingestão. A planilha manda deixar por último. Nenhuma API cita Event Hub como dependência.</t>
-        </is>
-      </c>
-      <c r="M40" s="24" t="inlineStr">
-        <is>
-          <t>No fim da produção, antes do cutover. Fora do teste funcional de HML, como o card pede.</t>
         </is>
       </c>
       <c r="N40" s="25" t="inlineStr">
@@ -3092,7 +3068,11 @@
           <t>10. Produção — planejar depois do teste de HML</t>
         </is>
       </c>
-      <c r="C41" s="24" t="n"/>
+      <c r="C41" s="24" t="inlineStr">
+        <is>
+          <t>[DP] Migração GCP | Cutover &amp; Go-Live</t>
+        </is>
+      </c>
       <c r="D41" s="24" t="inlineStr">
         <is>
           <t>Card da planilha</t>
@@ -3105,14 +3085,10 @@
       </c>
       <c r="F41" s="24" t="inlineStr">
         <is>
-          <t>[DP] Migração GCP | Cutover &amp; Go-Live</t>
-        </is>
-      </c>
-      <c r="G41" s="24" t="inlineStr">
-        <is>
           <t>Sem Definição de Escopo</t>
         </is>
       </c>
+      <c r="G41" s="24" t="n"/>
       <c r="H41" s="24" t="inlineStr">
         <is>
           <t>??</t>
@@ -3123,12 +3099,12 @@
       <c r="K41" s="24" t="n"/>
       <c r="L41" s="24" t="inlineStr">
         <is>
+          <t>Última linha de produção. Sem escopo preenchido.</t>
+        </is>
+      </c>
+      <c r="M41" s="24" t="inlineStr">
+        <is>
           <t>Sem definição de escopo. O template do documento deixa em branco big bang ou gradual, DNS e janela.</t>
-        </is>
-      </c>
-      <c r="M41" s="24" t="inlineStr">
-        <is>
-          <t>Última linha de produção. Sem escopo preenchido.</t>
         </is>
       </c>
       <c r="N41" s="25" t="inlineStr">
@@ -3151,7 +3127,7 @@
       </c>
       <c r="C42" s="26" t="inlineStr">
         <is>
-          <t>Equipe — encerrada</t>
+          <t>Criação de Workloads do projeto BUSCA -&gt; dp-backend-api</t>
         </is>
       </c>
       <c r="D42" s="26" t="inlineStr">
@@ -3166,14 +3142,10 @@
       </c>
       <c r="F42" s="26" t="inlineStr">
         <is>
-          <t>Criação de Workloads do projeto BUSCA -&gt; dp-backend-api</t>
-        </is>
-      </c>
-      <c r="G42" s="26" t="inlineStr">
-        <is>
           <t>Cancelado</t>
         </is>
       </c>
+      <c r="G42" s="26" t="n"/>
       <c r="H42" s="26" t="n"/>
       <c r="I42" s="26" t="n"/>
       <c r="J42" s="26" t="n"/>
@@ -3184,12 +3156,12 @@
       </c>
       <c r="L42" s="26" t="inlineStr">
         <is>
+          <t>Cancelado pela equipe. Os backends 469049 e 468966 continuam no caminho. O documento não descreve este card além da observação de Cognitive Search.</t>
+        </is>
+      </c>
+      <c r="M42" s="26" t="inlineStr">
+        <is>
           <t>Complexidade Cancelado. A observação cita Cognitive Search.</t>
-        </is>
-      </c>
-      <c r="M42" s="26" t="inlineStr">
-        <is>
-          <t>Cancelado pela equipe. Os backends 469049 e 468966 continuam no caminho. O documento não descreve este card além da observação de Cognitive Search.</t>
         </is>
       </c>
       <c r="N42" s="27" t="inlineStr">
@@ -3212,7 +3184,7 @@
       </c>
       <c r="C43" s="26" t="inlineStr">
         <is>
-          <t>Equipe — encerrada</t>
+          <t>[DP] Migração GCP | Converter ETL's (DataBricks)</t>
         </is>
       </c>
       <c r="D43" s="26" t="inlineStr">
@@ -3227,26 +3199,22 @@
       </c>
       <c r="F43" s="26" t="inlineStr">
         <is>
-          <t>[DP] Migração GCP | Converter ETL's (DataBricks)</t>
-        </is>
-      </c>
-      <c r="G43" s="26" t="inlineStr">
-        <is>
           <t>Cancelado</t>
         </is>
       </c>
+      <c r="G43" s="26" t="n"/>
       <c r="H43" s="26" t="n"/>
       <c r="I43" s="26" t="n"/>
       <c r="J43" s="26" t="n"/>
       <c r="K43" s="26" t="n"/>
       <c r="L43" s="26" t="inlineStr">
         <is>
+          <t>Fora da ordem.</t>
+        </is>
+      </c>
+      <c r="M43" s="26" t="inlineStr">
+        <is>
           <t>Complexidade Cancelado.</t>
-        </is>
-      </c>
-      <c r="M43" s="26" t="inlineStr">
-        <is>
-          <t>Fora da ordem.</t>
         </is>
       </c>
       <c r="N43" s="27" t="inlineStr">
@@ -3269,7 +3237,7 @@
       </c>
       <c r="C44" s="26" t="inlineStr">
         <is>
-          <t>Equipe — encerrada</t>
+          <t>[DP] PostgreSQL - Levantamento de recursos para reescrita de código</t>
         </is>
       </c>
       <c r="D44" s="26" t="inlineStr">
@@ -3284,26 +3252,22 @@
       </c>
       <c r="F44" s="26" t="inlineStr">
         <is>
-          <t>[DP] PostgreSQL - Levantamento de recursos para reescrita de código</t>
-        </is>
-      </c>
-      <c r="G44" s="26" t="inlineStr">
-        <is>
           <t>Cancelado</t>
         </is>
       </c>
+      <c r="G44" s="26" t="n"/>
       <c r="H44" s="26" t="n"/>
       <c r="I44" s="26" t="n"/>
       <c r="J44" s="26" t="n"/>
       <c r="K44" s="26" t="n"/>
       <c r="L44" s="26" t="inlineStr">
         <is>
+          <t>Fora da ordem.</t>
+        </is>
+      </c>
+      <c r="M44" s="26" t="inlineStr">
+        <is>
           <t>Complexidade Cancelado.</t>
-        </is>
-      </c>
-      <c r="M44" s="26" t="inlineStr">
-        <is>
-          <t>Fora da ordem.</t>
         </is>
       </c>
       <c r="N44" s="27" t="inlineStr">
@@ -3326,7 +3290,7 @@
       </c>
       <c r="C45" s="26" t="inlineStr">
         <is>
-          <t>Equipe — encerrada</t>
+          <t>[DP] Migração GCP | Migrar banco de dados SQL Server -- ABORTADO</t>
         </is>
       </c>
       <c r="D45" s="26" t="inlineStr">
@@ -3341,26 +3305,22 @@
       </c>
       <c r="F45" s="26" t="inlineStr">
         <is>
-          <t>[DP] Migração GCP | Migrar banco de dados SQL Server -- ABORTADO</t>
-        </is>
-      </c>
-      <c r="G45" s="26" t="inlineStr">
-        <is>
           <t>Concluído</t>
         </is>
       </c>
+      <c r="G45" s="26" t="n"/>
       <c r="H45" s="26" t="n"/>
       <c r="I45" s="26" t="n"/>
       <c r="J45" s="26" t="n"/>
       <c r="K45" s="26" t="n"/>
       <c r="L45" s="26" t="inlineStr">
         <is>
+          <t>Fora do caminho. A existência de réplica em produção não virou atividade.</t>
+        </is>
+      </c>
+      <c r="M45" s="26" t="inlineStr">
+        <is>
           <t>Título ABORTADO e status Concluído. A documentação diz que a réplica 3 não será migrada e está desligada. Master com 10 vCores, réplica com 18, HML com 6, staging com 2. Tamanho citado: 461 GB.</t>
-        </is>
-      </c>
-      <c r="M45" s="26" t="inlineStr">
-        <is>
-          <t>Fora do caminho. A existência de réplica em produção não virou atividade.</t>
         </is>
       </c>
       <c r="N45" s="27" t="inlineStr">
@@ -3436,20 +3396,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="62" customWidth="1" min="3" max="3"/>
+    <col width="62" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="42" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
     <col width="24" customWidth="1" min="7" max="7"/>
-    <col width="36" customWidth="1" min="8" max="8"/>
-    <col width="70" customWidth="1" min="9" max="9"/>
-    <col width="42" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="36" customWidth="1" min="9" max="9"/>
+    <col width="70" customWidth="1" min="10" max="10"/>
+    <col width="42" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -3460,50 +3421,55 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Descrição</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Card ID</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Descrição</t>
-        </is>
-      </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>Complexidade</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Depêndencia</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Cronograma original</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Recurso Responsável</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Observações</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Por que não entra neste caminho</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Card URL</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Linha na planilha original</t>
         </is>
@@ -3515,50 +3481,51 @@
       </c>
       <c r="B2" s="28" t="inlineStr">
         <is>
+          <t>BigQuery =&gt; substituir dataBricks</t>
+        </is>
+      </c>
+      <c r="C2" s="28" t="inlineStr">
+        <is>
           <t>478328</t>
         </is>
       </c>
-      <c r="C2" s="28" t="inlineStr">
-        <is>
-          <t>BigQuery =&gt; substituir dataBricks</t>
-        </is>
-      </c>
-      <c r="D2" s="28" t="inlineStr">
+      <c r="D2" s="28" t="n"/>
+      <c r="E2" s="28" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="E2" s="28" t="inlineStr">
+      <c r="F2" s="28" t="inlineStr">
         <is>
           <t>Galerinha de dados DP</t>
         </is>
       </c>
-      <c r="F2" s="28" t="inlineStr">
+      <c r="G2" s="28" t="inlineStr">
         <is>
           <t>29/01/27</t>
         </is>
       </c>
-      <c r="G2" s="28" t="inlineStr">
+      <c r="H2" s="28" t="inlineStr">
         <is>
           <t>Dados</t>
         </is>
       </c>
-      <c r="H2" s="28" t="inlineStr">
+      <c r="I2" s="28" t="inlineStr">
         <is>
           <t>Levar toda a orquestração do dataBricks para o BigQuery</t>
         </is>
       </c>
-      <c r="I2" s="28" t="inlineStr">
+      <c r="J2" s="28" t="inlineStr">
         <is>
           <t>A equipe pediu levar a orquestração do Databricks para o BigQuery. O diagrama AS IS não passa pelo Databricks até as APIs. A ida para a GCP não exige essa troca: a decisão deste plano é levar os workspaces, e o card de converter os ETLs já está cancelado. O desenho com bronze, silver e gold está no documento sem a estratégia preenchida.</t>
         </is>
       </c>
-      <c r="J2" s="29" t="inlineStr">
+      <c r="K2" s="29" t="inlineStr">
         <is>
           <t>https://dasa.businessmap.io/ctrl_board/96/cards/478328/details</t>
         </is>
       </c>
-      <c r="K2" s="28" t="n">
+      <c r="L2" s="28" t="n">
         <v>9</v>
       </c>
     </row>
@@ -3568,12 +3535,12 @@
       </c>
       <c r="B3" s="28" t="inlineStr">
         <is>
+          <t>[DATP] DasaLogs -&gt; api local - unidades</t>
+        </is>
+      </c>
+      <c r="C3" s="28" t="inlineStr">
+        <is>
           <t>476063</t>
-        </is>
-      </c>
-      <c r="C3" s="28" t="inlineStr">
-        <is>
-          <t>[DATP] DasaLogs -&gt; api local - unidades</t>
         </is>
       </c>
       <c r="D3" s="28" t="inlineStr">
@@ -3585,17 +3552,18 @@
       <c r="F3" s="28" t="n"/>
       <c r="G3" s="28" t="n"/>
       <c r="H3" s="28" t="n"/>
-      <c r="I3" s="28" t="inlineStr">
+      <c r="I3" s="28" t="n"/>
+      <c r="J3" s="28" t="inlineStr">
         <is>
           <t>A equipe deixou em stand-by. O documento de arquitetura não cita DasaLogs no caminho de exame, unidade e convênio, nem nas APIs, no Airflow ou na busca.</t>
         </is>
       </c>
-      <c r="J3" s="29" t="inlineStr">
+      <c r="K3" s="29" t="inlineStr">
         <is>
           <t>https://dasa.businessmap.io/ctrl_board/96/cards/476063/details</t>
         </is>
       </c>
-      <c r="K3" s="28" t="n">
+      <c r="L3" s="28" t="n">
         <v>33</v>
       </c>
     </row>
@@ -3605,12 +3573,12 @@
       </c>
       <c r="B4" s="28" t="inlineStr">
         <is>
+          <t>Criação de Workloads do projeto BUSCA -&gt; dp-corporate-frontend</t>
+        </is>
+      </c>
+      <c r="C4" s="28" t="inlineStr">
+        <is>
           <t>470121</t>
-        </is>
-      </c>
-      <c r="C4" s="28" t="inlineStr">
-        <is>
-          <t>Criação de Workloads do projeto BUSCA -&gt; dp-corporate-frontend</t>
         </is>
       </c>
       <c r="D4" s="28" t="inlineStr">
@@ -3622,17 +3590,18 @@
       <c r="F4" s="28" t="n"/>
       <c r="G4" s="28" t="n"/>
       <c r="H4" s="28" t="n"/>
-      <c r="I4" s="28" t="inlineStr">
+      <c r="I4" s="28" t="n"/>
+      <c r="J4" s="28" t="inlineStr">
         <is>
           <t>A equipe cancelou o workload dp-corporate-frontend. A documentação ainda aponta essa URL como frontend do DP. O card 469051 segue no caminho com outro nome. Os dois não foram tratados como o mesmo frontend.</t>
         </is>
       </c>
-      <c r="J4" s="29" t="inlineStr">
+      <c r="K4" s="29" t="inlineStr">
         <is>
           <t>https://dasa.businessmap.io/ctrl_board/96/cards/470121/details</t>
         </is>
       </c>
-      <c r="K4" s="28" t="n">
+      <c r="L4" s="28" t="n">
         <v>32</v>
       </c>
     </row>
@@ -3642,12 +3611,12 @@
       </c>
       <c r="B5" s="28" t="inlineStr">
         <is>
+          <t>Criação de Workloads do projeto PORTAL-CADASTRO -&gt; datp-backoffice-frontend-portal</t>
+        </is>
+      </c>
+      <c r="C5" s="28" t="inlineStr">
+        <is>
           <t>468985</t>
-        </is>
-      </c>
-      <c r="C5" s="28" t="inlineStr">
-        <is>
-          <t>Criação de Workloads do projeto PORTAL-CADASTRO -&gt; datp-backoffice-frontend-portal</t>
         </is>
       </c>
       <c r="D5" s="28" t="inlineStr">
@@ -3658,36 +3627,37 @@
       <c r="E5" s="28" t="n"/>
       <c r="F5" s="28" t="n"/>
       <c r="G5" s="28" t="n"/>
-      <c r="H5" s="28" t="inlineStr">
+      <c r="H5" s="28" t="n"/>
+      <c r="I5" s="28" t="inlineStr">
         <is>
           <t>depende do airFlow</t>
         </is>
       </c>
-      <c r="I5" s="28" t="inlineStr">
+      <c r="J5" s="28" t="inlineStr">
         <is>
           <t>A equipe cancelou o workload do repositório datp-backoffice-frontend-portal. A documentação cita esse repositório como frontend do portal de cadastro. Os cards 470165 e 451677 seguem no caminho com outros nomes.</t>
         </is>
       </c>
-      <c r="J5" s="29" t="inlineStr">
+      <c r="K5" s="29" t="inlineStr">
         <is>
           <t>https://dasa.businessmap.io/ctrl_board/96/cards/468985/details</t>
         </is>
       </c>
-      <c r="K5" s="28" t="n">
+      <c r="L5" s="28" t="n">
         <v>20</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K5">
-    <sortState ref="A1:K5">
+  <autoFilter ref="A1:L5">
+    <sortState ref="A1:L5">
       <sortCondition descending="0" ref="A2:A200"/>
     </sortState>
   </autoFilter>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K5" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.6" bottom="0.6" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" scale="70" fitToHeight="0" fitToWidth="1"/>
@@ -3759,7 +3729,7 @@
     <row r="8" ht="48" customHeight="1">
       <c r="A8" s="31" t="inlineStr">
         <is>
-          <t>A coluna Indicação fica vazia quando a atividade é da equipe e permanece no caminho. O texto 'Inclusa por IA — gap identificado' marca o que não tinha card: a documentação ou a dependência de um card mostrou a falta. Nada disso recebeu responsável, prazo ou Card ID.</t>
+          <t>A coluna Origem recebe ' - IA' quando a linha não tinha card. A documentação ou a dependência de um card mostrou a falta. Essas linhas não têm responsável, prazo nem Card ID. Origem sem ' - IA' é atividade da equipe que permanece no caminho.</t>
         </is>
       </c>
     </row>
@@ -3773,7 +3743,7 @@
     <row r="10" ht="48" customHeight="1">
       <c r="A10" s="31" t="inlineStr">
         <is>
-          <t>Cards cancelados ou abortados que não entram nessa discussão ficam no fim, com Indicação 'Equipe — encerrada'.</t>
+          <t>Cards cancelados ou abortados que não entram nessa discussão ficam no fim, na etapa Encerrada pela equipe. O status deles sai da coluna Complexidade.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coloca todos os componentes na HML antes dos testes.
A carga do Corporate vira card do TIE, a busca entra como POC ao lado da spike de versão, elegibility segue como uma API só, e dp-corporate-frontend, teste funcional e teste de carga ficam na fila de homologação.

Co-authored-by: waneron <waneron@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/BM-GCP-Atividades-DP-ordem-temporal.xlsx
+++ b/BM-GCP-Atividades-DP-ordem-temporal.xlsx
@@ -13,12 +13,12 @@
     <sheet name="Dúvidas" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'BM - GCP Atividades - DP'!$A$1:$O$50</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'BM - GCP Atividades - DP'!$A$1:$O$52</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'BM - GCP Atividades - DP'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Discutir com a equipe'!$A$1:$L$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Discutir com a equipe'!$A$1:$L$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Discutir com a equipe'!$1:$1</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Regra de ordem'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Dúvidas'!$A$1:$C$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Dúvidas'!$A$1:$C$11</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Dúvidas'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -104,12 +104,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="00F8CBAD"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F8CBAD"/>
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
@@ -119,12 +119,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
+        <fgColor rgb="00E2D5F1"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E2D5F1"/>
+        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
     <fill>
@@ -174,7 +174,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -233,22 +233,28 @@
     <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -647,7 +653,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O50"/>
+  <dimension ref="A1:O52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1464,12 +1470,12 @@
       <c r="K14" s="8" t="n"/>
       <c r="L14" s="8" t="inlineStr">
         <is>
-          <t>Sobe com as APIs que não citam busca. A linha de agendamento, ao lado, cobre o nome da documentação.</t>
+          <t>Na fila das APIs, depois da conectividade.</t>
         </is>
       </c>
       <c r="M14" s="8" t="inlineStr">
         <is>
-          <t>Workload de elegibility. O documento chama a outra API de agendamento e o diagrama mostra busca-agendamento-backend. Este card não usa esse nome.</t>
+          <t>A planilha tem um card, datp-searcher-api-elegibility. É uma API. O esperado é esse workload no ar em HML, com as consultas que não citam busca.</t>
         </is>
       </c>
       <c r="N14" s="9" t="inlineStr">
@@ -1482,43 +1488,69 @@
       </c>
     </row>
     <row r="15" ht="52" customHeight="1">
-      <c r="A15" s="10" t="n">
+      <c r="A15" s="8" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="10" t="inlineStr">
+      <c r="B15" s="8" t="inlineStr">
         <is>
           <t>3. HML — APIs e gateway, em paralelo com o Airflow</t>
         </is>
       </c>
-      <c r="C15" s="10" t="inlineStr">
-        <is>
-          <t>API de agendamento documentada (busca-agendamento-backend)</t>
-        </is>
-      </c>
-      <c r="D15" s="11" t="inlineStr">
-        <is>
-          <t>IA</t>
-        </is>
-      </c>
-      <c r="E15" s="10" t="n"/>
-      <c r="F15" s="10" t="n"/>
-      <c r="G15" s="10" t="n"/>
-      <c r="H15" s="10" t="n"/>
-      <c r="I15" s="10" t="n"/>
-      <c r="J15" s="10" t="n"/>
-      <c r="K15" s="10" t="n"/>
-      <c r="L15" s="10" t="inlineStr">
-        <is>
-          <t>Na fila das APIs, para o nome do documento não ficar sem dono.</t>
-        </is>
-      </c>
-      <c r="M15" s="10" t="inlineStr">
-        <is>
-          <t>O documento lista agendamento entre as seis APIs e o diagrama mostra busca-agendamento-backend. Não há card com esse nome. O esperado é essa consulta existir em HML. Se for o mesmo serviço da elegibility (470113), as duas linhas viram uma.</t>
-        </is>
-      </c>
-      <c r="N15" s="10" t="n"/>
-      <c r="O15" s="10" t="n"/>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>Criação de Workloads do projeto BUSCA -&gt; datp-searcher-api-commons</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>Card da planilha</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>470112</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="n"/>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>Baixa</t>
+        </is>
+      </c>
+      <c r="H15" s="8" t="inlineStr">
+        <is>
+          <t>Backend Hj a conectividade está por IP, isso é errado</t>
+        </is>
+      </c>
+      <c r="I15" s="8" t="n"/>
+      <c r="J15" s="8" t="inlineStr">
+        <is>
+          <t>Back End</t>
+        </is>
+      </c>
+      <c r="K15" s="8" t="inlineStr">
+        <is>
+          <t>atuando</t>
+        </is>
+      </c>
+      <c r="L15" s="8" t="inlineStr">
+        <is>
+          <t>Na mesma fila, antes do teste de conectividade.</t>
+        </is>
+      </c>
+      <c r="M15" s="8" t="inlineStr">
+        <is>
+          <t>API commons. A continuação 476416 está concluída e este card segue em andamento. O esperado é ela no ar com as outras.</t>
+        </is>
+      </c>
+      <c r="N15" s="9" t="inlineStr">
+        <is>
+          <t>https://dasa.businessmap.io/ctrl_board/96/cards/470112/details</t>
+        </is>
+      </c>
+      <c r="O15" s="8" t="n">
+        <v>17</v>
+      </c>
     </row>
     <row r="16" ht="52" customHeight="1">
       <c r="A16" s="8" t="n">
@@ -1531,7 +1563,7 @@
       </c>
       <c r="C16" s="8" t="inlineStr">
         <is>
-          <t>Criação de Workloads do projeto BUSCA -&gt; datp-searcher-api-commons</t>
+          <t>[DP] Migração de aplicações, APIs</t>
         </is>
       </c>
       <c r="D16" s="8" t="inlineStr">
@@ -1541,7 +1573,7 @@
       </c>
       <c r="E16" s="8" t="inlineStr">
         <is>
-          <t>470112</t>
+          <t>424944</t>
         </is>
       </c>
       <c r="F16" s="8" t="n"/>
@@ -1552,37 +1584,37 @@
       </c>
       <c r="H16" s="8" t="inlineStr">
         <is>
-          <t>Backend Hj a conectividade está por IP, isso é errado</t>
-        </is>
-      </c>
-      <c r="I16" s="8" t="n"/>
+          <t>testar conectividade</t>
+        </is>
+      </c>
+      <c r="I16" s="8" t="inlineStr">
+        <is>
+          <t>15/12/26</t>
+        </is>
+      </c>
       <c r="J16" s="8" t="inlineStr">
         <is>
           <t>Back End</t>
         </is>
       </c>
-      <c r="K16" s="8" t="inlineStr">
-        <is>
-          <t>atuando</t>
-        </is>
-      </c>
+      <c r="K16" s="8" t="n"/>
       <c r="L16" s="8" t="inlineStr">
         <is>
-          <t>Na mesma fila, antes do teste de conectividade.</t>
+          <t>Logo depois dos workloads desta fila. O teste com o canal espera o dado e a busca.</t>
         </is>
       </c>
       <c r="M16" s="8" t="inlineStr">
         <is>
-          <t>API commons. A continuação 476416 está concluída e este card segue em andamento. O esperado é ela no ar com as outras.</t>
+          <t>Teste de conectividade das APIs, não teste funcional. O esperado é confirmar que a aplicação enxerga o destino novo, ainda sem exigir o dado completo.</t>
         </is>
       </c>
       <c r="N16" s="9" t="inlineStr">
         <is>
-          <t>https://dasa.businessmap.io/ctrl_board/96/cards/470112/details</t>
+          <t>https://dasa.businessmap.io/ctrl_board/96/cards/424944/details</t>
         </is>
       </c>
       <c r="O16" s="8" t="n">
-        <v>17</v>
+        <v>8</v>
       </c>
     </row>
     <row r="17" ht="52" customHeight="1">
@@ -1591,12 +1623,12 @@
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>3. HML — APIs e gateway, em paralelo com o Airflow</t>
+          <t>3. HML — front e back do DP, em paralelo com o Airflow</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>[DP] Migração de aplicações, APIs</t>
+          <t>[DP] Migração GCP | Migrar Backend -&gt; front do DP (adaptações)</t>
         </is>
       </c>
       <c r="D17" s="8" t="inlineStr">
@@ -1606,25 +1638,21 @@
       </c>
       <c r="E17" s="8" t="inlineStr">
         <is>
-          <t>424944</t>
+          <t>469049</t>
         </is>
       </c>
       <c r="F17" s="8" t="n"/>
       <c r="G17" s="8" t="inlineStr">
         <is>
-          <t>Baixa</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="H17" s="8" t="inlineStr">
         <is>
-          <t>testar conectividade</t>
-        </is>
-      </c>
-      <c r="I17" s="8" t="inlineStr">
-        <is>
-          <t>15/12/26</t>
-        </is>
-      </c>
+          <t>Ajuste de codigo, versao, eventual erro</t>
+        </is>
+      </c>
+      <c r="I17" s="8" t="n"/>
       <c r="J17" s="8" t="inlineStr">
         <is>
           <t>Back End</t>
@@ -1633,21 +1661,21 @@
       <c r="K17" s="8" t="n"/>
       <c r="L17" s="8" t="inlineStr">
         <is>
-          <t>Logo depois dos workloads desta fila. O teste com o canal espera o dado e a busca.</t>
+          <t>Sobe com as APIs. O teste da tela espera a integração.</t>
         </is>
       </c>
       <c r="M17" s="8" t="inlineStr">
         <is>
-          <t>Teste de conectividade das APIs, não teste funcional. O esperado é confirmar que a aplicação enxerga o destino novo, ainda sem exigir o dado completo.</t>
+          <t>Backend do frontend do DP, repositório datp-backoffice-backend. O esperado é o backoffice responder em HML. Não cita Airflow.</t>
         </is>
       </c>
       <c r="N17" s="9" t="inlineStr">
         <is>
-          <t>https://dasa.businessmap.io/ctrl_board/96/cards/424944/details</t>
+          <t>https://dasa.businessmap.io/ctrl_board/96/cards/469049/details</t>
         </is>
       </c>
       <c r="O17" s="8" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
     </row>
     <row r="18" ht="52" customHeight="1">
@@ -1661,7 +1689,7 @@
       </c>
       <c r="C18" s="8" t="inlineStr">
         <is>
-          <t>[DP] Migração GCP | Migrar Backend -&gt; front do DP (adaptações)</t>
+          <t>[DP] Migração GCP | Migrar Frontend  portal do DP (adaptações)</t>
         </is>
       </c>
       <c r="D18" s="8" t="inlineStr">
@@ -1671,13 +1699,13 @@
       </c>
       <c r="E18" s="8" t="inlineStr">
         <is>
-          <t>469049</t>
+          <t>469051</t>
         </is>
       </c>
       <c r="F18" s="8" t="n"/>
       <c r="G18" s="8" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Média</t>
         </is>
       </c>
       <c r="H18" s="8" t="inlineStr">
@@ -1691,90 +1719,68 @@
           <t>Back End</t>
         </is>
       </c>
-      <c r="K18" s="8" t="n"/>
+      <c r="K18" s="8" t="inlineStr">
+        <is>
+          <t>só é possivel testar o front com tudo integrado.</t>
+        </is>
+      </c>
       <c r="L18" s="8" t="inlineStr">
         <is>
-          <t>Sobe com as APIs. O teste da tela espera a integração.</t>
+          <t>A adaptação entra aqui. O teste da tela é o card 451689.</t>
         </is>
       </c>
       <c r="M18" s="8" t="inlineStr">
         <is>
-          <t>Backend do frontend do DP, repositório datp-backoffice-backend. O esperado é o backoffice responder em HML. Não cita Airflow.</t>
+          <t>Frontend do DP. A documentação cita a URL dp-corporate-frontend; o workload com esse nome está cancelado e ficou para discussão. O esperado é esta adaptação ser a tela aberta em HML, testada só com tudo integrado.</t>
         </is>
       </c>
       <c r="N18" s="9" t="inlineStr">
         <is>
-          <t>https://dasa.businessmap.io/ctrl_board/96/cards/469049/details</t>
+          <t>https://dasa.businessmap.io/ctrl_board/96/cards/469051/details</t>
         </is>
       </c>
       <c r="O18" s="8" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="19" ht="52" customHeight="1">
-      <c r="A19" s="8" t="n">
+      <c r="A19" s="10" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="8" t="inlineStr">
+      <c r="B19" s="10" t="inlineStr">
         <is>
           <t>3. HML — front e back do DP, em paralelo com o Airflow</t>
         </is>
       </c>
-      <c r="C19" s="8" t="inlineStr">
-        <is>
-          <t>[DP] Migração GCP | Migrar Frontend  portal do DP (adaptações)</t>
-        </is>
-      </c>
-      <c r="D19" s="8" t="inlineStr">
-        <is>
-          <t>Card da planilha</t>
-        </is>
-      </c>
-      <c r="E19" s="8" t="inlineStr">
-        <is>
-          <t>469051</t>
-        </is>
-      </c>
-      <c r="F19" s="8" t="n"/>
-      <c r="G19" s="8" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="H19" s="8" t="inlineStr">
-        <is>
-          <t>Ajuste de codigo, versao, eventual erro</t>
-        </is>
-      </c>
-      <c r="I19" s="8" t="n"/>
-      <c r="J19" s="8" t="inlineStr">
-        <is>
-          <t>Back End</t>
-        </is>
-      </c>
-      <c r="K19" s="8" t="inlineStr">
-        <is>
-          <t>só é possivel testar o front com tudo integrado.</t>
-        </is>
-      </c>
-      <c r="L19" s="8" t="inlineStr">
-        <is>
-          <t>A adaptação entra aqui. O teste da tela é o card 451689.</t>
-        </is>
-      </c>
-      <c r="M19" s="8" t="inlineStr">
-        <is>
-          <t>Frontend do DP. A documentação cita a URL dp-corporate-frontend; o workload com esse nome está cancelado e ficou para discussão. O esperado é esta adaptação ser a tela aberta em HML, testada só com tudo integrado.</t>
-        </is>
-      </c>
-      <c r="N19" s="9" t="inlineStr">
-        <is>
-          <t>https://dasa.businessmap.io/ctrl_board/96/cards/469051/details</t>
-        </is>
-      </c>
-      <c r="O19" s="8" t="n">
-        <v>14</v>
-      </c>
+      <c r="C19" s="10" t="inlineStr">
+        <is>
+          <t>dp-corporate-frontend na HML</t>
+        </is>
+      </c>
+      <c r="D19" s="11" t="inlineStr">
+        <is>
+          <t>IA</t>
+        </is>
+      </c>
+      <c r="E19" s="10" t="n"/>
+      <c r="F19" s="10" t="n"/>
+      <c r="G19" s="10" t="n"/>
+      <c r="H19" s="10" t="n"/>
+      <c r="I19" s="10" t="n"/>
+      <c r="J19" s="10" t="n"/>
+      <c r="K19" s="10" t="n"/>
+      <c r="L19" s="10" t="inlineStr">
+        <is>
+          <t>Com os frontends do DP, antes dos testes.</t>
+        </is>
+      </c>
+      <c r="M19" s="10" t="inlineStr">
+        <is>
+          <t>A documentação cita a URL dp-corporate-frontend. O workload 470121 foi cancelado pela equipe. O esperado é este frontend estar na HML para ser homologado.</t>
+        </is>
+      </c>
+      <c r="N19" s="10" t="n"/>
+      <c r="O19" s="10" t="n"/>
     </row>
     <row r="20" ht="52" customHeight="1">
       <c r="A20" s="12" t="n">
@@ -1782,12 +1788,12 @@
       </c>
       <c r="B20" s="12" t="inlineStr">
         <is>
-          <t>4. HML — índice e exam, em paralelo com o Airflow</t>
+          <t>5. HML — migrar o Airflow da Azure para a GCP</t>
         </is>
       </c>
       <c r="C20" s="12" t="inlineStr">
         <is>
-          <t>[DP] Migração GCP | Index (cognitive search &gt; vertex - adaptar na aplicação)</t>
+          <t>Spike -&gt; Airflow na versao mais nova do airflow</t>
         </is>
       </c>
       <c r="D20" s="12" t="inlineStr">
@@ -1797,7 +1803,7 @@
       </c>
       <c r="E20" s="12" t="inlineStr">
         <is>
-          <t>451682</t>
+          <t>478326</t>
         </is>
       </c>
       <c r="F20" s="12" t="n"/>
@@ -1808,98 +1814,102 @@
       </c>
       <c r="H20" s="12" t="inlineStr">
         <is>
+          <t>Victor, subir um docker e testar ambienteLocal</t>
+        </is>
+      </c>
+      <c r="I20" s="12" t="inlineStr">
+        <is>
+          <t>20/10/26</t>
+        </is>
+      </c>
+      <c r="J20" s="12" t="inlineStr">
+        <is>
+          <t>Back End</t>
+        </is>
+      </c>
+      <c r="K20" s="12" t="inlineStr">
+        <is>
+          <t>Aqui já vai ser possivel pegar imcompatibilidade de versao</t>
+        </is>
+      </c>
+      <c r="L20" s="12" t="inlineStr">
+        <is>
+          <t>Abre a frente do Airflow, em paralelo com as APIs. A migração e a carga esperam o resultado.</t>
+        </is>
+      </c>
+      <c r="M20" s="12" t="inlineStr">
+        <is>
+          <t>O Airflow já está na Azure. Esta spike, em docker local, acha o que quebra da versão 2.2.5 para a versão do Google. O esperado é a lista de incompatibilidades antes de migrar.</t>
+        </is>
+      </c>
+      <c r="N20" s="13" t="inlineStr">
+        <is>
+          <t>https://dasa.businessmap.io/ctrl_board/96/cards/478326/details</t>
+        </is>
+      </c>
+      <c r="O20" s="12" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="21" ht="52" customHeight="1">
+      <c r="A21" s="14" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="14" t="inlineStr">
+        <is>
+          <t>4. HML — POC de busca, como a spike de versão</t>
+        </is>
+      </c>
+      <c r="C21" s="14" t="inlineStr">
+        <is>
+          <t>[DP] Migração GCP | Index (cognitive search &gt; vertex - adaptar na aplicação)</t>
+        </is>
+      </c>
+      <c r="D21" s="14" t="inlineStr">
+        <is>
+          <t>Card da planilha</t>
+        </is>
+      </c>
+      <c r="E21" s="14" t="inlineStr">
+        <is>
+          <t>451682</t>
+        </is>
+      </c>
+      <c r="F21" s="14" t="n"/>
+      <c r="G21" s="14" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="H21" s="14" t="inlineStr">
+        <is>
           <t>Maior Risco, descoberta</t>
         </is>
       </c>
-      <c r="I20" s="12" t="n"/>
-      <c r="J20" s="12" t="inlineStr">
+      <c r="I21" s="14" t="n"/>
+      <c r="J21" s="14" t="inlineStr">
         <is>
           <t>Felipe Paixão | Back End</t>
         </is>
       </c>
-      <c r="K20" s="12" t="n"/>
-      <c r="L20" s="12" t="inlineStr">
-        <is>
-          <t>Antes da API de exam. As outras APIs não esperam este card: a planilha só cita a busca na exam.</t>
-        </is>
-      </c>
-      <c r="M20" s="12" t="inlineStr">
-        <is>
-          <t>O diagrama coloca o busca-search entre o Corporate e as APIs. O documento marca o Cognitive Search como dependência alta, ainda sem decisão de desacoplamento. O card troca o índice para Vertex. O esperado é a busca de exam funcionar como hoje.</t>
-        </is>
-      </c>
-      <c r="N20" s="13" t="inlineStr">
+      <c r="K21" s="14" t="n"/>
+      <c r="L21" s="14" t="inlineStr">
+        <is>
+          <t>Ao lado da spike de versão. A API de exam sobe depois desta POC.</t>
+        </is>
+      </c>
+      <c r="M21" s="14" t="inlineStr">
+        <is>
+          <t>A busca entra como POC, no mesmo espírito da spike de versão do Airflow. O card está em descoberta e é o maior risco. O esperado é saber o que quebra ao sair do Cognitive Search antes de homologar a API de exam.</t>
+        </is>
+      </c>
+      <c r="N21" s="15" t="inlineStr">
         <is>
           <t>https://dasa.businessmap.io/ctrl_board/96/cards/451682/details</t>
         </is>
       </c>
-      <c r="O20" s="12" t="n">
+      <c r="O21" s="14" t="n">
         <v>41</v>
-      </c>
-    </row>
-    <row r="21" ht="52" customHeight="1">
-      <c r="A21" s="12" t="n">
-        <v>20</v>
-      </c>
-      <c r="B21" s="12" t="inlineStr">
-        <is>
-          <t>4. HML — índice e exam, em paralelo com o Airflow</t>
-        </is>
-      </c>
-      <c r="C21" s="12" t="inlineStr">
-        <is>
-          <t>Criação de Workloads do projeto BUSCA -&gt; datp-searcher-api-exam</t>
-        </is>
-      </c>
-      <c r="D21" s="12" t="inlineStr">
-        <is>
-          <t>Card da planilha</t>
-        </is>
-      </c>
-      <c r="E21" s="12" t="inlineStr">
-        <is>
-          <t>470114</t>
-        </is>
-      </c>
-      <c r="F21" s="12" t="n"/>
-      <c r="G21" s="12" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="H21" s="12" t="inlineStr">
-        <is>
-          <t>Backend Hj a conectividade está por IP, isso é errado</t>
-        </is>
-      </c>
-      <c r="I21" s="12" t="n"/>
-      <c r="J21" s="12" t="inlineStr">
-        <is>
-          <t>Back End</t>
-        </is>
-      </c>
-      <c r="K21" s="12" t="inlineStr">
-        <is>
-          <t>depende cognitiveSearch</t>
-        </is>
-      </c>
-      <c r="L21" s="12" t="inlineStr">
-        <is>
-          <t>Depois do índice e depois da conectividade.</t>
-        </is>
-      </c>
-      <c r="M21" s="12" t="inlineStr">
-        <is>
-          <t>API de exam. Depende do Cognitive Search e também registra conectividade por IP errada. O esperado é o canal buscar exame na HML pelo índice novo.</t>
-        </is>
-      </c>
-      <c r="N21" s="13" t="inlineStr">
-        <is>
-          <t>https://dasa.businessmap.io/ctrl_board/96/cards/470114/details</t>
-        </is>
-      </c>
-      <c r="O21" s="12" t="n">
-        <v>18</v>
       </c>
     </row>
     <row r="22" ht="52" customHeight="1">
@@ -1908,12 +1918,12 @@
       </c>
       <c r="B22" s="14" t="inlineStr">
         <is>
-          <t>5. HML — migrar o Airflow da Azure para a GCP</t>
+          <t>4. HML — API de exam, depois da POC de busca</t>
         </is>
       </c>
       <c r="C22" s="14" t="inlineStr">
         <is>
-          <t>Spike -&gt; Airflow na versao mais nova do airflow</t>
+          <t>Criação de Workloads do projeto BUSCA -&gt; datp-searcher-api-exam</t>
         </is>
       </c>
       <c r="D22" s="14" t="inlineStr">
@@ -1923,7 +1933,7 @@
       </c>
       <c r="E22" s="14" t="inlineStr">
         <is>
-          <t>478326</t>
+          <t>470114</t>
         </is>
       </c>
       <c r="F22" s="14" t="n"/>
@@ -1934,14 +1944,10 @@
       </c>
       <c r="H22" s="14" t="inlineStr">
         <is>
-          <t>Victor, subir um docker e testar ambienteLocal</t>
-        </is>
-      </c>
-      <c r="I22" s="14" t="inlineStr">
-        <is>
-          <t>20/10/26</t>
-        </is>
-      </c>
+          <t>Backend Hj a conectividade está por IP, isso é errado</t>
+        </is>
+      </c>
+      <c r="I22" s="14" t="n"/>
       <c r="J22" s="14" t="inlineStr">
         <is>
           <t>Back End</t>
@@ -1949,78 +1955,78 @@
       </c>
       <c r="K22" s="14" t="inlineStr">
         <is>
-          <t>Aqui já vai ser possivel pegar imcompatibilidade de versao</t>
+          <t>depende cognitiveSearch</t>
         </is>
       </c>
       <c r="L22" s="14" t="inlineStr">
         <is>
-          <t>Abre a frente do Airflow, em paralelo com as APIs. A migração e a carga esperam o resultado.</t>
+          <t>Depois da POC de busca e antes do teste funcional.</t>
         </is>
       </c>
       <c r="M22" s="14" t="inlineStr">
         <is>
-          <t>O Airflow já está na Azure. Esta spike, em docker local, acha o que quebra da versão 2.2.5 para a versão do Google. O esperado é a lista de incompatibilidades antes de migrar.</t>
+          <t>API de exam. Depende da busca. O esperado é o workload no ar depois da POC, para a homologação incluir a consulta de exame.</t>
         </is>
       </c>
       <c r="N22" s="15" t="inlineStr">
         <is>
-          <t>https://dasa.businessmap.io/ctrl_board/96/cards/478326/details</t>
+          <t>https://dasa.businessmap.io/ctrl_board/96/cards/470114/details</t>
         </is>
       </c>
       <c r="O22" s="14" t="n">
-        <v>2</v>
+        <v>18</v>
       </c>
     </row>
     <row r="23" ht="52" customHeight="1">
-      <c r="A23" s="14" t="n">
+      <c r="A23" s="12" t="n">
         <v>22</v>
       </c>
-      <c r="B23" s="14" t="inlineStr">
+      <c r="B23" s="12" t="inlineStr">
         <is>
           <t>5. HML — migrar o Airflow da Azure para a GCP</t>
         </is>
       </c>
-      <c r="C23" s="14" t="inlineStr">
+      <c r="C23" s="12" t="inlineStr">
         <is>
           <t>Criar historia adequação airflow, vinculada ao fim da poc do Victor =&gt; necessario devido versao de airflow</t>
         </is>
       </c>
-      <c r="D23" s="14" t="inlineStr">
+      <c r="D23" s="12" t="inlineStr">
         <is>
           <t>Card da planilha</t>
         </is>
       </c>
-      <c r="E23" s="14" t="n"/>
-      <c r="F23" s="14" t="n"/>
-      <c r="G23" s="14" t="inlineStr">
+      <c r="E23" s="12" t="n"/>
+      <c r="F23" s="12" t="n"/>
+      <c r="G23" s="12" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="H23" s="14" t="inlineStr">
+      <c r="H23" s="12" t="inlineStr">
         <is>
           <t>as adequações levarão tempo, pode ser a maior data.</t>
         </is>
       </c>
-      <c r="I23" s="14" t="inlineStr">
+      <c r="I23" s="12" t="inlineStr">
         <is>
           <t>entre março e abril de 2027</t>
         </is>
       </c>
-      <c r="J23" s="14" t="n"/>
-      <c r="K23" s="14" t="n"/>
-      <c r="L23" s="14" t="inlineStr">
+      <c r="J23" s="12" t="n"/>
+      <c r="K23" s="12" t="n"/>
+      <c r="L23" s="12" t="inlineStr">
         <is>
           <t>Depois da spike. Carga e portal vêm em seguida.</t>
         </is>
       </c>
-      <c r="M23" s="14" t="inlineStr">
+      <c r="M23" s="12" t="inlineStr">
         <is>
           <t>É a ida do Airflow da Azure para a GCP, por causa da versão. Não tem Card ID. Portal, Blob e backoffice dependem desse Airflow já na GCP. Os workloads com prd no nome ficam na produção.</t>
         </is>
       </c>
-      <c r="N23" s="14" t="n"/>
-      <c r="O23" s="14" t="n">
+      <c r="N23" s="12" t="n"/>
+      <c r="O23" s="12" t="n">
         <v>13</v>
       </c>
     </row>
@@ -2113,7 +2119,7 @@
       </c>
       <c r="C26" s="16" t="inlineStr">
         <is>
-          <t>Carga, no banco de HML, dos dados de exame, unidade e convênio que hoje estão no Corporate</t>
+          <t>[TIE] Card a criar — Migração da carga do Corporate para o banco de HML</t>
         </is>
       </c>
       <c r="D26" s="17" t="inlineStr">
@@ -2126,16 +2132,20 @@
       <c r="G26" s="16" t="n"/>
       <c r="H26" s="16" t="n"/>
       <c r="I26" s="16" t="n"/>
-      <c r="J26" s="16" t="n"/>
+      <c r="J26" s="16" t="inlineStr">
+        <is>
+          <t>TIE</t>
+        </is>
+      </c>
       <c r="K26" s="16" t="n"/>
       <c r="L26" s="16" t="inlineStr">
         <is>
-          <t>Depois do Airflow na GCP e das fontes. Antes do teste com os canais.</t>
+          <t>Depois do Airflow na GCP e das fontes. Antes dos testes, senão o canal consulta vazio.</t>
         </is>
       </c>
       <c r="M26" s="16" t="inlineStr">
         <is>
-          <t>As APIs servem exame, unidade e convênio. O banco de HML existe e a cópia do SQL Server foi abortada. O esperado é esse banco receber os dados do Corporate, para o NAV e o CDC não consultarem vazio.</t>
+          <t>Card a criar, responsabilidade do TIE. O banco de HML existe e a cópia do SQL Server foi abortada. O esperado é o TIE migrar a carga do Corporate para esse banco, com exame, unidade e convênio.</t>
         </is>
       </c>
       <c r="N26" s="16" t="n"/>
@@ -2619,56 +2629,38 @@
       </c>
       <c r="B35" s="20" t="inlineStr">
         <is>
-          <t>8. HML — teste funcional, e em seguida carga</t>
+          <t>8. HML — Databricks, antes da homologação</t>
         </is>
       </c>
       <c r="C35" s="20" t="inlineStr">
         <is>
-          <t>[DP] Migração GCP | Testes Integrados, Homologação &amp; Plano de Rollback</t>
-        </is>
-      </c>
-      <c r="D35" s="20" t="inlineStr">
-        <is>
-          <t>Card da planilha</t>
-        </is>
-      </c>
-      <c r="E35" s="20" t="inlineStr">
-        <is>
-          <t>451689</t>
-        </is>
-      </c>
-      <c r="F35" s="20" t="inlineStr">
-        <is>
-          <t>Sem Definição de Escopo</t>
-        </is>
-      </c>
+          <t>Workspaces Databricks de HML e de PRD na GCP</t>
+        </is>
+      </c>
+      <c r="D35" s="21" t="inlineStr">
+        <is>
+          <t>IA</t>
+        </is>
+      </c>
+      <c r="E35" s="20" t="n"/>
+      <c r="F35" s="20" t="n"/>
       <c r="G35" s="20" t="n"/>
-      <c r="H35" s="20" t="inlineStr">
-        <is>
-          <t>??</t>
-        </is>
-      </c>
+      <c r="H35" s="20" t="n"/>
       <c r="I35" s="20" t="n"/>
       <c r="J35" s="20" t="n"/>
       <c r="K35" s="20" t="n"/>
       <c r="L35" s="20" t="inlineStr">
         <is>
-          <t>Fecha a homologação, depois das APIs, da busca, do dado e do portal.</t>
+          <t>Antes do teste funcional. Componente que precisa estar no ambiente para ser homologado.</t>
         </is>
       </c>
       <c r="M35" s="20" t="inlineStr">
         <is>
-          <t>Único card de teste da equipe, sem escopo. O documento não define SLA. O esperado é o NAV, o CDC e o portal usarem exame, unidade e convênio na HML, com o mesmo contrato de hoje, e haver plano de rollback.</t>
-        </is>
-      </c>
-      <c r="N35" s="21" t="inlineStr">
-        <is>
-          <t>https://dasa.businessmap.io/ctrl_board/96/cards/451689/details</t>
-        </is>
-      </c>
-      <c r="O35" s="20" t="n">
-        <v>36</v>
-      </c>
+          <t>A decisão oficial é levar o Databricks para a GCP. A documentação lista os workspaces de HML e de PRD, sem jobs. O esperado é o Databricks na GCP antes da homologação, junto dos outros componentes.</t>
+        </is>
+      </c>
+      <c r="N35" s="20" t="n"/>
+      <c r="O35" s="20" t="n"/>
     </row>
     <row r="36" ht="52" customHeight="1">
       <c r="A36" s="22" t="n">
@@ -2676,38 +2668,64 @@
       </c>
       <c r="B36" s="22" t="inlineStr">
         <is>
-          <t>8. HML — teste funcional, e em seguida carga</t>
+          <t>8. HML — Event Hub, antes da homologação</t>
         </is>
       </c>
       <c r="C36" s="22" t="inlineStr">
         <is>
-          <t>Teste de carga em HML</t>
-        </is>
-      </c>
-      <c r="D36" s="23" t="inlineStr">
-        <is>
-          <t>IA</t>
-        </is>
-      </c>
-      <c r="E36" s="22" t="n"/>
+          <t>[DP] Migração GCP | Event Hub para Pub/Sub</t>
+        </is>
+      </c>
+      <c r="D36" s="22" t="inlineStr">
+        <is>
+          <t>Card da planilha</t>
+        </is>
+      </c>
+      <c r="E36" s="22" t="inlineStr">
+        <is>
+          <t>451683</t>
+        </is>
+      </c>
       <c r="F36" s="22" t="n"/>
-      <c r="G36" s="22" t="n"/>
-      <c r="H36" s="22" t="n"/>
+      <c r="G36" s="22" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="H36" s="22" t="inlineStr">
+        <is>
+          <t>Ultima demanda, por ultimo -&gt; falar depois</t>
+        </is>
+      </c>
       <c r="I36" s="22" t="n"/>
-      <c r="J36" s="22" t="n"/>
-      <c r="K36" s="22" t="n"/>
+      <c r="J36" s="22" t="inlineStr">
+        <is>
+          <t>BD</t>
+        </is>
+      </c>
+      <c r="K36" s="22" t="inlineStr">
+        <is>
+          <t>pode ficar por ultimo</t>
+        </is>
+      </c>
       <c r="L36" s="22" t="inlineStr">
         <is>
-          <t>Logo depois do teste funcional. Produção só começa depois.</t>
+          <t>Antes do teste funcional, com os demais componentes.</t>
         </is>
       </c>
       <c r="M36" s="22" t="inlineStr">
         <is>
-          <t>Não há card, volume nem meta. O documento cita performance sem plano. O esperado é exercitar a HML depois do teste funcional e antes de planejar produção.</t>
-        </is>
-      </c>
-      <c r="N36" s="22" t="n"/>
-      <c r="O36" s="22" t="n"/>
+          <t>A documentação lista o Event Hub data-provider-prd. O esperado é a troca para Pub/Sub estar na HML antes do teste, para o componente poder ser homologado.</t>
+        </is>
+      </c>
+      <c r="N36" s="23" t="inlineStr">
+        <is>
+          <t>https://dasa.businessmap.io/ctrl_board/96/cards/451683/details</t>
+        </is>
+      </c>
+      <c r="O36" s="22" t="n">
+        <v>29</v>
+      </c>
     </row>
     <row r="37" ht="52" customHeight="1">
       <c r="A37" s="24" t="n">
@@ -2715,12 +2733,12 @@
       </c>
       <c r="B37" s="24" t="inlineStr">
         <is>
-          <t>9. HML — Databricks na GCP, antes da produção</t>
+          <t>9. HML — teste funcional</t>
         </is>
       </c>
       <c r="C37" s="24" t="inlineStr">
         <is>
-          <t>Workspaces Databricks de HML e de PRD na GCP</t>
+          <t>Teste funcional em HML</t>
         </is>
       </c>
       <c r="D37" s="25" t="inlineStr">
@@ -2737,123 +2755,111 @@
       <c r="K37" s="24" t="n"/>
       <c r="L37" s="24" t="inlineStr">
         <is>
-          <t>Depois do teste dos canais e antes da produção. O diagrama até as APIs não passa pelo Databricks, então o NAV e o CDC não esperam esta linha.</t>
+          <t>Depois que todos os componentes da HML estão no ar. Antes do teste de carga.</t>
         </is>
       </c>
       <c r="M37" s="24" t="inlineStr">
         <is>
-          <t>A decisão oficial é levar o Databricks para a GCP, não o desenho de BigQuery. A documentação lista o workspace de PRD adb-7665073515379548 e o de HML adb-887971986833958, sem jobs. O esperado é os dois workspaces rodarem na GCP. O card 478328 ficou na aba de discussão.</t>
+          <t>Linha nova. O esperado é provar, na HML, que NAV, CDC e portal consultam exame, unidade e convênio, com gateway, APIs, busca, Airflow, carga do TIE, Blob, portal, Databricks, Event Hub, Redis e o frontend dp-corporate-frontend.</t>
         </is>
       </c>
       <c r="N37" s="24" t="n"/>
       <c r="O37" s="24" t="n"/>
     </row>
     <row r="38" ht="52" customHeight="1">
-      <c r="A38" s="26" t="n">
+      <c r="A38" s="24" t="n">
         <v>37</v>
       </c>
-      <c r="B38" s="26" t="inlineStr">
-        <is>
-          <t>10. Produção — planejar depois do teste de HML</t>
-        </is>
-      </c>
-      <c r="C38" s="26" t="inlineStr">
-        <is>
-          <t>GKE de produção</t>
-        </is>
-      </c>
-      <c r="D38" s="27" t="inlineStr">
+      <c r="B38" s="24" t="inlineStr">
+        <is>
+          <t>9. HML — teste de carga</t>
+        </is>
+      </c>
+      <c r="C38" s="24" t="inlineStr">
+        <is>
+          <t>Teste de carga em HML</t>
+        </is>
+      </c>
+      <c r="D38" s="25" t="inlineStr">
         <is>
           <t>IA</t>
         </is>
       </c>
-      <c r="E38" s="26" t="n"/>
-      <c r="F38" s="26" t="n"/>
-      <c r="G38" s="26" t="n"/>
-      <c r="H38" s="26" t="n"/>
-      <c r="I38" s="26" t="n"/>
-      <c r="J38" s="26" t="n"/>
-      <c r="K38" s="26" t="n"/>
-      <c r="L38" s="26" t="inlineStr">
-        <is>
-          <t>Primeira linha de produção.</t>
-        </is>
-      </c>
-      <c r="M38" s="26" t="inlineStr">
-        <is>
-          <t>A documentação cita o cluster aks-prd-cadastro01. O único GKE com card é o de HML, já concluído. O esperado é o cluster de produção existir só depois da HML testada.</t>
-        </is>
-      </c>
-      <c r="N38" s="26" t="n"/>
-      <c r="O38" s="26" t="n"/>
+      <c r="E38" s="24" t="n"/>
+      <c r="F38" s="24" t="n"/>
+      <c r="G38" s="24" t="n"/>
+      <c r="H38" s="24" t="n"/>
+      <c r="I38" s="24" t="n"/>
+      <c r="J38" s="24" t="n"/>
+      <c r="K38" s="24" t="n"/>
+      <c r="L38" s="24" t="inlineStr">
+        <is>
+          <t>Imediatamente depois do teste funcional.</t>
+        </is>
+      </c>
+      <c r="M38" s="24" t="inlineStr">
+        <is>
+          <t>Linha nova, depois do teste funcional. O documento não traz volume nem meta. O esperado é a mesma HML, já funcional, receber carga antes de qualquer plano de produção.</t>
+        </is>
+      </c>
+      <c r="N38" s="24" t="n"/>
+      <c r="O38" s="24" t="n"/>
     </row>
     <row r="39" ht="52" customHeight="1">
-      <c r="A39" s="28" t="n">
+      <c r="A39" s="26" t="n">
         <v>38</v>
       </c>
-      <c r="B39" s="28" t="inlineStr">
-        <is>
-          <t>10. Produção — planejar depois do teste de HML</t>
-        </is>
-      </c>
-      <c r="C39" s="28" t="inlineStr">
-        <is>
-          <t>Criação de Workloads do projeto DATAPROVIDER-DATA -&gt; dp-data-stack-airflow-prd-worker-statefulset</t>
-        </is>
-      </c>
-      <c r="D39" s="28" t="inlineStr">
+      <c r="B39" s="26" t="inlineStr">
+        <is>
+          <t>10. HML — homologação e rollback</t>
+        </is>
+      </c>
+      <c r="C39" s="26" t="inlineStr">
+        <is>
+          <t>[DP] Migração GCP | Testes Integrados, Homologação &amp; Plano de Rollback</t>
+        </is>
+      </c>
+      <c r="D39" s="26" t="inlineStr">
         <is>
           <t>Card da planilha</t>
         </is>
       </c>
-      <c r="E39" s="28" t="inlineStr">
-        <is>
-          <t>470150</t>
-        </is>
-      </c>
-      <c r="F39" s="28" t="n"/>
-      <c r="G39" s="28" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="H39" s="28" t="inlineStr">
-        <is>
-          <t>infra managedAirFlow - infra =&gt; sem data depende de infra</t>
-        </is>
-      </c>
-      <c r="I39" s="28" t="inlineStr">
-        <is>
-          <t>09/10/26</t>
-        </is>
-      </c>
-      <c r="J39" s="28" t="inlineStr">
-        <is>
-          <t>Infra</t>
-        </is>
-      </c>
-      <c r="K39" s="28" t="inlineStr">
-        <is>
-          <t>infra</t>
-        </is>
-      </c>
-      <c r="L39" s="28" t="inlineStr">
-        <is>
-          <t>No bloco de produção, na ordem original da planilha.</t>
-        </is>
-      </c>
-      <c r="M39" s="28" t="inlineStr">
-        <is>
-          <t>Worker do Airflow de produção. O esperado é esta peça no ar depois da HML. A data 09/10/26 da planilha não antecipa a linha.</t>
-        </is>
-      </c>
-      <c r="N39" s="29" t="inlineStr">
-        <is>
-          <t>https://dasa.businessmap.io/ctrl_board/96/cards/470150/details</t>
-        </is>
-      </c>
-      <c r="O39" s="28" t="n">
-        <v>23</v>
+      <c r="E39" s="26" t="inlineStr">
+        <is>
+          <t>451689</t>
+        </is>
+      </c>
+      <c r="F39" s="26" t="inlineStr">
+        <is>
+          <t>Sem Definição de Escopo</t>
+        </is>
+      </c>
+      <c r="G39" s="26" t="n"/>
+      <c r="H39" s="26" t="inlineStr">
+        <is>
+          <t>??</t>
+        </is>
+      </c>
+      <c r="I39" s="26" t="n"/>
+      <c r="J39" s="26" t="n"/>
+      <c r="K39" s="26" t="n"/>
+      <c r="L39" s="26" t="inlineStr">
+        <is>
+          <t>Fecha a homologação. Produção só começa depois.</t>
+        </is>
+      </c>
+      <c r="M39" s="26" t="inlineStr">
+        <is>
+          <t>Card da equipe para homologação e rollback. O esperado é o aceite da HML e o plano de volta, depois dos testes funcional e de carga.</t>
+        </is>
+      </c>
+      <c r="N39" s="27" t="inlineStr">
+        <is>
+          <t>https://dasa.businessmap.io/ctrl_board/96/cards/451689/details</t>
+        </is>
+      </c>
+      <c r="O39" s="26" t="n">
+        <v>36</v>
       </c>
     </row>
     <row r="40" ht="52" customHeight="1">
@@ -2862,465 +2868,451 @@
       </c>
       <c r="B40" s="28" t="inlineStr">
         <is>
-          <t>10. Produção — planejar depois do teste de HML</t>
+          <t>11. Produção — depois da homologação</t>
         </is>
       </c>
       <c r="C40" s="28" t="inlineStr">
         <is>
+          <t>GKE de produção</t>
+        </is>
+      </c>
+      <c r="D40" s="29" t="inlineStr">
+        <is>
+          <t>IA</t>
+        </is>
+      </c>
+      <c r="E40" s="28" t="n"/>
+      <c r="F40" s="28" t="n"/>
+      <c r="G40" s="28" t="n"/>
+      <c r="H40" s="28" t="n"/>
+      <c r="I40" s="28" t="n"/>
+      <c r="J40" s="28" t="n"/>
+      <c r="K40" s="28" t="n"/>
+      <c r="L40" s="28" t="inlineStr">
+        <is>
+          <t>Primeira linha de produção.</t>
+        </is>
+      </c>
+      <c r="M40" s="28" t="inlineStr">
+        <is>
+          <t>A documentação cita o cluster aks-prd-cadastro01. O único GKE com card é o de HML, já concluído. O esperado é o cluster de produção existir só depois da HML testada.</t>
+        </is>
+      </c>
+      <c r="N40" s="28" t="n"/>
+      <c r="O40" s="28" t="n"/>
+    </row>
+    <row r="41" ht="52" customHeight="1">
+      <c r="A41" s="30" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="30" t="inlineStr">
+        <is>
+          <t>11. Produção — depois da homologação</t>
+        </is>
+      </c>
+      <c r="C41" s="30" t="inlineStr">
+        <is>
+          <t>Criação de Workloads do projeto DATAPROVIDER-DATA -&gt; dp-data-stack-airflow-prd-worker-statefulset</t>
+        </is>
+      </c>
+      <c r="D41" s="30" t="inlineStr">
+        <is>
+          <t>Card da planilha</t>
+        </is>
+      </c>
+      <c r="E41" s="30" t="inlineStr">
+        <is>
+          <t>470150</t>
+        </is>
+      </c>
+      <c r="F41" s="30" t="n"/>
+      <c r="G41" s="30" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="H41" s="30" t="inlineStr">
+        <is>
+          <t>infra managedAirFlow - infra =&gt; sem data depende de infra</t>
+        </is>
+      </c>
+      <c r="I41" s="30" t="inlineStr">
+        <is>
+          <t>09/10/26</t>
+        </is>
+      </c>
+      <c r="J41" s="30" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="K41" s="30" t="inlineStr">
+        <is>
+          <t>infra</t>
+        </is>
+      </c>
+      <c r="L41" s="30" t="inlineStr">
+        <is>
+          <t>No bloco de produção, na ordem original da planilha.</t>
+        </is>
+      </c>
+      <c r="M41" s="30" t="inlineStr">
+        <is>
+          <t>Worker do Airflow de produção. O esperado é esta peça no ar depois da HML. A data 09/10/26 da planilha não antecipa a linha.</t>
+        </is>
+      </c>
+      <c r="N41" s="31" t="inlineStr">
+        <is>
+          <t>https://dasa.businessmap.io/ctrl_board/96/cards/470150/details</t>
+        </is>
+      </c>
+      <c r="O41" s="30" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="42" ht="52" customHeight="1">
+      <c r="A42" s="30" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="30" t="inlineStr">
+        <is>
+          <t>11. Produção — depois da homologação</t>
+        </is>
+      </c>
+      <c r="C42" s="30" t="inlineStr">
+        <is>
           <t>Criação de Workloads do projeto DATAPROVIDER-DATA -&gt; dp-data-stack-airflow-prd</t>
         </is>
       </c>
-      <c r="D40" s="28" t="inlineStr">
+      <c r="D42" s="30" t="inlineStr">
         <is>
           <t>Card da planilha</t>
         </is>
       </c>
-      <c r="E40" s="28" t="inlineStr">
+      <c r="E42" s="30" t="inlineStr">
         <is>
           <t>470149</t>
         </is>
       </c>
-      <c r="F40" s="28" t="n"/>
-      <c r="G40" s="28" t="inlineStr">
+      <c r="F42" s="30" t="n"/>
+      <c r="G42" s="30" t="inlineStr">
         <is>
           <t>Média</t>
         </is>
       </c>
-      <c r="H40" s="28" t="inlineStr">
+      <c r="H42" s="30" t="inlineStr">
         <is>
           <t>infra managedAirFlow - infra =&gt; sem data depende de infra</t>
         </is>
       </c>
-      <c r="I40" s="28" t="inlineStr">
+      <c r="I42" s="30" t="inlineStr">
         <is>
           <t>09/10/26</t>
         </is>
       </c>
-      <c r="J40" s="28" t="inlineStr">
+      <c r="J42" s="30" t="inlineStr">
         <is>
           <t>Infra</t>
         </is>
       </c>
-      <c r="K40" s="28" t="inlineStr">
+      <c r="K42" s="30" t="inlineStr">
         <is>
           <t>infra</t>
         </is>
       </c>
-      <c r="L40" s="28" t="inlineStr">
+      <c r="L42" s="30" t="inlineStr">
         <is>
           <t>No bloco de produção, na ordem original da planilha.</t>
         </is>
       </c>
-      <c r="M40" s="28" t="inlineStr">
+      <c r="M42" s="30" t="inlineStr">
         <is>
           <t>Workload principal do Airflow de produção. O esperado é ele no ar depois da HML.</t>
         </is>
       </c>
-      <c r="N40" s="29" t="inlineStr">
+      <c r="N42" s="31" t="inlineStr">
         <is>
           <t>https://dasa.businessmap.io/ctrl_board/96/cards/470149/details</t>
         </is>
       </c>
-      <c r="O40" s="28" t="n">
+      <c r="O42" s="30" t="n">
         <v>24</v>
       </c>
     </row>
-    <row r="41" ht="52" customHeight="1">
-      <c r="A41" s="28" t="n">
-        <v>40</v>
-      </c>
-      <c r="B41" s="28" t="inlineStr">
-        <is>
-          <t>10. Produção — planejar depois do teste de HML</t>
-        </is>
-      </c>
-      <c r="C41" s="28" t="inlineStr">
+    <row r="43" ht="52" customHeight="1">
+      <c r="A43" s="30" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="30" t="inlineStr">
+        <is>
+          <t>11. Produção — depois da homologação</t>
+        </is>
+      </c>
+      <c r="C43" s="30" t="inlineStr">
         <is>
           <t>Criação de Workloads do projeto DATAPROVIDER-DATA -&gt; dp-data-stack-airflow-prd-sync-users</t>
         </is>
       </c>
-      <c r="D41" s="28" t="inlineStr">
+      <c r="D43" s="30" t="inlineStr">
         <is>
           <t>Card da planilha</t>
         </is>
       </c>
-      <c r="E41" s="28" t="inlineStr">
+      <c r="E43" s="30" t="inlineStr">
         <is>
           <t>470148</t>
         </is>
       </c>
-      <c r="F41" s="28" t="n"/>
-      <c r="G41" s="28" t="inlineStr">
+      <c r="F43" s="30" t="n"/>
+      <c r="G43" s="30" t="inlineStr">
         <is>
           <t>Média</t>
         </is>
       </c>
-      <c r="H41" s="28" t="inlineStr">
+      <c r="H43" s="30" t="inlineStr">
         <is>
           <t>infra managedAirFlow - infra =&gt; sem data depende de infra</t>
         </is>
       </c>
-      <c r="I41" s="28" t="inlineStr">
+      <c r="I43" s="30" t="inlineStr">
         <is>
           <t>09/10/26</t>
         </is>
       </c>
-      <c r="J41" s="28" t="inlineStr">
+      <c r="J43" s="30" t="inlineStr">
         <is>
           <t>Infra</t>
         </is>
       </c>
-      <c r="K41" s="28" t="inlineStr">
+      <c r="K43" s="30" t="inlineStr">
         <is>
           <t>infra</t>
         </is>
       </c>
-      <c r="L41" s="28" t="inlineStr">
+      <c r="L43" s="30" t="inlineStr">
         <is>
           <t>No bloco de produção, na ordem original da planilha.</t>
         </is>
       </c>
-      <c r="M41" s="28" t="inlineStr">
+      <c r="M43" s="30" t="inlineStr">
         <is>
           <t>Sincronização de usuários do Airflow de produção. O esperado é ela no ar depois da HML.</t>
         </is>
       </c>
-      <c r="N41" s="29" t="inlineStr">
+      <c r="N43" s="31" t="inlineStr">
         <is>
           <t>https://dasa.businessmap.io/ctrl_board/96/cards/470148/details</t>
         </is>
       </c>
-      <c r="O41" s="28" t="n">
+      <c r="O43" s="30" t="n">
         <v>25</v>
       </c>
     </row>
-    <row r="42" ht="52" customHeight="1">
-      <c r="A42" s="28" t="n">
-        <v>41</v>
-      </c>
-      <c r="B42" s="28" t="inlineStr">
-        <is>
-          <t>10. Produção — planejar depois do teste de HML</t>
-        </is>
-      </c>
-      <c r="C42" s="28" t="inlineStr">
+    <row r="44" ht="52" customHeight="1">
+      <c r="A44" s="30" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="30" t="inlineStr">
+        <is>
+          <t>11. Produção — depois da homologação</t>
+        </is>
+      </c>
+      <c r="C44" s="30" t="inlineStr">
         <is>
           <t>Criação de Workloads do projeto DATAPROVIDER-DATA -&gt; dp-data-stack-airflow-prd-scheduler</t>
         </is>
       </c>
-      <c r="D42" s="28" t="inlineStr">
+      <c r="D44" s="30" t="inlineStr">
         <is>
           <t>Card da planilha</t>
         </is>
       </c>
-      <c r="E42" s="28" t="inlineStr">
+      <c r="E44" s="30" t="inlineStr">
         <is>
           <t>470146</t>
         </is>
       </c>
-      <c r="F42" s="28" t="n"/>
-      <c r="G42" s="28" t="inlineStr">
+      <c r="F44" s="30" t="n"/>
+      <c r="G44" s="30" t="inlineStr">
         <is>
           <t>Média</t>
         </is>
       </c>
-      <c r="H42" s="28" t="inlineStr">
+      <c r="H44" s="30" t="inlineStr">
         <is>
           <t>infra managedAirFlow - infra =&gt; sem data depende de infra</t>
         </is>
       </c>
-      <c r="I42" s="28" t="inlineStr">
+      <c r="I44" s="30" t="inlineStr">
         <is>
           <t>09/10/26</t>
         </is>
       </c>
-      <c r="J42" s="28" t="inlineStr">
+      <c r="J44" s="30" t="inlineStr">
         <is>
           <t>Infra</t>
         </is>
       </c>
-      <c r="K42" s="28" t="inlineStr">
+      <c r="K44" s="30" t="inlineStr">
         <is>
           <t>infra</t>
         </is>
       </c>
-      <c r="L42" s="28" t="inlineStr">
+      <c r="L44" s="30" t="inlineStr">
         <is>
           <t>No bloco de produção, na ordem original da planilha.</t>
         </is>
       </c>
-      <c r="M42" s="28" t="inlineStr">
+      <c r="M44" s="30" t="inlineStr">
         <is>
           <t>Scheduler do Airflow de produção. O esperado é ele no ar depois da HML.</t>
         </is>
       </c>
-      <c r="N42" s="29" t="inlineStr">
+      <c r="N44" s="31" t="inlineStr">
         <is>
           <t>https://dasa.businessmap.io/ctrl_board/96/cards/470146/details</t>
         </is>
       </c>
-      <c r="O42" s="28" t="n">
+      <c r="O44" s="30" t="n">
         <v>26</v>
       </c>
     </row>
-    <row r="43" ht="52" customHeight="1">
-      <c r="A43" s="28" t="n">
-        <v>42</v>
-      </c>
-      <c r="B43" s="28" t="inlineStr">
-        <is>
-          <t>10. Produção — planejar depois do teste de HML</t>
-        </is>
-      </c>
-      <c r="C43" s="28" t="inlineStr">
+    <row r="45" ht="52" customHeight="1">
+      <c r="A45" s="30" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="30" t="inlineStr">
+        <is>
+          <t>11. Produção — depois da homologação</t>
+        </is>
+      </c>
+      <c r="C45" s="30" t="inlineStr">
         <is>
           <t>Criação de Workloads do projeto DATAPROVIDER-DATA -&gt; dp-data-stack-airflow-prd-flower</t>
         </is>
       </c>
-      <c r="D43" s="28" t="inlineStr">
+      <c r="D45" s="30" t="inlineStr">
         <is>
           <t>Card da planilha</t>
         </is>
       </c>
-      <c r="E43" s="28" t="inlineStr">
+      <c r="E45" s="30" t="inlineStr">
         <is>
           <t>470145</t>
         </is>
       </c>
-      <c r="F43" s="28" t="n"/>
-      <c r="G43" s="28" t="inlineStr">
+      <c r="F45" s="30" t="n"/>
+      <c r="G45" s="30" t="inlineStr">
         <is>
           <t>Média</t>
         </is>
       </c>
-      <c r="H43" s="28" t="inlineStr">
+      <c r="H45" s="30" t="inlineStr">
         <is>
           <t>infra managedAirFlow - infra =&gt; sem data depende de infra</t>
         </is>
       </c>
-      <c r="I43" s="28" t="inlineStr">
+      <c r="I45" s="30" t="inlineStr">
         <is>
           <t>09/10/26</t>
         </is>
       </c>
-      <c r="J43" s="28" t="inlineStr">
+      <c r="J45" s="30" t="inlineStr">
         <is>
           <t>Infra</t>
         </is>
       </c>
-      <c r="K43" s="28" t="inlineStr">
+      <c r="K45" s="30" t="inlineStr">
         <is>
           <t>infra</t>
         </is>
       </c>
-      <c r="L43" s="28" t="inlineStr">
+      <c r="L45" s="30" t="inlineStr">
         <is>
           <t>No bloco de produção, na ordem original da planilha.</t>
         </is>
       </c>
-      <c r="M43" s="28" t="inlineStr">
+      <c r="M45" s="30" t="inlineStr">
         <is>
           <t>Flower do Airflow de produção. O esperado é ele no ar depois da HML.</t>
         </is>
       </c>
-      <c r="N43" s="29" t="inlineStr">
+      <c r="N45" s="31" t="inlineStr">
         <is>
           <t>https://dasa.businessmap.io/ctrl_board/96/cards/470145/details</t>
         </is>
       </c>
-      <c r="O43" s="28" t="n">
+      <c r="O45" s="30" t="n">
         <v>27</v>
       </c>
     </row>
-    <row r="44" ht="52" customHeight="1">
-      <c r="A44" s="28" t="n">
-        <v>43</v>
-      </c>
-      <c r="B44" s="28" t="inlineStr">
-        <is>
-          <t>10. Produção — planejar depois do teste de HML</t>
-        </is>
-      </c>
-      <c r="C44" s="28" t="inlineStr">
+    <row r="46" ht="52" customHeight="1">
+      <c r="A46" s="30" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="30" t="inlineStr">
+        <is>
+          <t>11. Produção — depois da homologação</t>
+        </is>
+      </c>
+      <c r="C46" s="30" t="inlineStr">
         <is>
           <t>Criação de Workloads do projeto DATAPROVIDER-DATA -&gt; dp-data-stack-airflow-prd-db-migrations</t>
         </is>
       </c>
-      <c r="D44" s="28" t="inlineStr">
+      <c r="D46" s="30" t="inlineStr">
         <is>
           <t>Card da planilha</t>
         </is>
       </c>
-      <c r="E44" s="28" t="inlineStr">
+      <c r="E46" s="30" t="inlineStr">
         <is>
           <t>468978</t>
         </is>
       </c>
-      <c r="F44" s="28" t="n"/>
-      <c r="G44" s="28" t="inlineStr">
+      <c r="F46" s="30" t="n"/>
+      <c r="G46" s="30" t="inlineStr">
         <is>
           <t>Média</t>
         </is>
       </c>
-      <c r="H44" s="28" t="inlineStr">
+      <c r="H46" s="30" t="inlineStr">
         <is>
           <t>infra managedAirFlow - infra</t>
         </is>
       </c>
-      <c r="I44" s="28" t="inlineStr">
+      <c r="I46" s="30" t="inlineStr">
         <is>
           <t>09/10/26</t>
         </is>
       </c>
-      <c r="J44" s="28" t="inlineStr">
+      <c r="J46" s="30" t="inlineStr">
         <is>
           <t>Infra</t>
         </is>
       </c>
-      <c r="K44" s="28" t="inlineStr">
+      <c r="K46" s="30" t="inlineStr">
         <is>
           <t>infra</t>
         </is>
       </c>
-      <c r="L44" s="28" t="inlineStr">
+      <c r="L46" s="30" t="inlineStr">
         <is>
           <t>No bloco de produção, na ordem original da planilha.</t>
         </is>
       </c>
-      <c r="M44" s="28" t="inlineStr">
+      <c r="M46" s="30" t="inlineStr">
         <is>
           <t>Migração do banco do Airflow de produção. O esperado é ela rodar depois da HML.</t>
         </is>
       </c>
-      <c r="N44" s="29" t="inlineStr">
+      <c r="N46" s="31" t="inlineStr">
         <is>
           <t>https://dasa.businessmap.io/ctrl_board/96/cards/468978/details</t>
         </is>
       </c>
-      <c r="O44" s="28" t="n">
+      <c r="O46" s="30" t="n">
         <v>28</v>
-      </c>
-    </row>
-    <row r="45" ht="52" customHeight="1">
-      <c r="A45" s="28" t="n">
-        <v>44</v>
-      </c>
-      <c r="B45" s="28" t="inlineStr">
-        <is>
-          <t>10. Produção — planejar depois do teste de HML</t>
-        </is>
-      </c>
-      <c r="C45" s="28" t="inlineStr">
-        <is>
-          <t>[DP] Migração GCP | Event Hub para Pub/Sub</t>
-        </is>
-      </c>
-      <c r="D45" s="28" t="inlineStr">
-        <is>
-          <t>Card da planilha</t>
-        </is>
-      </c>
-      <c r="E45" s="28" t="inlineStr">
-        <is>
-          <t>451683</t>
-        </is>
-      </c>
-      <c r="F45" s="28" t="n"/>
-      <c r="G45" s="28" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="H45" s="28" t="inlineStr">
-        <is>
-          <t>Ultima demanda, por ultimo -&gt; falar depois</t>
-        </is>
-      </c>
-      <c r="I45" s="28" t="n"/>
-      <c r="J45" s="28" t="inlineStr">
-        <is>
-          <t>BD</t>
-        </is>
-      </c>
-      <c r="K45" s="28" t="inlineStr">
-        <is>
-          <t>pode ficar por ultimo</t>
-        </is>
-      </c>
-      <c r="L45" s="28" t="inlineStr">
-        <is>
-          <t>No fim da produção, antes do cutover.</t>
-        </is>
-      </c>
-      <c r="M45" s="28" t="inlineStr">
-        <is>
-          <t>A documentação lista o Event Hub data-provider-prd. A planilha manda deixar por último e nenhuma API cita esse evento. O esperado é a troca para Pub/Sub na produção, não na prova dos canais.</t>
-        </is>
-      </c>
-      <c r="N45" s="29" t="inlineStr">
-        <is>
-          <t>https://dasa.businessmap.io/ctrl_board/96/cards/451683/details</t>
-        </is>
-      </c>
-      <c r="O45" s="28" t="n">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="46" ht="52" customHeight="1">
-      <c r="A46" s="28" t="n">
-        <v>45</v>
-      </c>
-      <c r="B46" s="28" t="inlineStr">
-        <is>
-          <t>10. Produção — planejar depois do teste de HML</t>
-        </is>
-      </c>
-      <c r="C46" s="28" t="inlineStr">
-        <is>
-          <t>[DP] Migração GCP | Cutover &amp; Go-Live</t>
-        </is>
-      </c>
-      <c r="D46" s="28" t="inlineStr">
-        <is>
-          <t>Card da planilha</t>
-        </is>
-      </c>
-      <c r="E46" s="28" t="inlineStr">
-        <is>
-          <t>451691</t>
-        </is>
-      </c>
-      <c r="F46" s="28" t="inlineStr">
-        <is>
-          <t>Sem Definição de Escopo</t>
-        </is>
-      </c>
-      <c r="G46" s="28" t="n"/>
-      <c r="H46" s="28" t="inlineStr">
-        <is>
-          <t>??</t>
-        </is>
-      </c>
-      <c r="I46" s="28" t="n"/>
-      <c r="J46" s="28" t="n"/>
-      <c r="K46" s="28" t="n"/>
-      <c r="L46" s="28" t="inlineStr">
-        <is>
-          <t>Última linha de produção.</t>
-        </is>
-      </c>
-      <c r="M46" s="28" t="inlineStr">
-        <is>
-          <t>Go-live sem escopo. O documento não define se a entrada é única ou gradual, nem DNS nem janela. O esperado é o plano de produção, só depois da HML aceita pelos canais.</t>
-        </is>
-      </c>
-      <c r="N46" s="29" t="inlineStr">
-        <is>
-          <t>https://dasa.businessmap.io/ctrl_board/96/cards/451691/details</t>
-        </is>
-      </c>
-      <c r="O46" s="28" t="n">
-        <v>34</v>
       </c>
     </row>
     <row r="47" ht="52" customHeight="1">
@@ -3329,12 +3321,12 @@
       </c>
       <c r="B47" s="30" t="inlineStr">
         <is>
-          <t>Encerrada pela equipe</t>
+          <t>11. Produção — depois da homologação</t>
         </is>
       </c>
       <c r="C47" s="30" t="inlineStr">
         <is>
-          <t>Criação de Workloads do projeto BUSCA -&gt; dp-backend-api</t>
+          <t>[DP] Migração GCP | Cutover &amp; Go-Live</t>
         </is>
       </c>
       <c r="D47" s="30" t="inlineStr">
@@ -3344,204 +3336,314 @@
       </c>
       <c r="E47" s="30" t="inlineStr">
         <is>
-          <t>470119</t>
+          <t>451691</t>
         </is>
       </c>
       <c r="F47" s="30" t="inlineStr">
         <is>
-          <t>Cancelado</t>
+          <t>Sem Definição de Escopo</t>
         </is>
       </c>
       <c r="G47" s="30" t="n"/>
-      <c r="H47" s="30" t="n"/>
+      <c r="H47" s="30" t="inlineStr">
+        <is>
+          <t>??</t>
+        </is>
+      </c>
       <c r="I47" s="30" t="n"/>
       <c r="J47" s="30" t="n"/>
-      <c r="K47" s="30" t="inlineStr">
+      <c r="K47" s="30" t="n"/>
+      <c r="L47" s="30" t="inlineStr">
+        <is>
+          <t>Última linha de produção.</t>
+        </is>
+      </c>
+      <c r="M47" s="30" t="inlineStr">
+        <is>
+          <t>Go-live sem escopo. O documento não define se a entrada é única ou gradual, nem DNS nem janela. O esperado é o plano de produção, só depois da HML aceita pelos canais.</t>
+        </is>
+      </c>
+      <c r="N47" s="31" t="inlineStr">
+        <is>
+          <t>https://dasa.businessmap.io/ctrl_board/96/cards/451691/details</t>
+        </is>
+      </c>
+      <c r="O47" s="30" t="n">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="48" ht="52" customHeight="1">
+      <c r="A48" s="32" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="32" t="inlineStr">
+        <is>
+          <t>Encerrada pela equipe</t>
+        </is>
+      </c>
+      <c r="C48" s="32" t="inlineStr">
+        <is>
+          <t>Criação de Workloads do projeto BUSCA -&gt; dp-corporate-frontend</t>
+        </is>
+      </c>
+      <c r="D48" s="32" t="inlineStr">
+        <is>
+          <t>Card da planilha</t>
+        </is>
+      </c>
+      <c r="E48" s="32" t="inlineStr">
+        <is>
+          <t>470121</t>
+        </is>
+      </c>
+      <c r="F48" s="32" t="inlineStr">
+        <is>
+          <t>Cancelado</t>
+        </is>
+      </c>
+      <c r="G48" s="32" t="n"/>
+      <c r="H48" s="32" t="n"/>
+      <c r="I48" s="32" t="n"/>
+      <c r="J48" s="32" t="n"/>
+      <c r="K48" s="32" t="n"/>
+      <c r="L48" s="32" t="inlineStr">
+        <is>
+          <t>Encerrado como card. O frontend segue na fila de HML.</t>
+        </is>
+      </c>
+      <c r="M48" s="32" t="inlineStr">
+        <is>
+          <t>A equipe cancelou este workload. A linha dp-corporate-frontend na HML cobre a URL que a documentação cita, para o frontend entrar na homologação.</t>
+        </is>
+      </c>
+      <c r="N48" s="33" t="inlineStr">
+        <is>
+          <t>https://dasa.businessmap.io/ctrl_board/96/cards/470121/details</t>
+        </is>
+      </c>
+      <c r="O48" s="32" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="49" ht="52" customHeight="1">
+      <c r="A49" s="32" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="32" t="inlineStr">
+        <is>
+          <t>Encerrada pela equipe</t>
+        </is>
+      </c>
+      <c r="C49" s="32" t="inlineStr">
+        <is>
+          <t>Criação de Workloads do projeto BUSCA -&gt; dp-backend-api</t>
+        </is>
+      </c>
+      <c r="D49" s="32" t="inlineStr">
+        <is>
+          <t>Card da planilha</t>
+        </is>
+      </c>
+      <c r="E49" s="32" t="inlineStr">
+        <is>
+          <t>470119</t>
+        </is>
+      </c>
+      <c r="F49" s="32" t="inlineStr">
+        <is>
+          <t>Cancelado</t>
+        </is>
+      </c>
+      <c r="G49" s="32" t="n"/>
+      <c r="H49" s="32" t="n"/>
+      <c r="I49" s="32" t="n"/>
+      <c r="J49" s="32" t="n"/>
+      <c r="K49" s="32" t="inlineStr">
         <is>
           <t>depende cognitiveSearch</t>
         </is>
       </c>
-      <c r="L47" s="30" t="inlineStr">
+      <c r="L49" s="32" t="inlineStr">
         <is>
           <t>Fora do caminho aberto. O cancelamento não tira a API de exam, que continua atrás do índice.</t>
         </is>
       </c>
-      <c r="M47" s="30" t="inlineStr">
+      <c r="M49" s="32" t="inlineStr">
         <is>
           <t>Cancelado pela equipe, com observação de Cognitive Search. Os backends 469049 e 468966 seguem no caminho. O documento não descreve este card além disso.</t>
         </is>
       </c>
-      <c r="N47" s="31" t="inlineStr">
+      <c r="N49" s="33" t="inlineStr">
         <is>
           <t>https://dasa.businessmap.io/ctrl_board/96/cards/470119/details</t>
         </is>
       </c>
-      <c r="O47" s="30" t="n">
+      <c r="O49" s="32" t="n">
         <v>16</v>
       </c>
     </row>
-    <row r="48" ht="52" customHeight="1">
-      <c r="A48" s="30" t="n">
-        <v>47</v>
-      </c>
-      <c r="B48" s="30" t="inlineStr">
+    <row r="50" ht="52" customHeight="1">
+      <c r="A50" s="32" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="32" t="inlineStr">
         <is>
           <t>Encerrada pela equipe</t>
         </is>
       </c>
-      <c r="C48" s="30" t="inlineStr">
+      <c r="C50" s="32" t="inlineStr">
         <is>
           <t>[DP] Migração GCP | Converter ETL's (DataBricks)</t>
         </is>
       </c>
-      <c r="D48" s="30" t="inlineStr">
+      <c r="D50" s="32" t="inlineStr">
         <is>
           <t>Card da planilha</t>
         </is>
       </c>
-      <c r="E48" s="30" t="inlineStr">
+      <c r="E50" s="32" t="inlineStr">
         <is>
           <t>451674</t>
         </is>
       </c>
-      <c r="F48" s="30" t="inlineStr">
+      <c r="F50" s="32" t="inlineStr">
         <is>
           <t>Cancelado</t>
         </is>
       </c>
-      <c r="G48" s="30" t="n"/>
-      <c r="H48" s="30" t="n"/>
-      <c r="I48" s="30" t="n"/>
-      <c r="J48" s="30" t="n"/>
-      <c r="K48" s="30" t="n"/>
-      <c r="L48" s="30" t="inlineStr">
+      <c r="G50" s="32" t="n"/>
+      <c r="H50" s="32" t="n"/>
+      <c r="I50" s="32" t="n"/>
+      <c r="J50" s="32" t="n"/>
+      <c r="K50" s="32" t="n"/>
+      <c r="L50" s="32" t="inlineStr">
         <is>
           <t>Encerrado. Não volta para o caminho.</t>
         </is>
       </c>
-      <c r="M48" s="30" t="inlineStr">
+      <c r="M50" s="32" t="inlineStr">
         <is>
           <t>Cancelado. A decisão oficial é levar o Databricks, não converter os ETLs para outra ferramenta.</t>
         </is>
       </c>
-      <c r="N48" s="31" t="inlineStr">
+      <c r="N50" s="33" t="inlineStr">
         <is>
           <t>https://dasa.businessmap.io/ctrl_board/96/cards/451674/details</t>
         </is>
       </c>
-      <c r="O48" s="30" t="n">
+      <c r="O50" s="32" t="n">
         <v>38</v>
       </c>
     </row>
-    <row r="49" ht="52" customHeight="1">
-      <c r="A49" s="30" t="n">
-        <v>48</v>
-      </c>
-      <c r="B49" s="30" t="inlineStr">
+    <row r="51" ht="52" customHeight="1">
+      <c r="A51" s="32" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="32" t="inlineStr">
         <is>
           <t>Encerrada pela equipe</t>
         </is>
       </c>
-      <c r="C49" s="30" t="inlineStr">
+      <c r="C51" s="32" t="inlineStr">
         <is>
           <t>[DP] PostgreSQL - Levantamento de recursos para reescrita de código</t>
         </is>
       </c>
-      <c r="D49" s="30" t="inlineStr">
+      <c r="D51" s="32" t="inlineStr">
         <is>
           <t>Card da planilha</t>
         </is>
       </c>
-      <c r="E49" s="30" t="inlineStr">
+      <c r="E51" s="32" t="inlineStr">
         <is>
           <t>424941</t>
         </is>
       </c>
-      <c r="F49" s="30" t="inlineStr">
+      <c r="F51" s="32" t="inlineStr">
         <is>
           <t>Cancelado</t>
         </is>
       </c>
-      <c r="G49" s="30" t="n"/>
-      <c r="H49" s="30" t="n"/>
-      <c r="I49" s="30" t="n"/>
-      <c r="J49" s="30" t="n"/>
-      <c r="K49" s="30" t="n"/>
-      <c r="L49" s="30" t="inlineStr">
+      <c r="G51" s="32" t="n"/>
+      <c r="H51" s="32" t="n"/>
+      <c r="I51" s="32" t="n"/>
+      <c r="J51" s="32" t="n"/>
+      <c r="K51" s="32" t="n"/>
+      <c r="L51" s="32" t="inlineStr">
         <is>
           <t>Encerrado.</t>
         </is>
       </c>
-      <c r="M49" s="30" t="inlineStr">
+      <c r="M51" s="32" t="inlineStr">
         <is>
           <t>Cancelado. Não há reescrita para PostgreSQL neste plano. O banco de HML já foi criado.</t>
         </is>
       </c>
-      <c r="N49" s="31" t="inlineStr">
+      <c r="N51" s="33" t="inlineStr">
         <is>
           <t>https://dasa.businessmap.io/ctrl_board/96/cards/424941/details</t>
         </is>
       </c>
-      <c r="O49" s="30" t="n">
+      <c r="O51" s="32" t="n">
         <v>42</v>
       </c>
     </row>
-    <row r="50" ht="52" customHeight="1">
-      <c r="A50" s="30" t="n">
-        <v>49</v>
-      </c>
-      <c r="B50" s="30" t="inlineStr">
+    <row r="52" ht="52" customHeight="1">
+      <c r="A52" s="32" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" s="32" t="inlineStr">
         <is>
           <t>Encerrada pela equipe</t>
         </is>
       </c>
-      <c r="C50" s="30" t="inlineStr">
+      <c r="C52" s="32" t="inlineStr">
         <is>
           <t>[DP] Migração GCP | Migrar banco de dados SQL Server -- ABORTADO</t>
         </is>
       </c>
-      <c r="D50" s="30" t="inlineStr">
+      <c r="D52" s="32" t="inlineStr">
         <is>
           <t>Card da planilha</t>
         </is>
       </c>
-      <c r="E50" s="30" t="inlineStr">
+      <c r="E52" s="32" t="inlineStr">
         <is>
           <t>451676</t>
         </is>
       </c>
-      <c r="F50" s="30" t="inlineStr">
+      <c r="F52" s="32" t="inlineStr">
         <is>
           <t>Concluído</t>
         </is>
       </c>
-      <c r="G50" s="30" t="n"/>
-      <c r="H50" s="30" t="n"/>
-      <c r="I50" s="30" t="n"/>
-      <c r="J50" s="30" t="n"/>
-      <c r="K50" s="30" t="n"/>
-      <c r="L50" s="30" t="inlineStr">
+      <c r="G52" s="32" t="n"/>
+      <c r="H52" s="32" t="n"/>
+      <c r="I52" s="32" t="n"/>
+      <c r="J52" s="32" t="n"/>
+      <c r="K52" s="32" t="n"/>
+      <c r="L52" s="32" t="inlineStr">
         <is>
           <t>Encerrado. A carga de HML cobre o que as APIs precisam ler.</t>
         </is>
       </c>
-      <c r="M50" s="30" t="inlineStr">
+      <c r="M52" s="32" t="inlineStr">
         <is>
           <t>Abortado e concluído. O SQL Server não é copiado. A documentação diz que a réplica 3 não migra e está desligada. O dado segue pela carga no banco já criado.</t>
         </is>
       </c>
-      <c r="N50" s="31" t="inlineStr">
+      <c r="N52" s="33" t="inlineStr">
         <is>
           <t>https://dasa.businessmap.io/ctrl_board/96/cards/451676/details</t>
         </is>
       </c>
-      <c r="O50" s="30" t="n">
+      <c r="O52" s="32" t="n">
         <v>37</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O50">
-    <sortState ref="A1:O50">
+  <autoFilter ref="A1:O52">
+    <sortState ref="A1:O52">
       <sortCondition descending="0" ref="A2:A200"/>
     </sortState>
   </autoFilter>
@@ -3557,10 +3659,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N12" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N13" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N14" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N16" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N17" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N18" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N19" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N15" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N16" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N17" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N18" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N20" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N21" r:id="rId17"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N22" r:id="rId18"/>
@@ -3570,19 +3672,20 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N32" r:id="rId22"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N33" r:id="rId23"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N34" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N35" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N36" r:id="rId25"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N39" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N40" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N41" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N42" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N43" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N44" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N45" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N46" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N47" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N48" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N49" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N50" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N41" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N42" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N43" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N44" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N45" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N46" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N47" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N48" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N49" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N50" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N51" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N52" r:id="rId38"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.6" bottom="0.6" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" scale="70" fitToHeight="0" fitToWidth="1"/>
@@ -3603,7 +3706,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3683,180 +3786,142 @@
       </c>
     </row>
     <row r="2" ht="60" customHeight="1">
-      <c r="A2" s="32" t="n">
+      <c r="A2" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="32" t="inlineStr">
+      <c r="B2" s="34" t="inlineStr">
         <is>
           <t>BigQuery =&gt; substituir dataBricks</t>
         </is>
       </c>
-      <c r="C2" s="32" t="inlineStr">
+      <c r="C2" s="34" t="inlineStr">
         <is>
           <t>478328</t>
         </is>
       </c>
-      <c r="D2" s="32" t="n"/>
-      <c r="E2" s="32" t="inlineStr">
+      <c r="D2" s="34" t="n"/>
+      <c r="E2" s="34" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="F2" s="32" t="inlineStr">
+      <c r="F2" s="34" t="inlineStr">
         <is>
           <t>Galerinha de dados DP</t>
         </is>
       </c>
-      <c r="G2" s="32" t="inlineStr">
+      <c r="G2" s="34" t="inlineStr">
         <is>
           <t>29/01/27</t>
         </is>
       </c>
-      <c r="H2" s="32" t="inlineStr">
+      <c r="H2" s="34" t="inlineStr">
         <is>
           <t>Dados</t>
         </is>
       </c>
-      <c r="I2" s="32" t="inlineStr">
+      <c r="I2" s="34" t="inlineStr">
         <is>
           <t>Levar toda a orquestração do dataBricks para o BigQuery</t>
         </is>
       </c>
-      <c r="J2" s="32" t="inlineStr">
+      <c r="J2" s="34" t="inlineStr">
         <is>
           <t>A equipe pediu levar a orquestração do Databricks para o BigQuery. O diagrama AS IS não passa pelo Databricks até as APIs. A ida para a GCP não exige essa troca: a decisão deste plano é levar os workspaces, e o card de converter os ETLs já está cancelado. O desenho com bronze, silver e gold está no documento sem a estratégia preenchida.</t>
         </is>
       </c>
-      <c r="K2" s="33" t="inlineStr">
+      <c r="K2" s="35" t="inlineStr">
         <is>
           <t>https://dasa.businessmap.io/ctrl_board/96/cards/478328/details</t>
         </is>
       </c>
-      <c r="L2" s="32" t="n">
+      <c r="L2" s="34" t="n">
         <v>9</v>
       </c>
     </row>
     <row r="3" ht="60" customHeight="1">
-      <c r="A3" s="32" t="n">
+      <c r="A3" s="34" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="32" t="inlineStr">
+      <c r="B3" s="34" t="inlineStr">
         <is>
           <t>[DATP] DasaLogs -&gt; api local - unidades</t>
         </is>
       </c>
-      <c r="C3" s="32" t="inlineStr">
+      <c r="C3" s="34" t="inlineStr">
         <is>
           <t>476063</t>
         </is>
       </c>
-      <c r="D3" s="32" t="inlineStr">
+      <c r="D3" s="34" t="inlineStr">
         <is>
           <t>Stand By</t>
         </is>
       </c>
-      <c r="E3" s="32" t="n"/>
-      <c r="F3" s="32" t="n"/>
-      <c r="G3" s="32" t="n"/>
-      <c r="H3" s="32" t="n"/>
-      <c r="I3" s="32" t="n"/>
-      <c r="J3" s="32" t="inlineStr">
+      <c r="E3" s="34" t="n"/>
+      <c r="F3" s="34" t="n"/>
+      <c r="G3" s="34" t="n"/>
+      <c r="H3" s="34" t="n"/>
+      <c r="I3" s="34" t="n"/>
+      <c r="J3" s="34" t="inlineStr">
         <is>
           <t>A equipe deixou em stand-by. O documento de arquitetura não cita DasaLogs no caminho de exame, unidade e convênio, nem nas APIs, no Airflow ou na busca.</t>
         </is>
       </c>
-      <c r="K3" s="33" t="inlineStr">
+      <c r="K3" s="35" t="inlineStr">
         <is>
           <t>https://dasa.businessmap.io/ctrl_board/96/cards/476063/details</t>
         </is>
       </c>
-      <c r="L3" s="32" t="n">
+      <c r="L3" s="34" t="n">
         <v>33</v>
       </c>
     </row>
     <row r="4" ht="60" customHeight="1">
-      <c r="A4" s="32" t="n">
+      <c r="A4" s="34" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="32" t="inlineStr">
-        <is>
-          <t>Criação de Workloads do projeto BUSCA -&gt; dp-corporate-frontend</t>
-        </is>
-      </c>
-      <c r="C4" s="32" t="inlineStr">
-        <is>
-          <t>470121</t>
-        </is>
-      </c>
-      <c r="D4" s="32" t="inlineStr">
+      <c r="B4" s="34" t="inlineStr">
+        <is>
+          <t>Criação de Workloads do projeto PORTAL-CADASTRO -&gt; datp-backoffice-frontend-portal</t>
+        </is>
+      </c>
+      <c r="C4" s="34" t="inlineStr">
+        <is>
+          <t>468985</t>
+        </is>
+      </c>
+      <c r="D4" s="34" t="inlineStr">
         <is>
           <t>Cancelado</t>
         </is>
       </c>
-      <c r="E4" s="32" t="n"/>
-      <c r="F4" s="32" t="n"/>
-      <c r="G4" s="32" t="n"/>
-      <c r="H4" s="32" t="n"/>
-      <c r="I4" s="32" t="n"/>
-      <c r="J4" s="32" t="inlineStr">
-        <is>
-          <t>A equipe cancelou o workload dp-corporate-frontend. A documentação ainda aponta essa URL como frontend do DP. O card 469051 segue no caminho com outro nome. Os dois não foram tratados como o mesmo frontend.</t>
-        </is>
-      </c>
-      <c r="K4" s="33" t="inlineStr">
-        <is>
-          <t>https://dasa.businessmap.io/ctrl_board/96/cards/470121/details</t>
-        </is>
-      </c>
-      <c r="L4" s="32" t="n">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="5" ht="60" customHeight="1">
-      <c r="A5" s="32" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" s="32" t="inlineStr">
-        <is>
-          <t>Criação de Workloads do projeto PORTAL-CADASTRO -&gt; datp-backoffice-frontend-portal</t>
-        </is>
-      </c>
-      <c r="C5" s="32" t="inlineStr">
-        <is>
-          <t>468985</t>
-        </is>
-      </c>
-      <c r="D5" s="32" t="inlineStr">
-        <is>
-          <t>Cancelado</t>
-        </is>
-      </c>
-      <c r="E5" s="32" t="n"/>
-      <c r="F5" s="32" t="n"/>
-      <c r="G5" s="32" t="n"/>
-      <c r="H5" s="32" t="n"/>
-      <c r="I5" s="32" t="inlineStr">
+      <c r="E4" s="34" t="n"/>
+      <c r="F4" s="34" t="n"/>
+      <c r="G4" s="34" t="n"/>
+      <c r="H4" s="34" t="n"/>
+      <c r="I4" s="34" t="inlineStr">
         <is>
           <t>depende do airFlow</t>
         </is>
       </c>
-      <c r="J5" s="32" t="inlineStr">
+      <c r="J4" s="34" t="inlineStr">
         <is>
           <t>A equipe cancelou o workload do repositório datp-backoffice-frontend-portal. A documentação cita esse repositório como frontend do portal de cadastro. Os cards 470165 e 451677 seguem no caminho com outros nomes.</t>
         </is>
       </c>
-      <c r="K5" s="33" t="inlineStr">
+      <c r="K4" s="35" t="inlineStr">
         <is>
           <t>https://dasa.businessmap.io/ctrl_board/96/cards/468985/details</t>
         </is>
       </c>
-      <c r="L5" s="32" t="n">
+      <c r="L4" s="34" t="n">
         <v>20</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L5">
-    <sortState ref="A1:L5">
+  <autoFilter ref="A1:L4">
+    <sortState ref="A1:L4">
       <sortCondition descending="0" ref="A2:A200"/>
     </sortState>
   </autoFilter>
@@ -3864,7 +3929,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K3" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K5" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.6" bottom="0.6" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" scale="70" fitToHeight="0" fitToWidth="1"/>
@@ -3892,63 +3956,63 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="34" t="inlineStr">
+      <c r="A1" s="36" t="inlineStr">
         <is>
           <t>Como a aba foi ordenada</t>
         </is>
       </c>
     </row>
     <row r="3" ht="48" customHeight="1">
-      <c r="A3" s="35" t="inlineStr">
+      <c r="A3" s="37" t="inlineStr">
         <is>
           <t>A ordem segue dependência e arquitetura. A coluna Cronograma original guarda a data da planilha e não foi usada para ordenar. Várias datas se contradizem: portal e Blob em fevereiro de 2027, adequação do Airflow em março–abril de 2027, Airflow com nome prd em 09/10/26.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="48" customHeight="1">
-      <c r="A4" s="35" t="inlineStr">
-        <is>
-          <t>O teste funcional (card 451689) e o teste de carga fecham o que a HML precisa para testar. A linha de Databricks na GCP fica depois desse teste e antes da produção, e não bloqueia o teste. O único cluster concluído é o GKE de HML.</t>
+      <c r="A4" s="37" t="inlineStr">
+        <is>
+          <t>Todos os componentes da HML entram antes dos testes, Databricks e Event Hub incluídos. O teste funcional prova o uso pelo NAV, pelo CDC e pelo portal. O teste de carga vem em seguida. O card 451689 fecha a homologação e o rollback. Produção só começa depois. A planilha trata elegibility como uma API. A carga do Corporate é card do TIE. A busca é POC, como a spike de versão do Airflow.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="48" customHeight="1">
-      <c r="A5" s="35" t="inlineStr">
+      <c r="A5" s="37" t="inlineStr">
         <is>
           <t>A passagem do Data Factory para o Airflow não entra nesta aba. Está concluída e é pré-requisito de outro projeto. O Airflow de partida está na Azure. Nesta lista a frente é migrar esse Airflow para a GCP: primeiro a spike, por causa da versão 2.2.5, depois a adequação. Carga, Blob e portal esperam essa migração. As APIs que não citam Airflow nem Cognitive Search não esperam.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="48" customHeight="1">
-      <c r="A6" s="35" t="inlineStr">
+      <c r="A6" s="37" t="inlineStr">
         <is>
           <t>Exam fica depois do índice. As outras APIs não foram colocadas atrás do índice: só a exam e o dp-backend-api cancelado citam Cognitive Search. O diagrama desenha busca-search na frente do conjunto de APIs, e essa diferença está na aba Dúvidas.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="48" customHeight="1">
-      <c r="A7" s="35" t="inlineStr">
+      <c r="A7" s="37" t="inlineStr">
         <is>
           <t>Lacuna só entra quando a documentação nomeia o componente ou quando um card cita a dependência e não existe card para ela. Lacuna não tem Card ID, responsável, complexidade nem prazo.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="48" customHeight="1">
-      <c r="A8" s="35" t="inlineStr">
+      <c r="A8" s="37" t="inlineStr">
         <is>
           <t>A coluna Origem fica 'IA' quando a linha não tinha card. A base explica o que se espera e a coluna ao lado das observações diz por que a linha está naquele ponto. Essas linhas não têm responsável, prazo nem Card ID. Origem 'Card da planilha' é atividade da equipe.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="48" customHeight="1">
-      <c r="A9" s="35" t="inlineStr">
+      <c r="A9" s="37" t="inlineStr">
         <is>
           <t>O card de BigQuery no lugar do Databricks, o DasaLogs, o frontend dp-corporate-frontend e o repositório datp-backoffice-frontend-portal foram para a aba Discutir com a equipe. São itens da planilha que não se sustentam neste caminho.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="48" customHeight="1">
-      <c r="A10" s="35" t="inlineStr">
+      <c r="A10" s="37" t="inlineStr">
         <is>
           <t>Cards cancelados ou abortados que não entram nessa discussão ficam no fim, na etapa Encerrada pela equipe. O status deles sai da coluna Complexidade.</t>
         </is>
@@ -3974,7 +4038,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4000,212 +4064,178 @@
       </c>
     </row>
     <row r="2" ht="48" customHeight="1">
-      <c r="A2" s="36" t="inlineStr">
+      <c r="A2" s="38" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B2" s="36" t="inlineStr">
+      <c r="B2" s="38" t="inlineStr">
         <is>
           <t>O banco criado no card 451661 já tem, em HML, exame, unidade e convênio?</t>
         </is>
       </c>
-      <c r="C2" s="36" t="inlineStr">
-        <is>
-          <t>Se já tiver, a lacuna de carga sai da frente do teste funcional. Se não tiver, ela continua depois da migração do Airflow da Azure para a GCP. A migração do SQL Server está abortada.</t>
+      <c r="C2" s="38" t="inlineStr">
+        <is>
+          <t>O card da migração da carga do Corporate é do TIE e fica antes dos testes. Se o banco já tiver esses dados, o card do TIE fecha sem nova carga.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="48" customHeight="1">
-      <c r="A3" s="36" t="inlineStr">
+      <c r="A3" s="38" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B3" s="36" t="inlineStr">
+      <c r="B3" s="38" t="inlineStr">
         <is>
           <t>Quais APIs leem o Cognitive Search além da exam?</t>
         </is>
       </c>
-      <c r="C3" s="36" t="inlineStr">
-        <is>
-          <t>O diagrama coloca busca-search na frente das APIs. A planilha só trava a exam e o dp-backend-api cancelado. Se brand, local, health insurance, elegibility ou commons leem o índice, elas saem da etapa 3 e vão para depois do card 451682.</t>
+      <c r="C3" s="38" t="inlineStr">
+        <is>
+          <t>A busca é uma POC, como a spike de versão. A planilha só trava a exam. Se outra API lê o índice, ela sobe para depois da POC.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="48" customHeight="1">
-      <c r="A4" s="36" t="inlineStr">
+      <c r="A4" s="38" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="B4" s="36" t="inlineStr">
+      <c r="B4" s="38" t="inlineStr">
         <is>
           <t>O que o Databricks de HML entrega para a API ou para o portal?</t>
         </is>
       </c>
-      <c r="C4" s="36" t="inlineStr">
-        <is>
-          <t>A linha dos workspaces foi inclusa por gap e ficou depois do teste funcional, porque o diagrama até as APIs não passa pelo Databricks. Se a API ou o portal consomem a saída, ela sobe para antes do card 451689.</t>
+      <c r="C4" s="38" t="inlineStr">
+        <is>
+          <t>O Databricks entra na HML antes dos testes, para poder ser homologado. A documentação não lista jobs. Falta saber o que a homologação precisa ver rodando.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="48" customHeight="1">
-      <c r="A5" s="36" t="inlineStr">
+      <c r="A5" s="38" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="B5" s="36" t="inlineStr">
-        <is>
-          <t>datp-searcher-api-elegibility é a API de agendamento do documento?</t>
-        </is>
-      </c>
-      <c r="C5" s="36" t="inlineStr">
-        <is>
-          <t>O documento lista agendamento entre as seis APIs. O diagrama nomeia busca-agendamento-backend. A planilha tem elegibility e não tem card chamado agendamento. Se forem duas APIs, falta o workload de agendamento.</t>
+      <c r="B5" s="38" t="inlineStr">
+        <is>
+          <t>O card 469051 é o mesmo frontend da URL dp-corporate-frontend?</t>
+        </is>
+      </c>
+      <c r="C5" s="38" t="inlineStr">
+        <is>
+          <t>A documentação cita a URL e a planilha tem o card 469051 no caminho. O workload 470121 foi cancelado e a linha dp-corporate-frontend existe para a homologação. Se forem o mesmo frontend, as duas linhas viram uma.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="48" customHeight="1">
-      <c r="A6" s="36" t="inlineStr">
+      <c r="A6" s="38" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="B6" s="36" t="inlineStr">
-        <is>
-          <t>O card cancelado dp-corporate-frontend (470121) é o mesmo frontend do card 469051?</t>
-        </is>
-      </c>
-      <c r="C6" s="36" t="inlineStr">
-        <is>
-          <t>A documentação cita a URL dp-corporate-frontend e o repositório datp-backoffice-frontend. Um card está cancelado e o outro está na fila de HML. Sem essa resposta os dois não foram unidos.</t>
+      <c r="B6" s="38" t="inlineStr">
+        <is>
+          <t>O download D+1 de cadastro lê o Blob?</t>
+        </is>
+      </c>
+      <c r="C6" s="38" t="inlineStr">
+        <is>
+          <t>O Blob depende de Airflow, backend e frontend. O portal depende de Airflow, cargas de cadastro e D+1. A planilha não liga um ao outro. Se o D+1 ler o Blob, o card 451688 fica antes das cargas.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="48" customHeight="1">
-      <c r="A7" s="36" t="inlineStr">
+      <c r="A7" s="38" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="B7" s="36" t="inlineStr">
-        <is>
-          <t>O download D+1 de cadastro lê o Blob?</t>
-        </is>
-      </c>
-      <c r="C7" s="36" t="inlineStr">
-        <is>
-          <t>O Blob depende de Airflow, backend e frontend. O portal depende de Airflow, cargas de cadastro e D+1. A planilha não liga um ao outro. Se o D+1 ler o Blob, o card 451688 fica antes das cargas.</t>
+      <c r="B7" s="38" t="inlineStr">
+        <is>
+          <t>A conectividade do card 424949 inclui as fontes do diagrama?</t>
+        </is>
+      </c>
+      <c r="C7" s="38" t="inlineStr">
+        <is>
+          <t>K2/Gliese, base federada, MDM, GSC, hospitais e MV estão no desenho. A seção de rede do documento está vazia. Há uma linha de fontes antes da carga do TIE. Se o 424949 já cobre essas fontes, a linha se junta a ele.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="48" customHeight="1">
-      <c r="A8" s="36" t="inlineStr">
+      <c r="A8" s="38" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="B8" s="36" t="inlineStr">
-        <is>
-          <t>A conectividade do card 424949 inclui as fontes do diagrama?</t>
-        </is>
-      </c>
-      <c r="C8" s="36" t="inlineStr">
-        <is>
-          <t>K2/Gliese, base federada, MDM, GSC, hospitais e MV estão no desenho. A seção de rede do documento está vazia. O texto dos workloads fala só do IP da aplicação. Se as fontes forem outro trabalho, falta uma atividade antes da carga.</t>
+      <c r="B8" s="38" t="inlineStr">
+        <is>
+          <t>O que entra no teste de carga?</t>
+        </is>
+      </c>
+      <c r="C8" s="38" t="inlineStr">
+        <is>
+          <t>A linha existe, depois do teste funcional. O documento não traz volume, API nem meta.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="48" customHeight="1">
-      <c r="A9" s="36" t="inlineStr">
+      <c r="A9" s="38" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="B9" s="36" t="inlineStr">
-        <is>
-          <t>No teste de HML a autenticação continua como está?</t>
-        </is>
-      </c>
-      <c r="C9" s="36" t="inlineStr">
-        <is>
-          <t>O documento marca Azure AD como dependência interna que não pode ser desacoplada. Frontend do DP usa AD, portal usa SSO, APIs usam API key. O template GCP escreve Azure AD para Google IAM e não foi preenchido. Nenhuma atividade de identidade foi criada.</t>
+      <c r="B9" s="38" t="inlineStr">
+        <is>
+          <t>dp-api-gtw e dp-cad-proxy entram nesta migração?</t>
+        </is>
+      </c>
+      <c r="C9" s="38" t="inlineStr">
+        <is>
+          <t>Estão no diagrama e têm linha na fila das APIs, para poderem ser homologados. Não há card. O Zuul tem card próprio.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="48" customHeight="1">
-      <c r="A10" s="36" t="inlineStr">
+      <c r="A10" s="38" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="B10" s="36" t="inlineStr">
-        <is>
-          <t>O que entra no teste de carga?</t>
-        </is>
-      </c>
-      <c r="C10" s="36" t="inlineStr">
-        <is>
-          <t>Não há card, volume, API nem meta. O template do documento cita Performance sem conteúdo. A linha está depois do teste funcional e antes da produção, sem cenário.</t>
+      <c r="B10" s="38" t="inlineStr">
+        <is>
+          <t>O staging SQL ainda faz parte do caminho em HML?</t>
+        </is>
+      </c>
+      <c r="C10" s="38" t="inlineStr">
+        <is>
+          <t>STAGING_PRD está na documentação e há uma linha antes da carga. Não há card. Se o staging saiu do caminho, a linha sai.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="48" customHeight="1">
-      <c r="A11" s="36" t="inlineStr">
+      <c r="A11" s="38" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="B11" s="36" t="inlineStr">
-        <is>
-          <t>dp-api-gtw e dp-cad-proxy entram nesta migração?</t>
-        </is>
-      </c>
-      <c r="C11" s="36" t="inlineStr">
-        <is>
-          <t>Estão no diagrama AS IS e não têm card. Ficaram fora do caminho. O Zuul tem card próprio.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="48" customHeight="1">
-      <c r="A12" s="36" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="B12" s="36" t="inlineStr">
-        <is>
-          <t>O staging SQL ainda faz parte do caminho em HML?</t>
-        </is>
-      </c>
-      <c r="C12" s="36" t="inlineStr">
-        <is>
-          <t>STAGING_PRD está na documentação e não há card. Ficou fora do caminho.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="48" customHeight="1">
-      <c r="A13" s="36" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="B13" s="36" t="inlineStr">
-        <is>
-          <t>Event Hub entra no teste funcional de algum canal?</t>
-        </is>
-      </c>
-      <c r="C13" s="36" t="inlineStr">
-        <is>
-          <t>O card manda deixar por último e nenhuma API o cita. Ele está no fim da produção. Se NAV ou CDC dependem do evento para o teste de HML, ele sobe para antes do card 451689.</t>
+      <c r="B11" s="38" t="inlineStr">
+        <is>
+          <t>Qual canal precisa do Event Hub no teste funcional?</t>
+        </is>
+      </c>
+      <c r="C11" s="38" t="inlineStr">
+        <is>
+          <t>O Event Hub entra na HML antes dos testes, para poder ser homologado. Nenhuma API cita o evento. Falta o canal que prova essa troca.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C13">
-    <sortState ref="A1:C13">
+  <autoFilter ref="A1:C11">
+    <sortState ref="A1:C11">
       <sortCondition descending="0" ref="A2:A200"/>
     </sortState>
   </autoFilter>

</xml_diff>

<commit_message>
Encurta a coluna Base para o fato que sustenta cada linha.
Cada célula afirma o que a planilha ou a documentação já estabelece, sem ressalva nem texto de expectativa.

Co-authored-by: waneron <waneron@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/BM-GCP-Atividades-DP-ordem-temporal.xlsx
+++ b/BM-GCP-Atividades-DP-ordem-temporal.xlsx
@@ -791,7 +791,7 @@
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>Homologação já tem cluster GKE. É aqui que as APIs sobem para o NAV e o CDC experimentarem antes da produção.</t>
+          <t>Cluster GKE de HML provisionado.</t>
         </is>
       </c>
       <c r="N2" s="3" t="inlineStr">
@@ -844,7 +844,7 @@
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>O banco de homologação já foi criado. A migração do SQL Server foi abortada, então este banco é o que as APIs vão ler no lugar do Corporate.</t>
+          <t>Banco de HML criado. As APIs leem este banco.</t>
         </is>
       </c>
       <c r="N3" s="3" t="inlineStr">
@@ -905,7 +905,7 @@
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>O Redis já foi migrado. No diagrama ele é o busca-cache, entre o Corporate e as APIs. O teste deste cache espera os pods no ar.</t>
+          <t>Redis migrado. No diagrama é o busca-cache.</t>
         </is>
       </c>
       <c r="N4" s="3" t="inlineStr">
@@ -958,7 +958,7 @@
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>A continuação do workload da API commons já foi concluída. O card 470112, da criação, ainda está em andamento.</t>
+          <t>Continuação do workload da API commons concluída. A criação segue no card 470112.</t>
         </is>
       </c>
       <c r="N5" s="3" t="inlineStr">
@@ -1007,7 +1007,7 @@
       </c>
       <c r="M6" s="4" t="inlineStr">
         <is>
-          <t>Os workloads registram que a conectividade por IP está errada. O esperado é um endereço de homologação que o NAV e o CDC consigam chamar.</t>
+          <t>Conectividade por IP está errada. HML usa endereço que NAV e CDC chamam.</t>
         </is>
       </c>
       <c r="N6" s="5" t="inlineStr">
@@ -1052,7 +1052,7 @@
       </c>
       <c r="M7" s="6" t="inlineStr">
         <is>
-          <t>O documento diz que o Azure AD não pode ser desacoplado. As APIs usam API key, o frontend do DP usa AD e o portal usa SSO. O esperado é a HML aceitar esse mesmo acesso.</t>
+          <t>Azure AD permanece. APIs usam API key, o frontend do DP usa AD e o portal usa SSO.</t>
         </is>
       </c>
       <c r="N7" s="6" t="n"/>
@@ -1111,7 +1111,7 @@
       </c>
       <c r="M8" s="4" t="inlineStr">
         <is>
-          <t>A esteira precisa publicar no GKE de homologação. Nenhum workload cita este card como bloqueio.</t>
+          <t>A esteira publica no GKE de HML.</t>
         </is>
       </c>
       <c r="N8" s="5" t="inlineStr">
@@ -1176,7 +1176,7 @@
       </c>
       <c r="M9" s="8" t="inlineStr">
         <is>
-          <t>API de brand, uma das consultas do documento. O esperado é ela responder em HML sem depender de Airflow nem de busca.</t>
+          <t>API de brand. Consulta direta, sem Airflow e sem busca.</t>
         </is>
       </c>
       <c r="N9" s="9" t="inlineStr">
@@ -1241,7 +1241,7 @@
       </c>
       <c r="M10" s="8" t="inlineStr">
         <is>
-          <t>Gateway Zuul. No diagrama ele fica na entrada, com autorização, limite de taxa e WAF. O esperado é o NAV e o CDC entrarem por aqui.</t>
+          <t>Gateway Zuul na entrada: autorização, limite de taxa e WAF. NAV e CDC entram por aqui.</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
@@ -1286,7 +1286,7 @@
       </c>
       <c r="M11" s="10" t="inlineStr">
         <is>
-          <t>O diagrama AS IS nomeia dp-api-gtw e dp-cad-proxy e não há card. O esperado é decidir se o Zuul já cobre os dois ou se cada um precisa de workload em HML.</t>
+          <t>dp-api-gtw e dp-cad-proxy estão no diagrama AS IS e sobem na HML.</t>
         </is>
       </c>
       <c r="N11" s="10" t="n"/>
@@ -1345,7 +1345,7 @@
       </c>
       <c r="M12" s="8" t="inlineStr">
         <is>
-          <t>API de local, a consulta de unidade. O esperado é o canal consultar unidade na HML, sem Airflow e sem índice de busca.</t>
+          <t>API de unidade. Consulta direta.</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
@@ -1410,7 +1410,7 @@
       </c>
       <c r="M13" s="8" t="inlineStr">
         <is>
-          <t>API de convênio. O esperado é o canal consultar convênio na HML.</t>
+          <t>API de convênio. Consulta direta.</t>
         </is>
       </c>
       <c r="N13" s="9" t="inlineStr">
@@ -1475,7 +1475,7 @@
       </c>
       <c r="M14" s="8" t="inlineStr">
         <is>
-          <t>A planilha tem um card, datp-searcher-api-elegibility. É uma API. O esperado é esse workload no ar em HML, com as consultas que não citam busca.</t>
+          <t>API de elegibility da planilha. Uma API.</t>
         </is>
       </c>
       <c r="N14" s="9" t="inlineStr">
@@ -1540,7 +1540,7 @@
       </c>
       <c r="M15" s="8" t="inlineStr">
         <is>
-          <t>API commons. A continuação 476416 está concluída e este card segue em andamento. O esperado é ela no ar com as outras.</t>
+          <t>API commons em andamento. A continuação 476416 está concluída.</t>
         </is>
       </c>
       <c r="N15" s="9" t="inlineStr">
@@ -1605,7 +1605,7 @@
       </c>
       <c r="M16" s="8" t="inlineStr">
         <is>
-          <t>Teste de conectividade das APIs, não teste funcional. O esperado é confirmar que a aplicação enxerga o destino novo, ainda sem exigir o dado completo.</t>
+          <t>Teste de conectividade das APIs. Confirma que a aplicação enxerga o destino de HML.</t>
         </is>
       </c>
       <c r="N16" s="9" t="inlineStr">
@@ -1666,7 +1666,7 @@
       </c>
       <c r="M17" s="8" t="inlineStr">
         <is>
-          <t>Backend do frontend do DP, repositório datp-backoffice-backend. O esperado é o backoffice responder em HML. Não cita Airflow.</t>
+          <t>Backend do frontend do DP, repositório datp-backoffice-backend.</t>
         </is>
       </c>
       <c r="N17" s="9" t="inlineStr">
@@ -1726,12 +1726,12 @@
       </c>
       <c r="L18" s="8" t="inlineStr">
         <is>
-          <t>A adaptação entra aqui. O teste da tela é o card 451689.</t>
+          <t>Com os frontends do DP, antes dos testes.</t>
         </is>
       </c>
       <c r="M18" s="8" t="inlineStr">
         <is>
-          <t>Frontend do DP. A documentação cita a URL dp-corporate-frontend; o workload com esse nome está cancelado e ficou para discussão. O esperado é esta adaptação ser a tela aberta em HML, testada só com tudo integrado.</t>
+          <t>Adaptação do frontend do DP. Sobe na HML.</t>
         </is>
       </c>
       <c r="N18" s="9" t="inlineStr">
@@ -1776,7 +1776,7 @@
       </c>
       <c r="M19" s="10" t="inlineStr">
         <is>
-          <t>A documentação cita a URL dp-corporate-frontend. O workload 470121 foi cancelado pela equipe. O esperado é este frontend estar na HML para ser homologado.</t>
+          <t>A documentação cita a URL dp-corporate-frontend. Este frontend sobe na HML.</t>
         </is>
       </c>
       <c r="N19" s="10" t="n"/>
@@ -1839,7 +1839,7 @@
       </c>
       <c r="M20" s="12" t="inlineStr">
         <is>
-          <t>O Airflow já está na Azure. Esta spike, em docker local, acha o que quebra da versão 2.2.5 para a versão do Google. O esperado é a lista de incompatibilidades antes de migrar.</t>
+          <t>Spike local do Airflow 2.2.5 para a versão do Google. Lista as incompatibilidades.</t>
         </is>
       </c>
       <c r="N20" s="13" t="inlineStr">
@@ -1900,7 +1900,7 @@
       </c>
       <c r="M21" s="14" t="inlineStr">
         <is>
-          <t>A busca entra como POC, no mesmo espírito da spike de versão do Airflow. O card está em descoberta e é o maior risco. O esperado é saber o que quebra ao sair do Cognitive Search antes de homologar a API de exam.</t>
+          <t>POC de busca, no mesmo espírito da spike de versão do Airflow. Maior risco, em descoberta.</t>
         </is>
       </c>
       <c r="N21" s="15" t="inlineStr">
@@ -1965,7 +1965,7 @@
       </c>
       <c r="M22" s="14" t="inlineStr">
         <is>
-          <t>API de exam. Depende da busca. O esperado é o workload no ar depois da POC, para a homologação incluir a consulta de exame.</t>
+          <t>API de exam. Depende da busca.</t>
         </is>
       </c>
       <c r="N22" s="15" t="inlineStr">
@@ -2022,7 +2022,7 @@
       </c>
       <c r="M23" s="12" t="inlineStr">
         <is>
-          <t>É a ida do Airflow da Azure para a GCP, por causa da versão. Não tem Card ID. Portal, Blob e backoffice dependem desse Airflow já na GCP. Os workloads com prd no nome ficam na produção.</t>
+          <t>Migração do Airflow da Azure para a GCP. Portal, Blob e backoffice dependem deste Airflow.</t>
         </is>
       </c>
       <c r="N23" s="12" t="n"/>
@@ -2063,7 +2063,7 @@
       </c>
       <c r="M24" s="16" t="inlineStr">
         <is>
-          <t>O diagrama lê K2/Gliese, base federada, MDM, GSC, hospitais e MV. O card 424949 não cita essas fontes. O esperado é o Airflow na GCP alcançar as mesmas origens que hoje alimentam o Corporate.</t>
+          <t>Airflow na GCP alcança K2/Gliese, base federada, MDM, GSC, hospitais e MV.</t>
         </is>
       </c>
       <c r="N24" s="16" t="n"/>
@@ -2102,7 +2102,7 @@
       </c>
       <c r="M25" s="16" t="inlineStr">
         <is>
-          <t>A documentação lista o banco STAGING_PRD, 2 vCores, no caminho até o Corporate. O esperado é saber se o Airflow que vai à GCP ainda grava nesse staging. Se não gravar, a linha sai.</t>
+          <t>STAGING_PRD está no caminho até o Corporate. O Airflow na GCP grava nesse staging.</t>
         </is>
       </c>
       <c r="N25" s="16" t="n"/>
@@ -2145,7 +2145,7 @@
       </c>
       <c r="M26" s="16" t="inlineStr">
         <is>
-          <t>Card a criar, responsabilidade do TIE. O banco de HML existe e a cópia do SQL Server foi abortada. O esperado é o TIE migrar a carga do Corporate para esse banco, com exame, unidade e convênio.</t>
+          <t>TIE migra exame, unidade e convênio do Corporate para o banco de HML.</t>
         </is>
       </c>
       <c r="N26" s="16" t="n"/>
@@ -2204,7 +2204,7 @@
       </c>
       <c r="M27" s="18" t="inlineStr">
         <is>
-          <t>Há 269 GB de Blob. A adaptação depende de Airflow, backend e frontend. O esperado é a aplicação ler o arquivo na GCP.</t>
+          <t>269 GB de Blob. A aplicação lê o arquivo na GCP. Depende de Airflow, backend e frontend.</t>
         </is>
       </c>
       <c r="N27" s="19" t="inlineStr">
@@ -2249,7 +2249,7 @@
       </c>
       <c r="M28" s="16" t="inlineStr">
         <is>
-          <t>Os cards 470165 e 470100 dependem das cargas de cadastro e não existe card só para elas. O diagrama tem o Portal de Cadastros. O esperado é a carga rodar no Airflow da GCP antes do portal abrir.</t>
+          <t>Cards 470165 e 470100 dependem das cargas de cadastro. A carga roda no Airflow da GCP.</t>
         </is>
       </c>
       <c r="N28" s="16" t="n"/>
@@ -2288,7 +2288,7 @@
       </c>
       <c r="M29" s="16" t="inlineStr">
         <is>
-          <t>Os mesmos cards dependem do download D+1 de cadastro. Não há card só para isso. O esperado é o arquivo do dia seguinte disponível em HML.</t>
+          <t>Cards 470165 e 470100 dependem do download D+1. O arquivo do dia seguinte fica em HML.</t>
         </is>
       </c>
       <c r="N29" s="16" t="n"/>
@@ -2347,7 +2347,7 @@
       </c>
       <c r="M30" s="18" t="inlineStr">
         <is>
-          <t>Backend do backoffice. A observação diz que depende do Airflow. O esperado é ele no ar depois que o Airflow estiver na GCP.</t>
+          <t>Backend do backoffice. Depende do Airflow na GCP.</t>
         </is>
       </c>
       <c r="N30" s="19" t="inlineStr">
@@ -2412,7 +2412,7 @@
       </c>
       <c r="M31" s="18" t="inlineStr">
         <is>
-          <t>Tela portal-cadastro-web. Depende do Airflow pronto, das cargas de cadastro e do D+1. O repositório datp-backoffice-frontend-portal está cancelado e em discussão. O esperado é o portal de cadastro abrir em HML com esses dados.</t>
+          <t>Tela portal-cadastro-web. Depende do Airflow, das cargas de cadastro e do D+1.</t>
         </is>
       </c>
       <c r="N31" s="19" t="inlineStr">
@@ -2477,7 +2477,7 @@
       </c>
       <c r="M32" s="18" t="inlineStr">
         <is>
-          <t>Frontend do backoffice, com a mesma dependência do portal-cadastro-web. O esperado é a mesma condição: Airflow, cargas e D+1 prontos.</t>
+          <t>Frontend do backoffice. Depende do Airflow, das cargas de cadastro e do D+1.</t>
         </is>
       </c>
       <c r="N32" s="19" t="inlineStr">
@@ -2542,7 +2542,7 @@
       </c>
       <c r="M33" s="18" t="inlineStr">
         <is>
-          <t>Adaptação do backend do portal de cadastro. O esperado é o código ajustado para a HML, no mesmo bloco do portal.</t>
+          <t>Adaptação do backend do portal de cadastro para a HML.</t>
         </is>
       </c>
       <c r="N33" s="19" t="inlineStr">
@@ -2611,7 +2611,7 @@
       </c>
       <c r="M34" s="18" t="inlineStr">
         <is>
-          <t>Adaptação do frontend do portal de cadastro. Só testa com tudo integrado. O esperado é a tela pronta para o teste do card 451689.</t>
+          <t>Adaptação do frontend do portal de cadastro. O teste é integrado.</t>
         </is>
       </c>
       <c r="N34" s="19" t="inlineStr">
@@ -2656,7 +2656,7 @@
       </c>
       <c r="M35" s="20" t="inlineStr">
         <is>
-          <t>A decisão oficial é levar o Databricks para a GCP. A documentação lista os workspaces de HML e de PRD, sem jobs. O esperado é o Databricks na GCP antes da homologação, junto dos outros componentes.</t>
+          <t>Databricks de HML (adb-887971986833958) e de PRD (adb-7665073515379548) na GCP.</t>
         </is>
       </c>
       <c r="N35" s="20" t="n"/>
@@ -2715,7 +2715,7 @@
       </c>
       <c r="M36" s="22" t="inlineStr">
         <is>
-          <t>A documentação lista o Event Hub data-provider-prd. O esperado é a troca para Pub/Sub estar na HML antes do teste, para o componente poder ser homologado.</t>
+          <t>Event Hub data-provider-prd vira Pub/Sub na HML.</t>
         </is>
       </c>
       <c r="N36" s="23" t="inlineStr">
@@ -2760,7 +2760,7 @@
       </c>
       <c r="M37" s="24" t="inlineStr">
         <is>
-          <t>Linha nova. O esperado é provar, na HML, que NAV, CDC e portal consultam exame, unidade e convênio, com gateway, APIs, busca, Airflow, carga do TIE, Blob, portal, Databricks, Event Hub, Redis e o frontend dp-corporate-frontend.</t>
+          <t>NAV, CDC e portal consultam exame, unidade e convênio na HML, com todos os componentes no ar.</t>
         </is>
       </c>
       <c r="N37" s="24" t="n"/>
@@ -2799,7 +2799,7 @@
       </c>
       <c r="M38" s="24" t="inlineStr">
         <is>
-          <t>Linha nova, depois do teste funcional. O documento não traz volume nem meta. O esperado é a mesma HML, já funcional, receber carga antes de qualquer plano de produção.</t>
+          <t>Teste de carga da HML já funcional, antes da produção.</t>
         </is>
       </c>
       <c r="N38" s="24" t="n"/>
@@ -2850,7 +2850,7 @@
       </c>
       <c r="M39" s="26" t="inlineStr">
         <is>
-          <t>Card da equipe para homologação e rollback. O esperado é o aceite da HML e o plano de volta, depois dos testes funcional e de carga.</t>
+          <t>Homologação e rollback da HML, depois dos testes funcional e de carga.</t>
         </is>
       </c>
       <c r="N39" s="27" t="inlineStr">
@@ -2895,7 +2895,7 @@
       </c>
       <c r="M40" s="28" t="inlineStr">
         <is>
-          <t>A documentação cita o cluster aks-prd-cadastro01. O único GKE com card é o de HML, já concluído. O esperado é o cluster de produção existir só depois da HML testada.</t>
+          <t>Cluster de produção aks-prd-cadastro01, depois da HML homologada.</t>
         </is>
       </c>
       <c r="N40" s="28" t="n"/>
@@ -2958,7 +2958,7 @@
       </c>
       <c r="M41" s="30" t="inlineStr">
         <is>
-          <t>Worker do Airflow de produção. O esperado é esta peça no ar depois da HML. A data 09/10/26 da planilha não antecipa a linha.</t>
+          <t>Worker do Airflow de produção.</t>
         </is>
       </c>
       <c r="N41" s="31" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="M42" s="30" t="inlineStr">
         <is>
-          <t>Workload principal do Airflow de produção. O esperado é ele no ar depois da HML.</t>
+          <t>Workload principal do Airflow de produção.</t>
         </is>
       </c>
       <c r="N42" s="31" t="inlineStr">
@@ -3096,7 +3096,7 @@
       </c>
       <c r="M43" s="30" t="inlineStr">
         <is>
-          <t>Sincronização de usuários do Airflow de produção. O esperado é ela no ar depois da HML.</t>
+          <t>Sincronização de usuários do Airflow de produção.</t>
         </is>
       </c>
       <c r="N43" s="31" t="inlineStr">
@@ -3165,7 +3165,7 @@
       </c>
       <c r="M44" s="30" t="inlineStr">
         <is>
-          <t>Scheduler do Airflow de produção. O esperado é ele no ar depois da HML.</t>
+          <t>Scheduler do Airflow de produção.</t>
         </is>
       </c>
       <c r="N44" s="31" t="inlineStr">
@@ -3234,7 +3234,7 @@
       </c>
       <c r="M45" s="30" t="inlineStr">
         <is>
-          <t>Flower do Airflow de produção. O esperado é ele no ar depois da HML.</t>
+          <t>Flower do Airflow de produção.</t>
         </is>
       </c>
       <c r="N45" s="31" t="inlineStr">
@@ -3303,7 +3303,7 @@
       </c>
       <c r="M46" s="30" t="inlineStr">
         <is>
-          <t>Migração do banco do Airflow de produção. O esperado é ela rodar depois da HML.</t>
+          <t>Migração do banco do Airflow de produção.</t>
         </is>
       </c>
       <c r="N46" s="31" t="inlineStr">
@@ -3360,7 +3360,7 @@
       </c>
       <c r="M47" s="30" t="inlineStr">
         <is>
-          <t>Go-live sem escopo. O documento não define se a entrada é única ou gradual, nem DNS nem janela. O esperado é o plano de produção, só depois da HML aceita pelos canais.</t>
+          <t>Cutover e go-live, depois da HML aceita.</t>
         </is>
       </c>
       <c r="N47" s="31" t="inlineStr">
@@ -3413,7 +3413,7 @@
       </c>
       <c r="M48" s="32" t="inlineStr">
         <is>
-          <t>A equipe cancelou este workload. A linha dp-corporate-frontend na HML cobre a URL que a documentação cita, para o frontend entrar na homologação.</t>
+          <t>Workload cancelado. A URL segue na linha dp-corporate-frontend.</t>
         </is>
       </c>
       <c r="N48" s="33" t="inlineStr">
@@ -3470,7 +3470,7 @@
       </c>
       <c r="M49" s="32" t="inlineStr">
         <is>
-          <t>Cancelado pela equipe, com observação de Cognitive Search. Os backends 469049 e 468966 seguem no caminho. O documento não descreve este card além disso.</t>
+          <t>Cancelado. A API de exam segue no caminho.</t>
         </is>
       </c>
       <c r="N49" s="33" t="inlineStr">
@@ -3523,7 +3523,7 @@
       </c>
       <c r="M50" s="32" t="inlineStr">
         <is>
-          <t>Cancelado. A decisão oficial é levar o Databricks, não converter os ETLs para outra ferramenta.</t>
+          <t>Cancelado. O Databricks vai para a GCP.</t>
         </is>
       </c>
       <c r="N50" s="33" t="inlineStr">
@@ -3576,7 +3576,7 @@
       </c>
       <c r="M51" s="32" t="inlineStr">
         <is>
-          <t>Cancelado. Não há reescrita para PostgreSQL neste plano. O banco de HML já foi criado.</t>
+          <t>Cancelado. O banco de HML já existe.</t>
         </is>
       </c>
       <c r="N51" s="33" t="inlineStr">
@@ -3629,7 +3629,7 @@
       </c>
       <c r="M52" s="32" t="inlineStr">
         <is>
-          <t>Abortado e concluído. O SQL Server não é copiado. A documentação diz que a réplica 3 não migra e está desligada. O dado segue pela carga no banco já criado.</t>
+          <t>Abortado. O dado de HML entra pela carga do TIE no banco já criado.</t>
         </is>
       </c>
       <c r="N52" s="33" t="inlineStr">

</xml_diff>